<commit_message>
🐛 FIX COMPLETO v2.1 — 10 bug risolti
Bug 1-3: Assumptions
- Churn M1-M6: 0% → 4% | M7+: 0% → 2%
- IRES: 20% → 24% | IRAP: 0% → 3,9% | Aliquota totale: 30% → 27,9%
- Seed: €75K → €100K (range €90-150K)

Bug 4-6: KPI Dashboard
- Revenue totale: 0 → collegato a MASTER R9 (include fee A.4)
- ARPU: ora Revenue/Merchant (non più totale ricavi)
- Gross Margin%, EBIT Margin%, Marketing% ora calcolati correttamente

Bug 7: MRR Waterfall cross-check → confronta SMB vs SMB (R16)

Bug 8: SP debiti vs collaboratori azzerati (evita doppio conteggio)

Bug 9: Unit Economics
- ARPU collegato a MASTER / Merchant (non più hardcoded)
- LTV = ARPU × Lifetime: ora funziona (M1: €980, M3: €2.031, M6: €4.201)
- LTV:CAC corretto (M3: 55x, M6: 15x — eccellente)
- Magic Number corretto
- EBITDA Margin% usa MASTER R9

Bug 10: A.4 Business Plus fee: 0.5 → 0.45
</commit_message>
<xml_diff>
--- a/03-FINANCIAL-MODELS/DLOOP_Budget_Guerriglia_FULL_v2.xlsx
+++ b/03-FINANCIAL-MODELS/DLOOP_Budget_Guerriglia_FULL_v2.xlsx
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="529">
   <si>
     <t xml:space="preserve">DLOOP — FOGLIO ASSUNZIONI CENTRALIZZATE  |  Modifica qui, non nei fogli area</t>
   </si>
@@ -303,10 +303,10 @@
     <t xml:space="preserve">Seed round atteso</t>
   </si>
   <si>
-    <t xml:space="preserve">€ 75.000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Range €50-100K via MoodCapital — ipotesi M3</t>
+    <t xml:space="preserve">€ 100.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range €90-150K via MoodCapital — ipotesi M3</t>
   </si>
   <si>
     <t xml:space="preserve">Cash runway target</t>
@@ -1213,6 +1213,9 @@
   </si>
   <si>
     <t xml:space="preserve">  Seed round ricevuto  (€50-100K — ipotesi €75K a M3)  [Una tantum M3 — input principale]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range €90-150K via MoodCapital — ipotesi €100K a M3</t>
   </si>
   <si>
     <t xml:space="preserve">  Tasso interesse annuo su conto deposito  (%)  [~2.5% annuo conto deposito vincolato]</t>
@@ -4671,8 +4674,8 @@
       <c r="C5" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="55" t="n">
-        <v>75000</v>
+      <c r="D5" s="55" t="s">
+        <v>383</v>
       </c>
       <c r="E5" s="54" t="n">
         <v>0</v>
@@ -4721,12 +4724,12 @@
       </c>
       <c r="T5" s="56" t="n">
         <f aca="false">SUM(B5:S5)</f>
-        <v>75000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B6" s="111" t="n">
         <v>0</v>
@@ -4789,7 +4792,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B7" s="54" t="n">
         <v>0</v>
@@ -4852,7 +4855,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B8" s="54" t="n">
         <v>0</v>
@@ -4915,7 +4918,7 @@
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -4939,7 +4942,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="41" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B10" s="54" t="n">
         <v>0</v>
@@ -5002,7 +5005,7 @@
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
@@ -5026,7 +5029,7 @@
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="40" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B12" s="40"/>
       <c r="C12" s="40"/>
@@ -5050,7 +5053,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B13" s="55" t="n">
         <v>4090</v>
@@ -5113,7 +5116,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B14" s="42" t="n">
         <v>18</v>
@@ -5208,7 +5211,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5232,7 +5235,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5318,7 +5321,7 @@
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -5342,318 +5345,318 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!B31</f>
-        <v>0</v>
+        <f aca="false">MASTER!B9</f>
+        <v>196</v>
       </c>
       <c r="C5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!C31</f>
-        <v>0</v>
+        <f aca="false">MASTER!C9</f>
+        <v>353</v>
       </c>
       <c r="D5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!D31</f>
-        <v>0</v>
+        <f aca="false">MASTER!D9</f>
+        <v>1056</v>
       </c>
       <c r="E5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!E31</f>
-        <v>0</v>
+        <f aca="false">MASTER!E9</f>
+        <v>2001</v>
       </c>
       <c r="F5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!F31</f>
-        <v>0</v>
+        <f aca="false">MASTER!F9</f>
+        <v>2984</v>
       </c>
       <c r="G5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!G31</f>
-        <v>0</v>
+        <f aca="false">MASTER!G9</f>
+        <v>4285</v>
       </c>
       <c r="H5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!H31</f>
-        <v>0</v>
+        <f aca="false">MASTER!H9</f>
+        <v>5828</v>
       </c>
       <c r="I5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!I31</f>
-        <v>0</v>
+        <f aca="false">MASTER!I9</f>
+        <v>7259</v>
       </c>
       <c r="J5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!J31</f>
-        <v>0</v>
+        <f aca="false">MASTER!J9</f>
+        <v>8861</v>
       </c>
       <c r="K5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!K31</f>
-        <v>0</v>
+        <f aca="false">MASTER!K9</f>
+        <v>10312</v>
       </c>
       <c r="L5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!L31</f>
-        <v>0</v>
+        <f aca="false">MASTER!L9</f>
+        <v>12173</v>
       </c>
       <c r="M5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!M31</f>
-        <v>0</v>
+        <f aca="false">MASTER!M9</f>
+        <v>13863</v>
       </c>
       <c r="N5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!N31</f>
-        <v>0</v>
+        <f aca="false">MASTER!N9</f>
+        <v>16823</v>
       </c>
       <c r="O5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!O31</f>
-        <v>0</v>
+        <f aca="false">MASTER!O9</f>
+        <v>18894</v>
       </c>
       <c r="P5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!P31</f>
-        <v>0</v>
+        <f aca="false">MASTER!P9</f>
+        <v>22094</v>
       </c>
       <c r="Q5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!Q31</f>
-        <v>0</v>
+        <f aca="false">MASTER!Q9</f>
+        <v>24134</v>
       </c>
       <c r="R5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!R31</f>
-        <v>0</v>
+        <f aca="false">MASTER!R9</f>
+        <v>27674</v>
       </c>
       <c r="S5" s="50" t="n">
-        <f aca="false">'A — Ricavi'!S31</f>
-        <v>0</v>
+        <f aca="false">MASTER!S9</f>
+        <v>30174</v>
       </c>
       <c r="T5" s="72" t="n">
         <f aca="false">SUM(B5:S5)</f>
-        <v>0</v>
+        <v>208964</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="90" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B6" s="91" t="n">
-        <f aca="false">'A — Ricavi'!B31</f>
-        <v>0</v>
+        <f aca="false">MASTER!B9</f>
+        <v>196</v>
       </c>
       <c r="C6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:C31)</f>
-        <v>0</v>
+        <f aca="false">B6+MASTER!C9</f>
+        <v>549</v>
       </c>
       <c r="D6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:D31)</f>
-        <v>0</v>
+        <f aca="false">C6+MASTER!D9</f>
+        <v>1605</v>
       </c>
       <c r="E6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:E31)</f>
-        <v>0</v>
+        <f aca="false">D6+MASTER!E9</f>
+        <v>3606</v>
       </c>
       <c r="F6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:F31)</f>
-        <v>0</v>
+        <f aca="false">E6+MASTER!F9</f>
+        <v>6590</v>
       </c>
       <c r="G6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:G31)</f>
-        <v>0</v>
+        <f aca="false">F6+MASTER!G9</f>
+        <v>10875</v>
       </c>
       <c r="H6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:H31)</f>
-        <v>0</v>
+        <f aca="false">G6+MASTER!H9</f>
+        <v>16703</v>
       </c>
       <c r="I6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:I31)</f>
-        <v>0</v>
+        <f aca="false">H6+MASTER!I9</f>
+        <v>23962</v>
       </c>
       <c r="J6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:J31)</f>
-        <v>0</v>
+        <f aca="false">I6+MASTER!J9</f>
+        <v>32823</v>
       </c>
       <c r="K6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:K31)</f>
-        <v>0</v>
+        <f aca="false">J6+MASTER!K9</f>
+        <v>43135</v>
       </c>
       <c r="L6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:L31)</f>
-        <v>0</v>
+        <f aca="false">K6+MASTER!L9</f>
+        <v>55308</v>
       </c>
       <c r="M6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:M31)</f>
-        <v>0</v>
+        <f aca="false">L6+MASTER!M9</f>
+        <v>69171</v>
       </c>
       <c r="N6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:N31)</f>
-        <v>0</v>
+        <f aca="false">M6+MASTER!N9</f>
+        <v>85994</v>
       </c>
       <c r="O6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:O31)</f>
-        <v>0</v>
+        <f aca="false">N6+MASTER!O9</f>
+        <v>104888</v>
       </c>
       <c r="P6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:P31)</f>
-        <v>0</v>
+        <f aca="false">O6+MASTER!P9</f>
+        <v>126982</v>
       </c>
       <c r="Q6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:Q31)</f>
-        <v>0</v>
+        <f aca="false">P6+MASTER!Q9</f>
+        <v>151116</v>
       </c>
       <c r="R6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:R31)</f>
-        <v>0</v>
+        <f aca="false">Q6+MASTER!R9</f>
+        <v>178790</v>
       </c>
       <c r="S6" s="91" t="n">
-        <f aca="false">SUM('A — Ricavi'!B31:S31)</f>
-        <v>0</v>
+        <f aca="false">R6+MASTER!S9</f>
+        <v>208964</v>
       </c>
       <c r="T6" s="112"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!B12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!B16</f>
+        <v>196</v>
       </c>
       <c r="C7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!C12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!C16</f>
+        <v>353</v>
       </c>
       <c r="D7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!D12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!D16</f>
+        <v>777</v>
       </c>
       <c r="E7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!E12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!E16</f>
+        <v>1201</v>
       </c>
       <c r="F7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!F12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!F16</f>
+        <v>1664</v>
       </c>
       <c r="G7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!G12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!G16</f>
+        <v>2166</v>
       </c>
       <c r="H7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!H12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!H16</f>
+        <v>2708</v>
       </c>
       <c r="I7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!I12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!I16</f>
+        <v>3289</v>
       </c>
       <c r="J7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!J12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!J16</f>
+        <v>3870</v>
       </c>
       <c r="K7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!K12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!K16</f>
+        <v>4491</v>
       </c>
       <c r="L7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!L12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!L16</f>
+        <v>5300</v>
       </c>
       <c r="M7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!M12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!M16</f>
+        <v>6109</v>
       </c>
       <c r="N7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!N12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!N16</f>
+        <v>6918</v>
       </c>
       <c r="O7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!O12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!O16</f>
+        <v>7609</v>
       </c>
       <c r="P7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!P12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!P16</f>
+        <v>8379</v>
       </c>
       <c r="Q7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!Q12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!Q16</f>
+        <v>9149</v>
       </c>
       <c r="R7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!R12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!R16</f>
+        <v>9801</v>
       </c>
       <c r="S7" s="50" t="n">
-        <f aca="false">'A — Ricavi'!S12</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!S16</f>
+        <v>10492</v>
       </c>
       <c r="T7" s="72" t="n">
         <f aca="false">SUM(B7:S7)</f>
-        <v>0</v>
+        <v>84472</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!B21</f>
+        <f aca="false">'A — Ricavi'!B22</f>
         <v>0</v>
       </c>
       <c r="C8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!C21</f>
+        <f aca="false">'A — Ricavi'!C22</f>
         <v>0</v>
       </c>
       <c r="D8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!D21</f>
+        <f aca="false">'A — Ricavi'!D22</f>
         <v>0</v>
       </c>
       <c r="E8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!E21</f>
+        <f aca="false">'A — Ricavi'!E22</f>
         <v>22</v>
       </c>
       <c r="F8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!F21</f>
+        <f aca="false">'A — Ricavi'!F22</f>
         <v>43</v>
       </c>
       <c r="G8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!G21</f>
+        <f aca="false">'A — Ricavi'!G22</f>
         <v>64</v>
       </c>
       <c r="H8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!H21</f>
+        <f aca="false">'A — Ricavi'!H22</f>
         <v>116</v>
       </c>
       <c r="I8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!I21</f>
+        <f aca="false">'A — Ricavi'!I22</f>
         <v>188</v>
       </c>
       <c r="J8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!J21</f>
+        <f aca="false">'A — Ricavi'!J22</f>
         <v>260</v>
       </c>
       <c r="K8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!K21</f>
+        <f aca="false">'A — Ricavi'!K22</f>
         <v>312</v>
       </c>
       <c r="L8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!L21</f>
+        <f aca="false">'A — Ricavi'!L22</f>
         <v>415</v>
       </c>
       <c r="M8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!M21</f>
+        <f aca="false">'A — Ricavi'!M22</f>
         <v>518</v>
       </c>
       <c r="N8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!N21</f>
+        <f aca="false">'A — Ricavi'!N22</f>
         <v>621</v>
       </c>
       <c r="O8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!O21</f>
+        <f aca="false">'A — Ricavi'!O22</f>
         <v>724</v>
       </c>
       <c r="P8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!P21</f>
+        <f aca="false">'A — Ricavi'!P22</f>
         <v>827</v>
       </c>
       <c r="Q8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!Q21</f>
+        <f aca="false">'A — Ricavi'!Q22</f>
         <v>869</v>
       </c>
       <c r="R8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!R21</f>
+        <f aca="false">'A — Ricavi'!R22</f>
         <v>931</v>
       </c>
       <c r="S8" s="50" t="n">
-        <f aca="false">'A — Ricavi'!S21</f>
+        <f aca="false">'A — Ricavi'!S22</f>
         <v>1013</v>
       </c>
       <c r="T8" s="72" t="n">
@@ -5663,88 +5666,88 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!B27</f>
+        <f aca="false">'A — Ricavi'!B28</f>
         <v>0</v>
       </c>
       <c r="C9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!C27</f>
+        <f aca="false">'A — Ricavi'!C28</f>
         <v>0</v>
       </c>
       <c r="D9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!D27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!D28</f>
+        <v>99</v>
       </c>
       <c r="E9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!E27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!E28</f>
+        <v>298</v>
       </c>
       <c r="F9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!F27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!F28</f>
+        <v>497</v>
       </c>
       <c r="G9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!G27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!G28</f>
+        <v>795</v>
       </c>
       <c r="H9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!H27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!H28</f>
+        <v>994</v>
       </c>
       <c r="I9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!I27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!I28</f>
+        <v>1292</v>
       </c>
       <c r="J9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!J27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!J28</f>
+        <v>1491</v>
       </c>
       <c r="K9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!K27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!K28</f>
+        <v>1789</v>
       </c>
       <c r="L9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!L27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!L28</f>
+        <v>1988</v>
       </c>
       <c r="M9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!M27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!M28</f>
+        <v>2286</v>
       </c>
       <c r="N9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!N27</f>
-        <v>0</v>
+        <f aca="false">'A — Ricavi'!N28</f>
+        <v>2684</v>
       </c>
       <c r="O9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!O27</f>
-        <v>1</v>
+        <f aca="false">'A — Ricavi'!O28</f>
+        <v>3481</v>
       </c>
       <c r="P9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!P27</f>
-        <v>1</v>
+        <f aca="false">'A — Ricavi'!P28</f>
+        <v>3978</v>
       </c>
       <c r="Q9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!Q27</f>
-        <v>1</v>
+        <f aca="false">'A — Ricavi'!Q28</f>
+        <v>4276</v>
       </c>
       <c r="R9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!R27</f>
-        <v>2</v>
+        <f aca="false">'A — Ricavi'!R28</f>
+        <v>5272</v>
       </c>
       <c r="S9" s="50" t="n">
-        <f aca="false">'A — Ricavi'!S27</f>
-        <v>2</v>
+        <f aca="false">'A — Ricavi'!S28</f>
+        <v>5769</v>
       </c>
       <c r="T9" s="72" t="n">
         <f aca="false">SUM(B9:S9)</f>
-        <v>7</v>
+        <v>36989</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -5768,7 +5771,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B11" s="101" t="n">
         <f aca="false">'A — Ricavi'!B9</f>
@@ -5849,88 +5852,88 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="41" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!B16</f>
-        <v>196</v>
+        <f aca="false">IF('A — Ricavi'!B9&gt;0,MASTER!B9/'A — Ricavi'!B9,0)</f>
+        <v>49</v>
       </c>
       <c r="C12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!C16</f>
-        <v>353</v>
+        <f aca="false">IF('A — Ricavi'!C9&gt;0,MASTER!C9/'A — Ricavi'!C9,0)</f>
+        <v>50.4285714285714</v>
       </c>
       <c r="D12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!D16</f>
-        <v>777</v>
+        <f aca="false">IF('A — Ricavi'!D9&gt;0,MASTER!D9/'A — Ricavi'!D9,0)</f>
+        <v>81.2307692307692</v>
       </c>
       <c r="E12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!E16</f>
-        <v>1201</v>
+        <f aca="false">IF('A — Ricavi'!E9&gt;0,MASTER!E9/'A — Ricavi'!E9,0)</f>
+        <v>105.315789473684</v>
       </c>
       <c r="F12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!F16</f>
-        <v>1664</v>
+        <f aca="false">IF('A — Ricavi'!F9&gt;0,MASTER!F9/'A — Ricavi'!F9,0)</f>
+        <v>114.769230769231</v>
       </c>
       <c r="G12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!G16</f>
-        <v>2166</v>
+        <f aca="false">IF('A — Ricavi'!G9&gt;0,MASTER!G9/'A — Ricavi'!G9,0)</f>
+        <v>126.029411764706</v>
       </c>
       <c r="H12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!H16</f>
-        <v>2708</v>
+        <f aca="false">IF('A — Ricavi'!H9&gt;0,MASTER!H9/'A — Ricavi'!H9,0)</f>
+        <v>138.761904761905</v>
       </c>
       <c r="I12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!I16</f>
-        <v>3289</v>
+        <f aca="false">IF('A — Ricavi'!I9&gt;0,MASTER!I9/'A — Ricavi'!I9,0)</f>
+        <v>142.333333333333</v>
       </c>
       <c r="J12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!J16</f>
-        <v>3870</v>
+        <f aca="false">IF('A — Ricavi'!J9&gt;0,MASTER!J9/'A — Ricavi'!J9,0)</f>
+        <v>147.683333333333</v>
       </c>
       <c r="K12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!K16</f>
-        <v>4491</v>
+        <f aca="false">IF('A — Ricavi'!K9&gt;0,MASTER!K9/'A — Ricavi'!K9,0)</f>
+        <v>149.449275362319</v>
       </c>
       <c r="L12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!L16</f>
-        <v>5300</v>
+        <f aca="false">IF('A — Ricavi'!L9&gt;0,MASTER!L9/'A — Ricavi'!L9,0)</f>
+        <v>152.1625</v>
       </c>
       <c r="M12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!M16</f>
-        <v>6109</v>
+        <f aca="false">IF('A — Ricavi'!M9&gt;0,MASTER!M9/'A — Ricavi'!M9,0)</f>
+        <v>152.340659340659</v>
       </c>
       <c r="N12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!N16</f>
-        <v>6918</v>
+        <f aca="false">IF('A — Ricavi'!N9&gt;0,MASTER!N9/'A — Ricavi'!N9,0)</f>
+        <v>164.93137254902</v>
       </c>
       <c r="O12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!O16</f>
-        <v>7609</v>
+        <f aca="false">IF('A — Ricavi'!O9&gt;0,MASTER!O9/'A — Ricavi'!O9,0)</f>
+        <v>170.216216216216</v>
       </c>
       <c r="P12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!P16</f>
-        <v>8379</v>
+        <f aca="false">IF('A — Ricavi'!P9&gt;0,MASTER!P9/'A — Ricavi'!P9,0)</f>
+        <v>182.595041322314</v>
       </c>
       <c r="Q12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!Q16</f>
-        <v>9149</v>
+        <f aca="false">IF('A — Ricavi'!Q9&gt;0,MASTER!Q9/'A — Ricavi'!Q9,0)</f>
+        <v>184.229007633588</v>
       </c>
       <c r="R12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!R16</f>
-        <v>9801</v>
+        <f aca="false">IF('A — Ricavi'!R9&gt;0,MASTER!R9/'A — Ricavi'!R9,0)</f>
+        <v>199.093525179856</v>
       </c>
       <c r="S12" s="50" t="n">
-        <f aca="false">'A — Ricavi'!S16</f>
-        <v>10492</v>
+        <f aca="false">IF('A — Ricavi'!S9&gt;0,MASTER!S9/'A — Ricavi'!S9,0)</f>
+        <v>203.878378378378</v>
       </c>
       <c r="T12" s="72" t="n">
         <f aca="false">SUM(B12:S12)</f>
-        <v>84472</v>
+        <v>2514.44832007788</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -5954,7 +5957,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B14" s="50" t="n">
         <f aca="false">MASTER!B18</f>
@@ -6035,7 +6038,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="113" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B15" s="114" t="n">
         <f aca="false">'B4 — Personale'!B34</f>
@@ -6116,7 +6119,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="88" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B16" s="76" t="n">
         <f aca="false">'B3 — Marketing'!B28</f>
@@ -6197,7 +6200,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B17" s="50" t="n">
         <f aca="false">'B1 — Infrastruttura'!B18</f>
@@ -6278,7 +6281,7 @@
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -6302,7 +6305,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="115" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B19" s="116" t="n">
         <f aca="false">MASTER!B20</f>
@@ -6383,7 +6386,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="115" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B20" s="116" t="n">
         <f aca="false">MASTER!B25</f>
@@ -6464,7 +6467,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="117" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B21" s="118" t="n">
         <f aca="false">MASTER!B30</f>
@@ -6545,7 +6548,7 @@
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -6569,169 +6572,169 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="41" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!B31&gt;0,('A — Ricavi'!B31-'B1 — Infrastruttura'!B18-'B6 — Costi Variabili'!B16)/'A — Ricavi'!B31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!B9&gt;0,(MASTER!B9-'B1 — Infrastruttura'!B18-'B6 — Costi Variabili'!B16)/MASTER!B9,0)</f>
+        <v>0.0204081632653061</v>
       </c>
       <c r="C23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!C31&gt;0,('A — Ricavi'!C31-'B1 — Infrastruttura'!C18-'B6 — Costi Variabili'!C16)/'A — Ricavi'!C31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!C9&gt;0,(MASTER!C9-'B1 — Infrastruttura'!C18-'B6 — Costi Variabili'!C16)/MASTER!C9,0)</f>
+        <v>0.286118980169972</v>
       </c>
       <c r="D23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!D31&gt;0,('A — Ricavi'!D31-'B1 — Infrastruttura'!D18-'B6 — Costi Variabili'!D16)/'A — Ricavi'!D31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!D9&gt;0,(MASTER!D9-'B1 — Infrastruttura'!D18-'B6 — Costi Variabili'!D16)/MASTER!D9,0)</f>
+        <v>0.670454545454545</v>
       </c>
       <c r="E23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!E31&gt;0,('A — Ricavi'!E31-'B1 — Infrastruttura'!E18-'B6 — Costi Variabili'!E16)/'A — Ricavi'!E31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!E9&gt;0,(MASTER!E9-'B1 — Infrastruttura'!E18-'B6 — Costi Variabili'!E16)/MASTER!E9,0)</f>
+        <v>0.762618690654673</v>
       </c>
       <c r="F23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!F31&gt;0,('A — Ricavi'!F31-'B1 — Infrastruttura'!F18-'B6 — Costi Variabili'!F16)/'A — Ricavi'!F31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!F9&gt;0,(MASTER!F9-'B1 — Infrastruttura'!F18-'B6 — Costi Variabili'!F16)/MASTER!F9,0)</f>
+        <v>0.770777479892761</v>
       </c>
       <c r="G23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!G31&gt;0,('A — Ricavi'!G31-'B1 — Infrastruttura'!G18-'B6 — Costi Variabili'!G16)/'A — Ricavi'!G31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!G9&gt;0,(MASTER!G9-'B1 — Infrastruttura'!G18-'B6 — Costi Variabili'!G16)/MASTER!G9,0)</f>
+        <v>0.790665110851809</v>
       </c>
       <c r="H23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!H31&gt;0,('A — Ricavi'!H31-'B1 — Infrastruttura'!H18-'B6 — Costi Variabili'!H16)/'A — Ricavi'!H31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!H9&gt;0,(MASTER!H9-'B1 — Infrastruttura'!H18-'B6 — Costi Variabili'!H16)/MASTER!H9,0)</f>
+        <v>0.810741249142073</v>
       </c>
       <c r="I23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!I31&gt;0,('A — Ricavi'!I31-'B1 — Infrastruttura'!I18-'B6 — Costi Variabili'!I16)/'A — Ricavi'!I31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!I9&gt;0,(MASTER!I9-'B1 — Infrastruttura'!I18-'B6 — Costi Variabili'!I16)/MASTER!I9,0)</f>
+        <v>0.81443725030996</v>
       </c>
       <c r="J23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!J31&gt;0,('A — Ricavi'!J31-'B1 — Infrastruttura'!J18-'B6 — Costi Variabili'!J16)/'A — Ricavi'!J31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!J9&gt;0,(MASTER!J9-'B1 — Infrastruttura'!J18-'B6 — Costi Variabili'!J16)/MASTER!J9,0)</f>
+        <v>0.816724974607832</v>
       </c>
       <c r="K23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!K31&gt;0,('A — Ricavi'!K31-'B1 — Infrastruttura'!K18-'B6 — Costi Variabili'!K16)/'A — Ricavi'!K31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!K9&gt;0,(MASTER!K9-'B1 — Infrastruttura'!K18-'B6 — Costi Variabili'!K16)/MASTER!K9,0)</f>
+        <v>0.815748642358417</v>
       </c>
       <c r="L23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!L31&gt;0,('A — Ricavi'!L31-'B1 — Infrastruttura'!L18-'B6 — Costi Variabili'!L16)/'A — Ricavi'!L31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!L9&gt;0,(MASTER!L9-'B1 — Infrastruttura'!L18-'B6 — Costi Variabili'!L16)/MASTER!L9,0)</f>
+        <v>0.81836852049618</v>
       </c>
       <c r="M23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!M31&gt;0,('A — Ricavi'!M31-'B1 — Infrastruttura'!M18-'B6 — Costi Variabili'!M16)/'A — Ricavi'!M31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!M9&gt;0,(MASTER!M9-'B1 — Infrastruttura'!M18-'B6 — Costi Variabili'!M16)/MASTER!M9,0)</f>
+        <v>0.813893096732309</v>
       </c>
       <c r="N23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!N31&gt;0,('A — Ricavi'!N31-'B1 — Infrastruttura'!N18-'B6 — Costi Variabili'!N16)/'A — Ricavi'!N31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!N9&gt;0,(MASTER!N9-'B1 — Infrastruttura'!N18-'B6 — Costi Variabili'!N16)/MASTER!N9,0)</f>
+        <v>0.823396540450574</v>
       </c>
       <c r="O23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!O31&gt;0,('A — Ricavi'!O31-'B1 — Infrastruttura'!O18-'B6 — Costi Variabili'!O16)/'A — Ricavi'!O31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!O9&gt;0,(MASTER!O9-'B1 — Infrastruttura'!O18-'B6 — Costi Variabili'!O16)/MASTER!O9,0)</f>
+        <v>0.823859426272891</v>
       </c>
       <c r="P23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!P31&gt;0,('A — Ricavi'!P31-'B1 — Infrastruttura'!P18-'B6 — Costi Variabili'!P16)/'A — Ricavi'!P31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!P9&gt;0,(MASTER!P9-'B1 — Infrastruttura'!P18-'B6 — Costi Variabili'!P16)/MASTER!P9,0)</f>
+        <v>0.832578980718747</v>
       </c>
       <c r="Q23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!Q31&gt;0,('A — Ricavi'!Q31-'B1 — Infrastruttura'!Q18-'B6 — Costi Variabili'!Q16)/'A — Ricavi'!Q31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!Q9&gt;0,(MASTER!Q9-'B1 — Infrastruttura'!Q18-'B6 — Costi Variabili'!Q16)/MASTER!Q9,0)</f>
+        <v>0.832269826800365</v>
       </c>
       <c r="R23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!R31&gt;0,('A — Ricavi'!R31-'B1 — Infrastruttura'!R18-'B6 — Costi Variabili'!R16)/'A — Ricavi'!R31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!R9&gt;0,(MASTER!R9-'B1 — Infrastruttura'!R18-'B6 — Costi Variabili'!R16)/MASTER!R9,0)</f>
+        <v>0.841728698417287</v>
       </c>
       <c r="S23" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!S31&gt;0,('A — Ricavi'!S31-'B1 — Infrastruttura'!S18-'B6 — Costi Variabili'!S16)/'A — Ricavi'!S31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!S9&gt;0,(MASTER!S9-'B1 — Infrastruttura'!S18-'B6 — Costi Variabili'!S16)/MASTER!S9,0)</f>
+        <v>0.844004772320541</v>
       </c>
       <c r="T23" s="120" t="n">
         <f aca="false">AVERAGE(B23:S23)</f>
-        <v>0</v>
+        <v>0.732710830495347</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="88" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!B31&gt;0,'B3 — Marketing'!B26/'A — Ricavi'!B31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!B9&gt;0,'B3 — Marketing'!B28/MASTER!B9,0)</f>
+        <v>0.86734693877551</v>
       </c>
       <c r="C24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!C31&gt;0,'B3 — Marketing'!C26/'A — Ricavi'!C31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!C9&gt;0,'B3 — Marketing'!C28/MASTER!C9,0)</f>
+        <v>0.509915014164306</v>
       </c>
       <c r="D24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!D31&gt;0,'B3 — Marketing'!D26/'A — Ricavi'!D31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!D9&gt;0,'B3 — Marketing'!D28/MASTER!D9,0)</f>
+        <v>0.208333333333333</v>
       </c>
       <c r="E24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!E31&gt;0,'B3 — Marketing'!E26/'A — Ricavi'!E31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!E9&gt;0,'B3 — Marketing'!E28/MASTER!E9,0)</f>
+        <v>0.114942528735632</v>
       </c>
       <c r="F24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!F31&gt;0,'B3 — Marketing'!F26/'A — Ricavi'!F31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!F9&gt;0,'B3 — Marketing'!F28/MASTER!F9,0)</f>
+        <v>0.103887399463807</v>
       </c>
       <c r="G24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!G31&gt;0,'B3 — Marketing'!G26/'A — Ricavi'!G31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!G9&gt;0,'B3 — Marketing'!G28/MASTER!G9,0)</f>
+        <v>0.0910151691948658</v>
       </c>
       <c r="H24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!H31&gt;0,'B3 — Marketing'!H26/'A — Ricavi'!H31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!H9&gt;0,'B3 — Marketing'!H28/MASTER!H9,0)</f>
+        <v>0.0806451612903226</v>
       </c>
       <c r="I24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!I31&gt;0,'B3 — Marketing'!I26/'A — Ricavi'!I31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!I9&gt;0,'B3 — Marketing'!I28/MASTER!I9,0)</f>
+        <v>0.0757680121228819</v>
       </c>
       <c r="J24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!J31&gt;0,'B3 — Marketing'!J26/'A — Ricavi'!J31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!J9&gt;0,'B3 — Marketing'!J28/MASTER!J9,0)</f>
+        <v>0.0722266109919874</v>
       </c>
       <c r="K24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!K31&gt;0,'B3 — Marketing'!K26/'A — Ricavi'!K31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!K9&gt;0,'B3 — Marketing'!K28/MASTER!K9,0)</f>
+        <v>0.0678820791311094</v>
       </c>
       <c r="L24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!L31&gt;0,'B3 — Marketing'!L26/'A — Ricavi'!L31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!L9&gt;0,'B3 — Marketing'!L28/MASTER!L9,0)</f>
+        <v>0.0648977244721926</v>
       </c>
       <c r="M24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!M31&gt;0,'B3 — Marketing'!M26/'A — Ricavi'!M31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!M9&gt;0,'B3 — Marketing'!M28/MASTER!M9,0)</f>
+        <v>0.0627569790088725</v>
       </c>
       <c r="N24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!N31&gt;0,'B3 — Marketing'!N26/'A — Ricavi'!N31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!N9&gt;0,'B3 — Marketing'!N28/MASTER!N9,0)</f>
+        <v>0.0570647328062771</v>
       </c>
       <c r="O24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!O31&gt;0,'B3 — Marketing'!O26/'A — Ricavi'!O31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!O9&gt;0,'B3 — Marketing'!O28/MASTER!O9,0)</f>
+        <v>0.0550439292897216</v>
       </c>
       <c r="P24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!P31&gt;0,'B3 — Marketing'!P26/'A — Ricavi'!P31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!P9&gt;0,'B3 — Marketing'!P28/MASTER!P9,0)</f>
+        <v>0.0511451072689418</v>
       </c>
       <c r="Q24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!Q31&gt;0,'B3 — Marketing'!Q26/'A — Ricavi'!Q31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!Q9&gt;0,'B3 — Marketing'!Q28/MASTER!Q9,0)</f>
+        <v>0.0501367365542388</v>
       </c>
       <c r="R24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!R31&gt;0,'B3 — Marketing'!R26/'A — Ricavi'!R31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!R9&gt;0,'B3 — Marketing'!R28/MASTER!R9,0)</f>
+        <v>0.0466141504661415</v>
       </c>
       <c r="S24" s="121" t="n">
-        <f aca="false">IF('A — Ricavi'!S31&gt;0,'B3 — Marketing'!S26/'A — Ricavi'!S31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!S9&gt;0,'B3 — Marketing'!S28/MASTER!S9,0)</f>
+        <v>0.0454033273679327</v>
       </c>
       <c r="T24" s="122" t="n">
         <f aca="false">AVERAGE(B24:S24)</f>
-        <v>0</v>
+        <v>0.145834718579893</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="41" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B25" s="119" t="n">
         <f aca="false">IF(MASTER!B18&gt;0,'B4 — Personale'!B34/MASTER!B18,0)</f>
@@ -6812,88 +6815,88 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!B31&gt;0,MASTER!B20/'A — Ricavi'!B31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!B9&gt;0,MASTER!B20/MASTER!B9,0)</f>
+        <v>-21.0867346938776</v>
       </c>
       <c r="C26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!C31&gt;0,MASTER!C20/'A — Ricavi'!C31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!C9&gt;0,MASTER!C20/MASTER!C9,0)</f>
+        <v>-11.4759206798867</v>
       </c>
       <c r="D26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!D31&gt;0,MASTER!D20/'A — Ricavi'!D31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!D9&gt;0,MASTER!D20/MASTER!D9,0)</f>
+        <v>-3.31818181818182</v>
       </c>
       <c r="E26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!E31&gt;0,MASTER!E20/'A — Ricavi'!E31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!E9&gt;0,MASTER!E20/MASTER!E9,0)</f>
+        <v>-2.11444277861069</v>
       </c>
       <c r="F26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!F31&gt;0,MASTER!F20/'A — Ricavi'!F31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!F9&gt;0,MASTER!F20/MASTER!F9,0)</f>
+        <v>-1.59752010723861</v>
       </c>
       <c r="G26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!G31&gt;0,MASTER!G20/'A — Ricavi'!G31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!G9&gt;0,MASTER!G20/MASTER!G9,0)</f>
+        <v>-1.04760793465578</v>
       </c>
       <c r="H26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!H31&gt;0,MASTER!H20/'A — Ricavi'!H31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!H9&gt;0,MASTER!H20/MASTER!H9,0)</f>
+        <v>-0.990391214824983</v>
       </c>
       <c r="I26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!I31&gt;0,MASTER!I20/'A — Ricavi'!I31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!I9&gt;0,MASTER!I20/MASTER!I9,0)</f>
+        <v>-0.648160903705745</v>
       </c>
       <c r="J26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!J31&gt;0,MASTER!J20/'A — Ricavi'!J31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!J9&gt;0,MASTER!J20/MASTER!J9,0)</f>
+        <v>-0.396117819659181</v>
       </c>
       <c r="K26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!K31&gt;0,MASTER!K20/'A — Ricavi'!K31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!K9&gt;0,MASTER!K20/MASTER!K9,0)</f>
+        <v>-0.236617532971296</v>
       </c>
       <c r="L26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!L31&gt;0,MASTER!L20/'A — Ricavi'!L31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!L9&gt;0,MASTER!L20/MASTER!L9,0)</f>
+        <v>-0.22755278074427</v>
       </c>
       <c r="M26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!M31&gt;0,MASTER!M20/'A — Ricavi'!M31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!M9&gt;0,MASTER!M20/MASTER!M9,0)</f>
+        <v>-0.113178965591863</v>
       </c>
       <c r="N26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!N31&gt;0,MASTER!N20/'A — Ricavi'!N31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!N9&gt;0,MASTER!N20/MASTER!N9,0)</f>
+        <v>0.0481483683052963</v>
       </c>
       <c r="O26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!O31&gt;0,MASTER!O20/'A — Ricavi'!O31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!O9&gt;0,MASTER!O20/MASTER!O9,0)</f>
+        <v>0.000476341695776437</v>
       </c>
       <c r="P26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!P31&gt;0,MASTER!P20/'A — Ricavi'!P31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!P9&gt;0,MASTER!P20/MASTER!P9,0)</f>
+        <v>0.120756766542953</v>
       </c>
       <c r="Q26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!Q31&gt;0,MASTER!Q20/'A — Ricavi'!Q31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!Q9&gt;0,MASTER!Q20/MASTER!Q9,0)</f>
+        <v>0.17543714262037</v>
       </c>
       <c r="R26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!R31&gt;0,MASTER!R20/'A — Ricavi'!R31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!R9&gt;0,MASTER!R20/MASTER!R9,0)</f>
+        <v>0.263315747633157</v>
       </c>
       <c r="S26" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!S31&gt;0,MASTER!S20/'A — Ricavi'!S31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!S9&gt;0,MASTER!S20/MASTER!S9,0)</f>
+        <v>0.309040896135746</v>
       </c>
       <c r="T26" s="120" t="n">
         <f aca="false">AVERAGE(B26:S26)</f>
-        <v>0</v>
+        <v>-2.35195844261195</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="38" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B27" s="38"/>
       <c r="C27" s="38"/>
@@ -6951,7 +6954,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -6975,7 +6978,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7061,7 +7064,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -7085,7 +7088,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="90" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B5" s="123" t="n">
         <v>0</v>
@@ -7148,7 +7151,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B6" s="55" t="n">
         <v>196</v>
@@ -7211,7 +7214,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B7" s="55" t="n">
         <v>6</v>
@@ -7274,7 +7277,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B8" s="55" t="n">
         <v>8</v>
@@ -7337,7 +7340,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B9" s="55" t="n">
         <v>1</v>
@@ -7400,7 +7403,7 @@
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="45" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B10" s="46" t="n">
         <f aca="false">B6+B7-B8-B9</f>
@@ -7503,7 +7506,7 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="124" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B12" s="46" t="n">
         <f aca="false">B5+B10</f>
@@ -7584,82 +7587,82 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="90" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B13" s="126" t="str">
-        <f aca="false">IF(ABS(B12-'A — Ricavi'!B31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(B12-'A — Ricavi'!B16)&lt;50,"✅","⚠ Δ="&amp;ROUND(B12-'A — Ricavi'!B16,0))</f>
+        <v>✅</v>
       </c>
       <c r="C13" s="126" t="str">
-        <f aca="false">IF(ABS(C12-'A — Ricavi'!C31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(C12-'A — Ricavi'!C16)&lt;50,"✅","⚠ Δ="&amp;ROUND(C12-'A — Ricavi'!C16,0))</f>
+        <v>✅</v>
       </c>
       <c r="D13" s="126" t="str">
-        <f aca="false">IF(ABS(D12-'A — Ricavi'!D31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(D12-'A — Ricavi'!D16)&lt;50,"✅","⚠ Δ="&amp;ROUND(D12-'A — Ricavi'!D16,0))</f>
+        <v>✅</v>
       </c>
       <c r="E13" s="126" t="str">
-        <f aca="false">IF(ABS(E12-'A — Ricavi'!E31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(E12-'A — Ricavi'!E16)&lt;50,"✅","⚠ Δ="&amp;ROUND(E12-'A — Ricavi'!E16,0))</f>
+        <v>⚠ Δ=156</v>
       </c>
       <c r="F13" s="126" t="str">
-        <f aca="false">IF(ABS(F12-'A — Ricavi'!F31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(F12-'A — Ricavi'!F16)&lt;50,"✅","⚠ Δ="&amp;ROUND(F12-'A — Ricavi'!F16,0))</f>
+        <v>⚠ Δ=525</v>
       </c>
       <c r="G13" s="126" t="str">
-        <f aca="false">IF(ABS(G12-'A — Ricavi'!G31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(G12-'A — Ricavi'!G16)&lt;50,"✅","⚠ Δ="&amp;ROUND(G12-'A — Ricavi'!G16,0))</f>
+        <v>⚠ Δ=855</v>
       </c>
       <c r="H13" s="126" t="str">
-        <f aca="false">IF(ABS(H12-'A — Ricavi'!H31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(H12-'A — Ricavi'!H16)&lt;50,"✅","⚠ Δ="&amp;ROUND(H12-'A — Ricavi'!H16,0))</f>
+        <v>⚠ Δ=1266</v>
       </c>
       <c r="I13" s="126" t="str">
-        <f aca="false">IF(ABS(I12-'A — Ricavi'!I31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(I12-'A — Ricavi'!I16)&lt;50,"✅","⚠ Δ="&amp;ROUND(I12-'A — Ricavi'!I16,0))</f>
+        <v>⚠ Δ=1685</v>
       </c>
       <c r="J13" s="126" t="str">
-        <f aca="false">IF(ABS(J12-'A — Ricavi'!J31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(J12-'A — Ricavi'!J16)&lt;50,"✅","⚠ Δ="&amp;ROUND(J12-'A — Ricavi'!J16,0))</f>
+        <v>⚠ Δ=2143</v>
       </c>
       <c r="K13" s="126" t="str">
-        <f aca="false">IF(ABS(K12-'A — Ricavi'!K31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(K12-'A — Ricavi'!K16)&lt;50,"✅","⚠ Δ="&amp;ROUND(K12-'A — Ricavi'!K16,0))</f>
+        <v>⚠ Δ=2477</v>
       </c>
       <c r="L13" s="126" t="str">
-        <f aca="false">IF(ABS(L12-'A — Ricavi'!L31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(L12-'A — Ricavi'!L16)&lt;50,"✅","⚠ Δ="&amp;ROUND(L12-'A — Ricavi'!L16,0))</f>
+        <v>⚠ Δ=2942</v>
       </c>
       <c r="M13" s="126" t="str">
-        <f aca="false">IF(ABS(M12-'A — Ricavi'!M31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(M12-'A — Ricavi'!M16)&lt;50,"✅","⚠ Δ="&amp;ROUND(M12-'A — Ricavi'!M16,0))</f>
+        <v>⚠ Δ=3389</v>
       </c>
       <c r="N13" s="126" t="str">
-        <f aca="false">IF(ABS(N12-'A — Ricavi'!N31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(N12-'A — Ricavi'!N16)&lt;50,"✅","⚠ Δ="&amp;ROUND(N12-'A — Ricavi'!N16,0))</f>
+        <v>⚠ Δ=3943</v>
       </c>
       <c r="O13" s="126" t="str">
-        <f aca="false">IF(ABS(O12-'A — Ricavi'!O31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(O12-'A — Ricavi'!O16)&lt;50,"✅","⚠ Δ="&amp;ROUND(O12-'A — Ricavi'!O16,0))</f>
+        <v>⚠ Δ=4530</v>
       </c>
       <c r="P13" s="126" t="str">
-        <f aca="false">IF(ABS(P12-'A — Ricavi'!P31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(P12-'A — Ricavi'!P16)&lt;50,"✅","⚠ Δ="&amp;ROUND(P12-'A — Ricavi'!P16,0))</f>
+        <v>⚠ Δ=5619</v>
       </c>
       <c r="Q13" s="126" t="str">
-        <f aca="false">IF(ABS(Q12-'A — Ricavi'!Q31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(Q12-'A — Ricavi'!Q16)&lt;50,"✅","⚠ Δ="&amp;ROUND(Q12-'A — Ricavi'!Q16,0))</f>
+        <v>⚠ Δ=6343</v>
       </c>
       <c r="R13" s="126" t="str">
-        <f aca="false">IF(ABS(R12-'A — Ricavi'!R31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(R12-'A — Ricavi'!R16)&lt;50,"✅","⚠ Δ="&amp;ROUND(R12-'A — Ricavi'!R16,0))</f>
+        <v>⚠ Δ=6701</v>
       </c>
       <c r="S13" s="126" t="str">
-        <f aca="false">IF(ABS(S12-'A — Ricavi'!S31)&gt;50,"⚠ CHECK","✓ OK")</f>
-        <v>⚠ CHECK</v>
+        <f aca="false">IF(ABS(S12-'A — Ricavi'!S16)&lt;50,"✅","⚠ Δ="&amp;ROUND(S12-'A — Ricavi'!S16,0))</f>
+        <v>⚠ Δ=7943</v>
       </c>
       <c r="T13" s="127" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7686,7 +7689,7 @@
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -7710,7 +7713,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="41" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B16" s="119" t="n">
         <f aca="false">IF(B5&gt;0,B12/B5,0)</f>
@@ -7791,7 +7794,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="128" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B17" s="128"/>
       <c r="C17" s="128"/>
@@ -7837,7 +7840,7 @@
     </row>
     <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -7861,7 +7864,7 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="129" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B20" s="19" t="n">
         <f aca="false">B12*12</f>
@@ -7942,7 +7945,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="90" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B21" s="93" t="n">
         <f aca="false">IF(B5&gt;0,(B12-B5)/B5,0)</f>
@@ -8045,7 +8048,7 @@
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -8069,7 +8072,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="41" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B24" s="47" t="n">
         <v>1</v>
@@ -8132,7 +8135,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="41" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B25" s="47"/>
       <c r="C25" s="47" t="n">
@@ -8193,7 +8196,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B26" s="47"/>
       <c r="C26" s="47"/>
@@ -8252,7 +8255,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B27" s="47"/>
       <c r="C27" s="47"/>
@@ -8309,7 +8312,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="41" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
@@ -8364,7 +8367,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="41" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B29" s="47"/>
       <c r="C29" s="47"/>
@@ -8417,7 +8420,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="128" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B30" s="128"/>
       <c r="C30" s="128"/>
@@ -8479,7 +8482,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="99" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -8503,7 +8506,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -8589,7 +8592,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="131" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B4" s="131"/>
       <c r="C4" s="131"/>
@@ -8613,7 +8616,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B5" s="55" t="n">
         <v>170</v>
@@ -8676,7 +8679,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B6" s="42" t="n">
         <v>4</v>
@@ -8739,7 +8742,7 @@
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="132" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B7" s="104" t="n">
         <f aca="false">IF(B6&gt;0,B5/B6,0)</f>
@@ -8820,7 +8823,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="134" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B8" s="134"/>
       <c r="C8" s="134"/>
@@ -8866,7 +8869,7 @@
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="131" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B10" s="131"/>
       <c r="C10" s="131"/>
@@ -8890,141 +8893,177 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="90" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B11" s="91" t="n">
+        <f aca="false">IF('A — Ricavi'!B9&gt;0,MASTER!B9/'A — Ricavi'!B9,0)</f>
         <v>49</v>
       </c>
       <c r="C11" s="91" t="n">
-        <v>50</v>
+        <f aca="false">IF('A — Ricavi'!C9&gt;0,MASTER!C9/'A — Ricavi'!C9,0)</f>
+        <v>50.4285714285714</v>
       </c>
       <c r="D11" s="91" t="n">
-        <v>67</v>
+        <f aca="false">IF('A — Ricavi'!D9&gt;0,MASTER!D9/'A — Ricavi'!D9,0)</f>
+        <v>81.2307692307692</v>
       </c>
       <c r="E11" s="91" t="n">
-        <v>84</v>
+        <f aca="false">IF('A — Ricavi'!E9&gt;0,MASTER!E9/'A — Ricavi'!E9,0)</f>
+        <v>105.315789473684</v>
       </c>
       <c r="F11" s="91" t="n">
-        <v>89</v>
+        <f aca="false">IF('A — Ricavi'!F9&gt;0,MASTER!F9/'A — Ricavi'!F9,0)</f>
+        <v>114.769230769231</v>
       </c>
       <c r="G11" s="91" t="n">
-        <v>94</v>
+        <f aca="false">IF('A — Ricavi'!G9&gt;0,MASTER!G9/'A — Ricavi'!G9,0)</f>
+        <v>126.029411764706</v>
       </c>
       <c r="H11" s="91" t="n">
-        <v>96</v>
+        <f aca="false">IF('A — Ricavi'!H9&gt;0,MASTER!H9/'A — Ricavi'!H9,0)</f>
+        <v>138.761904761905</v>
       </c>
       <c r="I11" s="91" t="n">
-        <v>100</v>
+        <f aca="false">IF('A — Ricavi'!I9&gt;0,MASTER!I9/'A — Ricavi'!I9,0)</f>
+        <v>142.333333333333</v>
       </c>
       <c r="J11" s="91" t="n">
-        <v>100</v>
+        <f aca="false">IF('A — Ricavi'!J9&gt;0,MASTER!J9/'A — Ricavi'!J9,0)</f>
+        <v>147.683333333333</v>
       </c>
       <c r="K11" s="91" t="n">
-        <v>102</v>
+        <f aca="false">IF('A — Ricavi'!K9&gt;0,MASTER!K9/'A — Ricavi'!K9,0)</f>
+        <v>149.449275362319</v>
       </c>
       <c r="L11" s="91" t="n">
-        <v>104</v>
+        <f aca="false">IF('A — Ricavi'!L9&gt;0,MASTER!L9/'A — Ricavi'!L9,0)</f>
+        <v>152.1625</v>
       </c>
       <c r="M11" s="91" t="n">
-        <v>106</v>
+        <f aca="false">IF('A — Ricavi'!M9&gt;0,MASTER!M9/'A — Ricavi'!M9,0)</f>
+        <v>152.340659340659</v>
       </c>
       <c r="N11" s="91" t="n">
-        <v>108</v>
+        <f aca="false">IF('A — Ricavi'!N9&gt;0,MASTER!N9/'A — Ricavi'!N9,0)</f>
+        <v>164.93137254902</v>
       </c>
       <c r="O11" s="91" t="n">
-        <v>115</v>
+        <f aca="false">IF('A — Ricavi'!O9&gt;0,MASTER!O9/'A — Ricavi'!O9,0)</f>
+        <v>170.216216216216</v>
       </c>
       <c r="P11" s="91" t="n">
-        <v>118</v>
+        <f aca="false">IF('A — Ricavi'!P9&gt;0,MASTER!P9/'A — Ricavi'!P9,0)</f>
+        <v>182.595041322314</v>
       </c>
       <c r="Q11" s="91" t="n">
-        <v>118</v>
+        <f aca="false">IF('A — Ricavi'!Q9&gt;0,MASTER!Q9/'A — Ricavi'!Q9,0)</f>
+        <v>184.229007633588</v>
       </c>
       <c r="R11" s="91" t="n">
-        <v>124</v>
+        <f aca="false">IF('A — Ricavi'!R9&gt;0,MASTER!R9/'A — Ricavi'!R9,0)</f>
+        <v>199.093525179856</v>
       </c>
       <c r="S11" s="91" t="n">
-        <v>125</v>
+        <f aca="false">IF('A — Ricavi'!S9&gt;0,MASTER!S9/'A — Ricavi'!S9,0)</f>
+        <v>203.878378378378</v>
       </c>
       <c r="T11" s="72" t="n">
         <f aca="false">SUM(B11:S11)</f>
-        <v>1749</v>
+        <v>2514.44832007788</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="41" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!B11/100</f>
+        <v>0.05</v>
+      </c>
+      <c r="C12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!C11/100</f>
+        <v>0.05</v>
+      </c>
+      <c r="D12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!D11/100</f>
         <v>0.04</v>
       </c>
-      <c r="C12" s="47" t="n">
+      <c r="E12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!E11/100</f>
         <v>0.04</v>
       </c>
-      <c r="D12" s="47" t="n">
+      <c r="F12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!F11/100</f>
         <v>0.04</v>
       </c>
-      <c r="E12" s="47" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F12" s="47" t="n">
-        <v>0.04</v>
-      </c>
       <c r="G12" s="47" t="n">
-        <v>0.04</v>
+        <f aca="false">'A — Ricavi'!G11/100</f>
+        <v>0.03</v>
       </c>
       <c r="H12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!H11/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="I12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!I11/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="J12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!J11/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="K12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!K11/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="L12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!L11/100</f>
         <v>0.02</v>
       </c>
-      <c r="I12" s="47" t="n">
+      <c r="M12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!M11/100</f>
         <v>0.02</v>
       </c>
-      <c r="J12" s="47" t="n">
+      <c r="N12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!N11/100</f>
         <v>0.02</v>
       </c>
-      <c r="K12" s="47" t="n">
+      <c r="O12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!O11/100</f>
         <v>0.02</v>
       </c>
-      <c r="L12" s="47" t="n">
+      <c r="P12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!P11/100</f>
         <v>0.02</v>
       </c>
-      <c r="M12" s="47" t="n">
+      <c r="Q12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!Q11/100</f>
         <v>0.02</v>
       </c>
-      <c r="N12" s="47" t="n">
+      <c r="R12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!R11/100</f>
         <v>0.02</v>
       </c>
-      <c r="O12" s="47" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P12" s="47" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="Q12" s="47" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="R12" s="47" t="n">
-        <v>0.02</v>
-      </c>
       <c r="S12" s="47" t="n">
+        <f aca="false">'A — Ricavi'!S11/100</f>
         <v>0.02</v>
       </c>
       <c r="T12" s="120" t="n">
         <f aca="false">AVERAGE(B12:S12)</f>
-        <v>0.0266666666666667</v>
+        <v>0.0294444444444444</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="41" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B13" s="135" t="n">
         <f aca="false">IF(B12&gt;0,1/B12,0)</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C13" s="135" t="n">
         <f aca="false">IF(C12&gt;0,1/C12,0)</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D13" s="135" t="n">
         <f aca="false">IF(D12&gt;0,1/D12,0)</f>
@@ -9040,23 +9079,23 @@
       </c>
       <c r="G13" s="135" t="n">
         <f aca="false">IF(G12&gt;0,1/G12,0)</f>
-        <v>25</v>
+        <v>33.3333333333333</v>
       </c>
       <c r="H13" s="135" t="n">
         <f aca="false">IF(H12&gt;0,1/H12,0)</f>
-        <v>50</v>
+        <v>33.3333333333333</v>
       </c>
       <c r="I13" s="135" t="n">
         <f aca="false">IF(I12&gt;0,1/I12,0)</f>
-        <v>50</v>
+        <v>33.3333333333333</v>
       </c>
       <c r="J13" s="135" t="n">
         <f aca="false">IF(J12&gt;0,1/J12,0)</f>
-        <v>50</v>
+        <v>33.3333333333333</v>
       </c>
       <c r="K13" s="135" t="n">
         <f aca="false">IF(K12&gt;0,1/K12,0)</f>
-        <v>50</v>
+        <v>33.3333333333333</v>
       </c>
       <c r="L13" s="135" t="n">
         <f aca="false">IF(L12&gt;0,1/L12,0)</f>
@@ -9092,88 +9131,88 @@
       </c>
       <c r="T13" s="136" t="n">
         <f aca="false">AVERAGE(B13:S13)</f>
-        <v>41.6666666666667</v>
+        <v>37.8703703703704</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="132" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B14" s="104" t="n">
         <f aca="false">B11*B13</f>
-        <v>1225</v>
+        <v>980</v>
       </c>
       <c r="C14" s="104" t="n">
         <f aca="false">C11*C13</f>
-        <v>1250</v>
+        <v>1008.57142857143</v>
       </c>
       <c r="D14" s="104" t="n">
         <f aca="false">D11*D13</f>
-        <v>1675</v>
+        <v>2030.76923076923</v>
       </c>
       <c r="E14" s="104" t="n">
         <f aca="false">E11*E13</f>
-        <v>2100</v>
+        <v>2632.89473684211</v>
       </c>
       <c r="F14" s="104" t="n">
         <f aca="false">F11*F13</f>
-        <v>2225</v>
+        <v>2869.23076923077</v>
       </c>
       <c r="G14" s="104" t="n">
         <f aca="false">G11*G13</f>
-        <v>2350</v>
+        <v>4200.98039215686</v>
       </c>
       <c r="H14" s="104" t="n">
         <f aca="false">H11*H13</f>
-        <v>4800</v>
+        <v>4625.39682539683</v>
       </c>
       <c r="I14" s="104" t="n">
         <f aca="false">I11*I13</f>
-        <v>5000</v>
+        <v>4744.44444444445</v>
       </c>
       <c r="J14" s="104" t="n">
         <f aca="false">J11*J13</f>
-        <v>5000</v>
+        <v>4922.77777777778</v>
       </c>
       <c r="K14" s="104" t="n">
         <f aca="false">K11*K13</f>
-        <v>5100</v>
+        <v>4981.6425120773</v>
       </c>
       <c r="L14" s="104" t="n">
         <f aca="false">L11*L13</f>
-        <v>5200</v>
+        <v>7608.125</v>
       </c>
       <c r="M14" s="104" t="n">
         <f aca="false">M11*M13</f>
-        <v>5300</v>
+        <v>7617.03296703297</v>
       </c>
       <c r="N14" s="104" t="n">
         <f aca="false">N11*N13</f>
-        <v>5400</v>
+        <v>8246.56862745098</v>
       </c>
       <c r="O14" s="104" t="n">
         <f aca="false">O11*O13</f>
-        <v>5750</v>
+        <v>8510.81081081081</v>
       </c>
       <c r="P14" s="104" t="n">
         <f aca="false">P11*P13</f>
-        <v>5900</v>
+        <v>9129.7520661157</v>
       </c>
       <c r="Q14" s="104" t="n">
         <f aca="false">Q11*Q13</f>
-        <v>5900</v>
+        <v>9211.45038167939</v>
       </c>
       <c r="R14" s="104" t="n">
         <f aca="false">R11*R13</f>
-        <v>6200</v>
+        <v>9954.67625899281</v>
       </c>
       <c r="S14" s="104" t="n">
         <f aca="false">S11*S13</f>
-        <v>6250</v>
+        <v>10193.9189189189</v>
       </c>
       <c r="T14" s="133" t="n">
         <f aca="false">AVERAGE(B14:S14)</f>
-        <v>4256.94444444444</v>
+        <v>5748.2801749038</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9200,7 +9239,7 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="131" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B16" s="131"/>
       <c r="C16" s="131"/>
@@ -9224,88 +9263,88 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="137" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B17" s="138" t="n">
         <f aca="false">IF(B7&gt;0,B14/B7,0)</f>
-        <v>28.8235294117647</v>
+        <v>23.0588235294118</v>
       </c>
       <c r="C17" s="138" t="n">
         <f aca="false">IF(C7&gt;0,C14/C7,0)</f>
-        <v>20.8333333333333</v>
+        <v>16.8095238095238</v>
       </c>
       <c r="D17" s="138" t="n">
         <f aca="false">IF(D7&gt;0,D14/D7,0)</f>
-        <v>45.6818181818182</v>
+        <v>55.3846153846154</v>
       </c>
       <c r="E17" s="138" t="n">
         <f aca="false">IF(E7&gt;0,E14/E7,0)</f>
-        <v>15.1807228915663</v>
+        <v>19.0329740012682</v>
       </c>
       <c r="F17" s="138" t="n">
         <f aca="false">IF(F7&gt;0,F14/F7,0)</f>
-        <v>7.38151658767773</v>
+        <v>9.51877506379876</v>
       </c>
       <c r="G17" s="138" t="n">
         <f aca="false">IF(G7&gt;0,G14/G7,0)</f>
-        <v>8.58447488584475</v>
+        <v>15.3460470946369</v>
       </c>
       <c r="H17" s="138" t="n">
         <f aca="false">IF(H7&gt;0,H14/H7,0)</f>
-        <v>14.3820224719101</v>
+        <v>13.8588668925748</v>
       </c>
       <c r="I17" s="138" t="n">
         <f aca="false">IF(I7&gt;0,I14/I7,0)</f>
-        <v>16.3636363636364</v>
+        <v>15.5272727272727</v>
       </c>
       <c r="J17" s="138" t="n">
         <f aca="false">IF(J7&gt;0,J14/J7,0)</f>
-        <v>15.8450704225352</v>
+        <v>15.6003521126761</v>
       </c>
       <c r="K17" s="138" t="n">
         <f aca="false">IF(K7&gt;0,K14/K7,0)</f>
-        <v>15.8275862068966</v>
+        <v>15.4602698650675</v>
       </c>
       <c r="L17" s="138" t="n">
         <f aca="false">IF(L7&gt;0,L14/L7,0)</f>
-        <v>18.5113268608414</v>
+        <v>27.0839401294498</v>
       </c>
       <c r="M17" s="138" t="n">
         <f aca="false">IF(M7&gt;0,M14/M7,0)</f>
-        <v>18.391167192429</v>
+        <v>26.431344680556</v>
       </c>
       <c r="N17" s="138" t="n">
         <f aca="false">IF(N7&gt;0,N14/N7,0)</f>
-        <v>18.2208588957055</v>
+        <v>27.8258450619512</v>
       </c>
       <c r="O17" s="138" t="n">
         <f aca="false">IF(O7&gt;0,O14/O7,0)</f>
-        <v>12.8094059405941</v>
+        <v>18.9597270537865</v>
       </c>
       <c r="P17" s="138" t="n">
         <f aca="false">IF(P7&gt;0,P14/P7,0)</f>
-        <v>14.2857142857143</v>
+        <v>22.1059372060913</v>
       </c>
       <c r="Q17" s="138" t="n">
         <f aca="false">IF(Q7&gt;0,Q14/Q7,0)</f>
-        <v>14.0142517814727</v>
+        <v>21.8799296476945</v>
       </c>
       <c r="R17" s="138" t="n">
         <f aca="false">IF(R7&gt;0,R14/R7,0)</f>
-        <v>11.5617715617716</v>
+        <v>18.5634988512686</v>
       </c>
       <c r="S17" s="138" t="n">
         <f aca="false">IF(S7&gt;0,S14/S7,0)</f>
-        <v>12.8718535469108</v>
+        <v>20.9943410229451</v>
       </c>
       <c r="T17" s="139" t="n">
         <f aca="false">AVERAGE(B17:S17)</f>
-        <v>17.1983367123568</v>
+        <v>21.3023380074772</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="128" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B18" s="128"/>
       <c r="C18" s="128"/>
@@ -9351,7 +9390,7 @@
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="131" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B20" s="131"/>
       <c r="C20" s="131"/>
@@ -9375,70 +9414,88 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="90" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B21" s="91" t="n">
+        <f aca="false">IF('A — Ricavi'!B9&gt;0,B11-('B1 — Infrastruttura'!B18+'B6 — Costi Variabili'!B16)/'A — Ricavi'!B9,0)</f>
         <v>1</v>
       </c>
       <c r="C21" s="91" t="n">
-        <v>14</v>
+        <f aca="false">IF('A — Ricavi'!C9&gt;0,C11-('B1 — Infrastruttura'!C18+'B6 — Costi Variabili'!C16)/'A — Ricavi'!C9,0)</f>
+        <v>14.4285714285714</v>
       </c>
       <c r="D21" s="91" t="n">
-        <v>41</v>
+        <f aca="false">IF('A — Ricavi'!D9&gt;0,D11-('B1 — Infrastruttura'!D18+'B6 — Costi Variabili'!D16)/'A — Ricavi'!D9,0)</f>
+        <v>54.4615384615385</v>
       </c>
       <c r="E21" s="91" t="n">
-        <v>59</v>
+        <f aca="false">IF('A — Ricavi'!E9&gt;0,E11-('B1 — Infrastruttura'!E18+'B6 — Costi Variabili'!E16)/'A — Ricavi'!E9,0)</f>
+        <v>80.3157894736842</v>
       </c>
       <c r="F21" s="91" t="n">
-        <v>63</v>
+        <f aca="false">IF('A — Ricavi'!F9&gt;0,F11-('B1 — Infrastruttura'!F18+'B6 — Costi Variabili'!F16)/'A — Ricavi'!F9,0)</f>
+        <v>88.4615384615385</v>
       </c>
       <c r="G21" s="91" t="n">
-        <v>67</v>
+        <f aca="false">IF('A — Ricavi'!G9&gt;0,G11-('B1 — Infrastruttura'!G18+'B6 — Costi Variabili'!G16)/'A — Ricavi'!G9,0)</f>
+        <v>99.6470588235294</v>
       </c>
       <c r="H21" s="91" t="n">
-        <v>70</v>
+        <f aca="false">IF('A — Ricavi'!H9&gt;0,H11-('B1 — Infrastruttura'!H18+'B6 — Costi Variabili'!H16)/'A — Ricavi'!H9,0)</f>
+        <v>112.5</v>
       </c>
       <c r="I21" s="91" t="n">
-        <v>73</v>
+        <f aca="false">IF('A — Ricavi'!I9&gt;0,I11-('B1 — Infrastruttura'!I18+'B6 — Costi Variabili'!I16)/'A — Ricavi'!I9,0)</f>
+        <v>115.921568627451</v>
       </c>
       <c r="J21" s="91" t="n">
-        <v>73</v>
+        <f aca="false">IF('A — Ricavi'!J9&gt;0,J11-('B1 — Infrastruttura'!J18+'B6 — Costi Variabili'!J16)/'A — Ricavi'!J9,0)</f>
+        <v>120.616666666667</v>
       </c>
       <c r="K21" s="91" t="n">
-        <v>75</v>
+        <f aca="false">IF('A — Ricavi'!K9&gt;0,K11-('B1 — Infrastruttura'!K18+'B6 — Costi Variabili'!K16)/'A — Ricavi'!K9,0)</f>
+        <v>121.913043478261</v>
       </c>
       <c r="L21" s="91" t="n">
-        <v>76</v>
+        <f aca="false">IF('A — Ricavi'!L9&gt;0,L11-('B1 — Infrastruttura'!L18+'B6 — Costi Variabili'!L16)/'A — Ricavi'!L9,0)</f>
+        <v>124.525</v>
       </c>
       <c r="M21" s="91" t="n">
-        <v>77</v>
+        <f aca="false">IF('A — Ricavi'!M9&gt;0,M11-('B1 — Infrastruttura'!M18+'B6 — Costi Variabili'!M16)/'A — Ricavi'!M9,0)</f>
+        <v>123.989010989011</v>
       </c>
       <c r="N21" s="91" t="n">
-        <v>79</v>
+        <f aca="false">IF('A — Ricavi'!N9&gt;0,N11-('B1 — Infrastruttura'!N18+'B6 — Costi Variabili'!N16)/'A — Ricavi'!N9,0)</f>
+        <v>135.803921568627</v>
       </c>
       <c r="O21" s="91" t="n">
-        <v>85</v>
+        <f aca="false">IF('A — Ricavi'!O9&gt;0,O11-('B1 — Infrastruttura'!O18+'B6 — Costi Variabili'!O16)/'A — Ricavi'!O9,0)</f>
+        <v>140.234234234234</v>
       </c>
       <c r="P21" s="91" t="n">
-        <v>87</v>
+        <f aca="false">IF('A — Ricavi'!P9&gt;0,P11-('B1 — Infrastruttura'!P18+'B6 — Costi Variabili'!P16)/'A — Ricavi'!P9,0)</f>
+        <v>152.02479338843</v>
       </c>
       <c r="Q21" s="91" t="n">
-        <v>87</v>
+        <f aca="false">IF('A — Ricavi'!Q9&gt;0,Q11-('B1 — Infrastruttura'!Q18+'B6 — Costi Variabili'!Q16)/'A — Ricavi'!Q9,0)</f>
+        <v>153.328244274809</v>
       </c>
       <c r="R21" s="91" t="n">
-        <v>92</v>
+        <f aca="false">IF('A — Ricavi'!R9&gt;0,R11-('B1 — Infrastruttura'!R18+'B6 — Costi Variabili'!R16)/'A — Ricavi'!R9,0)</f>
+        <v>167.58273381295</v>
       </c>
       <c r="S21" s="91" t="n">
-        <v>94</v>
+        <f aca="false">IF('A — Ricavi'!S9&gt;0,S11-('B1 — Infrastruttura'!S18+'B6 — Costi Variabili'!S16)/'A — Ricavi'!S9,0)</f>
+        <v>172.074324324324</v>
       </c>
       <c r="T21" s="72" t="n">
         <f aca="false">SUM(B21:S21)</f>
-        <v>1213</v>
+        <v>1978.82803801363</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="132" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B22" s="140" t="n">
         <f aca="false">IF(B21&gt;0,B7/B21,0)</f>
@@ -9446,80 +9503,80 @@
       </c>
       <c r="C22" s="140" t="n">
         <f aca="false">IF(C21&gt;0,C7/C21,0)</f>
-        <v>4.28571428571429</v>
+        <v>4.15841584158416</v>
       </c>
       <c r="D22" s="140" t="n">
         <f aca="false">IF(D21&gt;0,D7/D21,0)</f>
-        <v>0.894308943089431</v>
+        <v>0.673258003766478</v>
       </c>
       <c r="E22" s="140" t="n">
         <f aca="false">IF(E21&gt;0,E7/E21,0)</f>
-        <v>2.34463276836158</v>
+        <v>1.72236784622106</v>
       </c>
       <c r="F22" s="140" t="n">
         <f aca="false">IF(F21&gt;0,F7/F21,0)</f>
-        <v>4.78458049886621</v>
+        <v>3.40745341614907</v>
       </c>
       <c r="G22" s="140" t="n">
         <f aca="false">IF(G21&gt;0,G7/G21,0)</f>
-        <v>4.08582089552239</v>
+        <v>2.74719598583235</v>
       </c>
       <c r="H22" s="140" t="n">
         <f aca="false">IF(H21&gt;0,H7/H21,0)</f>
-        <v>4.76785714285714</v>
+        <v>2.96666666666667</v>
       </c>
       <c r="I22" s="140" t="n">
         <f aca="false">IF(I21&gt;0,I7/I21,0)</f>
-        <v>4.18569254185693</v>
+        <v>2.63588182228236</v>
       </c>
       <c r="J22" s="140" t="n">
         <f aca="false">IF(J21&gt;0,J7/J21,0)</f>
-        <v>4.32267884322679</v>
+        <v>2.61618534383492</v>
       </c>
       <c r="K22" s="140" t="n">
         <f aca="false">IF(K21&gt;0,K7/K21,0)</f>
-        <v>4.2962962962963</v>
+        <v>2.64304961166587</v>
       </c>
       <c r="L22" s="140" t="n">
         <f aca="false">IF(L21&gt;0,L7/L21,0)</f>
-        <v>3.69617224880383</v>
+        <v>2.25584493803727</v>
       </c>
       <c r="M22" s="140" t="n">
         <f aca="false">IF(M21&gt;0,M7/M21,0)</f>
-        <v>3.74262101534829</v>
+        <v>2.32425289856824</v>
       </c>
       <c r="N22" s="140" t="n">
         <f aca="false">IF(N21&gt;0,N7/N21,0)</f>
-        <v>3.75143843498274</v>
+        <v>2.18229070957919</v>
       </c>
       <c r="O22" s="140" t="n">
         <f aca="false">IF(O21&gt;0,O7/O21,0)</f>
-        <v>5.28104575163399</v>
+        <v>3.20099361857039</v>
       </c>
       <c r="P22" s="140" t="n">
         <f aca="false">IF(P21&gt;0,P7/P21,0)</f>
-        <v>4.74712643678161</v>
+        <v>2.71666213645012</v>
       </c>
       <c r="Q22" s="140" t="n">
         <f aca="false">IF(Q21&gt;0,Q7/Q21,0)</f>
-        <v>4.83908045977012</v>
+        <v>2.74574330379369</v>
       </c>
       <c r="R22" s="140" t="n">
         <f aca="false">IF(R21&gt;0,R7/R21,0)</f>
-        <v>5.82880434782609</v>
+        <v>3.19991199450502</v>
       </c>
       <c r="S22" s="140" t="n">
         <f aca="false">IF(S21&gt;0,S7/S21,0)</f>
-        <v>5.16548463356974</v>
+        <v>2.82177807445801</v>
       </c>
       <c r="T22" s="141" t="n">
         <f aca="false">AVERAGE(B22:S22)</f>
-        <v>6.30663086358375</v>
+        <v>4.86210845622027</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="128" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B23" s="128"/>
       <c r="C23" s="128"/>
@@ -9565,7 +9622,7 @@
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="131" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B25" s="131"/>
       <c r="C25" s="131"/>
@@ -9589,7 +9646,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B26" s="119" t="n">
         <f aca="false">IF('MRR Waterfall'!B5&gt;0,('MRR Waterfall'!B12-'MRR Waterfall'!B5)/'MRR Waterfall'!B5,0)</f>
@@ -9670,169 +9727,169 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!B31&gt;0,MASTER!B20/'A — Ricavi'!B31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!B9&gt;0,MASTER!B20/MASTER!B9,0)</f>
+        <v>-21.0867346938776</v>
       </c>
       <c r="C27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!C31&gt;0,MASTER!C20/'A — Ricavi'!C31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!C9&gt;0,MASTER!C20/MASTER!C9,0)</f>
+        <v>-11.4759206798867</v>
       </c>
       <c r="D27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!D31&gt;0,MASTER!D20/'A — Ricavi'!D31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!D9&gt;0,MASTER!D20/MASTER!D9,0)</f>
+        <v>-3.31818181818182</v>
       </c>
       <c r="E27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!E31&gt;0,MASTER!E20/'A — Ricavi'!E31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!E9&gt;0,MASTER!E20/MASTER!E9,0)</f>
+        <v>-2.11444277861069</v>
       </c>
       <c r="F27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!F31&gt;0,MASTER!F20/'A — Ricavi'!F31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!F9&gt;0,MASTER!F20/MASTER!F9,0)</f>
+        <v>-1.59752010723861</v>
       </c>
       <c r="G27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!G31&gt;0,MASTER!G20/'A — Ricavi'!G31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!G9&gt;0,MASTER!G20/MASTER!G9,0)</f>
+        <v>-1.04760793465578</v>
       </c>
       <c r="H27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!H31&gt;0,MASTER!H20/'A — Ricavi'!H31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!H9&gt;0,MASTER!H20/MASTER!H9,0)</f>
+        <v>-0.990391214824983</v>
       </c>
       <c r="I27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!I31&gt;0,MASTER!I20/'A — Ricavi'!I31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!I9&gt;0,MASTER!I20/MASTER!I9,0)</f>
+        <v>-0.648160903705745</v>
       </c>
       <c r="J27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!J31&gt;0,MASTER!J20/'A — Ricavi'!J31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!J9&gt;0,MASTER!J20/MASTER!J9,0)</f>
+        <v>-0.396117819659181</v>
       </c>
       <c r="K27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!K31&gt;0,MASTER!K20/'A — Ricavi'!K31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!K9&gt;0,MASTER!K20/MASTER!K9,0)</f>
+        <v>-0.236617532971296</v>
       </c>
       <c r="L27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!L31&gt;0,MASTER!L20/'A — Ricavi'!L31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!L9&gt;0,MASTER!L20/MASTER!L9,0)</f>
+        <v>-0.22755278074427</v>
       </c>
       <c r="M27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!M31&gt;0,MASTER!M20/'A — Ricavi'!M31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!M9&gt;0,MASTER!M20/MASTER!M9,0)</f>
+        <v>-0.113178965591863</v>
       </c>
       <c r="N27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!N31&gt;0,MASTER!N20/'A — Ricavi'!N31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!N9&gt;0,MASTER!N20/MASTER!N9,0)</f>
+        <v>0.0481483683052963</v>
       </c>
       <c r="O27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!O31&gt;0,MASTER!O20/'A — Ricavi'!O31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!O9&gt;0,MASTER!O20/MASTER!O9,0)</f>
+        <v>0.000476341695776437</v>
       </c>
       <c r="P27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!P31&gt;0,MASTER!P20/'A — Ricavi'!P31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!P9&gt;0,MASTER!P20/MASTER!P9,0)</f>
+        <v>0.120756766542953</v>
       </c>
       <c r="Q27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!Q31&gt;0,MASTER!Q20/'A — Ricavi'!Q31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!Q9&gt;0,MASTER!Q20/MASTER!Q9,0)</f>
+        <v>0.17543714262037</v>
       </c>
       <c r="R27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!R31&gt;0,MASTER!R20/'A — Ricavi'!R31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!R9&gt;0,MASTER!R20/MASTER!R9,0)</f>
+        <v>0.263315747633157</v>
       </c>
       <c r="S27" s="119" t="n">
-        <f aca="false">IF('A — Ricavi'!S31&gt;0,MASTER!S20/'A — Ricavi'!S31,0)</f>
-        <v>0</v>
+        <f aca="false">IF(MASTER!S9&gt;0,MASTER!S20/MASTER!S9,0)</f>
+        <v>0.309040896135746</v>
       </c>
       <c r="T27" s="120" t="n">
         <f aca="false">AVERAGE(B27:S27)</f>
-        <v>0</v>
+        <v>-2.35195844261195</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="137" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B28" s="142" t="n">
         <f aca="false">B26+B27</f>
-        <v>0</v>
+        <v>-21.0867346938776</v>
       </c>
       <c r="C28" s="142" t="n">
         <f aca="false">C26+C27</f>
-        <v>0.744897959183674</v>
+        <v>-10.731022720703</v>
       </c>
       <c r="D28" s="142" t="n">
         <f aca="false">D26+D27</f>
-        <v>1.10764872521246</v>
+        <v>-2.21053309296935</v>
       </c>
       <c r="E28" s="142" t="n">
         <f aca="false">E26+E27</f>
-        <v>0.549086757990868</v>
+        <v>-1.56535602061983</v>
       </c>
       <c r="F28" s="142" t="n">
         <f aca="false">F26+F27</f>
-        <v>0.368980612883052</v>
+        <v>-1.22853949435555</v>
       </c>
       <c r="G28" s="142" t="n">
         <f aca="false">G26+G27</f>
-        <v>0.3015941404567</v>
+        <v>-0.746013794199076</v>
       </c>
       <c r="H28" s="142" t="n">
         <f aca="false">H26+H27</f>
-        <v>0.249292675259352</v>
+        <v>-0.74109853956563</v>
       </c>
       <c r="I28" s="142" t="n">
         <f aca="false">I26+I27</f>
-        <v>0.227541954590326</v>
+        <v>-0.420618949115419</v>
       </c>
       <c r="J28" s="142" t="n">
         <f aca="false">J26+J27</f>
-        <v>0.183428458964771</v>
+        <v>-0.21268936069441</v>
       </c>
       <c r="K28" s="142" t="n">
         <f aca="false">K26+K27</f>
-        <v>0.159208118449509</v>
+        <v>-0.0774094145217864</v>
       </c>
       <c r="L28" s="142" t="n">
         <f aca="false">L26+L27</f>
-        <v>0.16742209631728</v>
+        <v>-0.0601306844269897</v>
       </c>
       <c r="M28" s="142" t="n">
         <f aca="false">M26+M27</f>
-        <v>0.145994208494209</v>
+        <v>0.0328152429023453</v>
       </c>
       <c r="N28" s="142" t="n">
         <f aca="false">N26+N27</f>
-        <v>0.129589183567343</v>
+        <v>0.177737551872639</v>
       </c>
       <c r="O28" s="142" t="n">
         <f aca="false">O26+O27</f>
-        <v>0.0993479442130049</v>
+        <v>0.0998242859087813</v>
       </c>
       <c r="P28" s="142" t="n">
         <f aca="false">P26+P27</f>
-        <v>0.0978823529411765</v>
+        <v>0.218639119484129</v>
       </c>
       <c r="Q28" s="142" t="n">
         <f aca="false">Q26+Q27</f>
-        <v>0.0881505935239166</v>
+        <v>0.263587736144286</v>
       </c>
       <c r="R28" s="142" t="n">
         <f aca="false">R26+R27</f>
-        <v>0.0698217179902755</v>
+        <v>0.333137465623433</v>
       </c>
       <c r="S28" s="142" t="n">
         <f aca="false">S26+S27</f>
-        <v>0.0709928542380759</v>
+        <v>0.380033750373822</v>
       </c>
       <c r="T28" s="143" t="n">
         <f aca="false">AVERAGE(B28:S28)</f>
-        <v>0.264493353015333</v>
+        <v>-2.08746508959662</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="128" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B29" s="128"/>
       <c r="C29" s="128"/>
@@ -9878,7 +9935,7 @@
     </row>
     <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="131" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B31" s="131"/>
       <c r="C31" s="131"/>
@@ -9902,88 +9959,88 @@
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="132" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!B20-'MRR Waterfall'!B20)/B5*4,0)</f>
-        <v>0</v>
+        <f aca="false">IF(B5&gt;0,'MRR Waterfall'!B10*12/(B5*4),0)</f>
+        <v>3.40588235294118</v>
       </c>
       <c r="C32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!C20-'MRR Waterfall'!B20)/B5*4,0)</f>
-        <v>42.0705882352941</v>
+        <f aca="false">IF(C5&gt;0,'MRR Waterfall'!C10*12/(C5*4),0)</f>
+        <v>2.43333333333333</v>
       </c>
       <c r="D32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!D20-'MRR Waterfall'!B20)/C5*4,0)</f>
-        <v>146.933333333333</v>
+        <f aca="false">IF(D5&gt;0,'MRR Waterfall'!D10*12/(D5*4),0)</f>
+        <v>5.33181818181818</v>
       </c>
       <c r="E32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!E20-'MRR Waterfall'!B20)/D5*4,0)</f>
-        <v>253.963636363636</v>
+        <f aca="false">IF(E5&gt;0,'MRR Waterfall'!E10*12/(E5*4),0)</f>
+        <v>1.73855421686747</v>
       </c>
       <c r="F32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!F20-'MRR Waterfall'!B20)/E5*4,0)</f>
-        <v>115.431325301205</v>
+        <f aca="false">IF(F5&gt;0,'MRR Waterfall'!F10*12/(F5*4),0)</f>
+        <v>0.838862559241706</v>
       </c>
       <c r="G32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!G20-'MRR Waterfall'!B20)/F5*4,0)</f>
-        <v>64.3336492890995</v>
+        <f aca="false">IF(G5&gt;0,'MRR Waterfall'!G10*12/(G5*4),0)</f>
+        <v>0.958904109589041</v>
       </c>
       <c r="H32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!H20-'MRR Waterfall'!B20)/G5*4,0)</f>
-        <v>82.8712328767123</v>
+        <f aca="false">IF(H5&gt;0,'MRR Waterfall'!H10*12/(H5*4),0)</f>
+        <v>0.891011235955056</v>
       </c>
       <c r="I32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!I20-'MRR Waterfall'!B20)/H5*4,0)</f>
-        <v>85.9505617977528</v>
+        <f aca="false">IF(I5&gt;0,'MRR Waterfall'!I10*12/(I5*4),0)</f>
+        <v>1.00581818181818</v>
       </c>
       <c r="J32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!J20-'MRR Waterfall'!B20)/I5*4,0)</f>
-        <v>101.585454545455</v>
+        <f aca="false">IF(J5&gt;0,'MRR Waterfall'!J10*12/(J5*4),0)</f>
+        <v>0.984507042253521</v>
       </c>
       <c r="K32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!K20-'MRR Waterfall'!B20)/J5*4,0)</f>
-        <v>114.507042253521</v>
+        <f aca="false">IF(K5&gt;0,'MRR Waterfall'!K10*12/(K5*4),0)</f>
+        <v>0.99</v>
       </c>
       <c r="L32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!L20-'MRR Waterfall'!B20)/K5*4,0)</f>
-        <v>133.224827586207</v>
+        <f aca="false">IF(L5&gt;0,'MRR Waterfall'!L10*12/(L5*4),0)</f>
+        <v>1.14757281553398</v>
       </c>
       <c r="M32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!M20-'MRR Waterfall'!B20)/L5*4,0)</f>
-        <v>144.543689320388</v>
+        <f aca="false">IF(M5&gt;0,'MRR Waterfall'!M10*12/(M5*4),0)</f>
+        <v>1.14511041009464</v>
       </c>
       <c r="N32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!N20-'MRR Waterfall'!B20)/M5*4,0)</f>
-        <v>161.534384858044</v>
+        <f aca="false">IF(N5&gt;0,'MRR Waterfall'!N10*12/(N5*4),0)</f>
+        <v>1.14662576687117</v>
       </c>
       <c r="O32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!O20-'MRR Waterfall'!B20)/N5*4,0)</f>
-        <v>175.892024539877</v>
+        <f aca="false">IF(O5&gt;0,'MRR Waterfall'!O10*12/(O5*4),0)</f>
+        <v>0.81460396039604</v>
       </c>
       <c r="P32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!P20-'MRR Waterfall'!B20)/O5*4,0)</f>
-        <v>164.019801980198</v>
+        <f aca="false">IF(P5&gt;0,'MRR Waterfall'!P10*12/(P5*4),0)</f>
+        <v>0.906537530266344</v>
       </c>
       <c r="Q32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!Q20-'MRR Waterfall'!B20)/P5*4,0)</f>
-        <v>177.809200968523</v>
+        <f aca="false">IF(Q5&gt;0,'MRR Waterfall'!Q10*12/(Q5*4),0)</f>
+        <v>0.894299287410926</v>
       </c>
       <c r="R32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!R20-'MRR Waterfall'!B20)/Q5*4,0)</f>
-        <v>185.945843230404</v>
+        <f aca="false">IF(R5&gt;0,'MRR Waterfall'!R10*12/(R5*4),0)</f>
+        <v>0.753146853146853</v>
       </c>
       <c r="S32" s="144" t="n">
-        <f aca="false">IF(B5&gt;0,('MRR Waterfall'!S20-'MRR Waterfall'!B20)/R5*4,0)</f>
-        <v>204.106293706294</v>
+        <f aca="false">IF(S5&gt;0,'MRR Waterfall'!S10*12/(S5*4),0)</f>
+        <v>0.838901601830664</v>
       </c>
       <c r="T32" s="145" t="n">
         <f aca="false">AVERAGE(B32:S32)</f>
-        <v>130.817938343664</v>
+        <v>1.45697163552046</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="128" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B33" s="128"/>
       <c r="C33" s="128"/>
@@ -10051,7 +10108,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="81" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B1" s="81"/>
       <c r="C1" s="81"/>
@@ -10075,7 +10132,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -10161,7 +10218,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="146" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B4" s="146"/>
       <c r="C4" s="146"/>
@@ -10185,7 +10242,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B5" s="50" t="n">
         <f aca="false">MASTER!B30</f>
@@ -10266,7 +10323,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="82" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B6" s="82"/>
       <c r="C6" s="82"/>
@@ -10290,7 +10347,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B7" s="50" t="n">
         <f aca="false">'B5 — Ammortamenti'!B14</f>
@@ -10371,7 +10428,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B8" s="147" t="n">
         <v>0</v>
@@ -10434,7 +10491,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B9" s="147" t="n">
         <v>0</v>
@@ -10497,7 +10554,7 @@
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="148" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B10" s="149" t="n">
         <f aca="false">B5+B7+B8+B9</f>
@@ -10600,7 +10657,7 @@
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="146" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B12" s="146"/>
       <c r="C12" s="146"/>
@@ -10624,7 +10681,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="41" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B13" s="147" t="n">
         <v>0</v>
@@ -10687,7 +10744,7 @@
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="148" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B14" s="149" t="n">
         <f aca="false">B13</f>
@@ -10790,7 +10847,7 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="146" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B16" s="146"/>
       <c r="C16" s="146"/>
@@ -10814,7 +10871,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B17" s="147" t="n">
         <v>0</v>
@@ -10877,7 +10934,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="41" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B18" s="55" t="n">
         <v>10000</v>
@@ -10940,7 +10997,7 @@
     </row>
     <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="148" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B19" s="149" t="n">
         <f aca="false">B17+B18</f>
@@ -11043,7 +11100,7 @@
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="151" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B21" s="151"/>
       <c r="C21" s="151"/>
@@ -11067,7 +11124,7 @@
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="152" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B22" s="153" t="n">
         <f aca="false">B10+B14+B19</f>
@@ -11148,7 +11205,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="90" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B23" s="91" t="n">
         <v>0</v>
@@ -11228,7 +11285,7 @@
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="155" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B24" s="156" t="n">
         <f aca="false">B23+B22</f>
@@ -11331,7 +11388,7 @@
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -11355,7 +11412,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B27" s="50" t="n">
         <f aca="false">B22</f>
@@ -11436,7 +11493,7 @@
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="158" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B28" s="159" t="n">
         <f aca="false">IF(B27&lt;0,-B24/B27,IF(B24&gt;0,99,0))</f>
@@ -11517,7 +11574,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="128" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B29" s="128"/>
       <c r="C29" s="128"/>
@@ -11541,7 +11598,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="161" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B30" s="161"/>
       <c r="C30" s="161"/>
@@ -11605,7 +11662,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -11629,7 +11686,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -11715,7 +11772,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="151" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B4" s="151"/>
       <c r="C4" s="151"/>
@@ -11739,7 +11796,7 @@
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -11763,7 +11820,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="90" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B6" s="123" t="n">
         <v>0</v>
@@ -11826,7 +11883,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="162" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B7" s="163" t="n">
         <v>-200</v>
@@ -11889,7 +11946,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B8" s="50" t="n">
         <f aca="false">MAX(0,B6+B7)</f>
@@ -11970,7 +12027,7 @@
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -11994,7 +12051,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="41" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!B24</f>
@@ -12075,7 +12132,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B11" s="147" t="n">
         <v>0</v>
@@ -12138,7 +12195,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="41" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(B10*0.025/12,0))</f>
@@ -12219,7 +12276,7 @@
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="124" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B13" s="46" t="n">
         <f aca="false">B10+B11+B12</f>
@@ -12300,7 +12357,7 @@
     </row>
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="164" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B14" s="58" t="n">
         <f aca="false">B8+B13</f>
@@ -12403,7 +12460,7 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="151" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B16" s="151"/>
       <c r="C16" s="151"/>
@@ -12427,7 +12484,7 @@
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -12451,7 +12508,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="41" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B18" s="147" t="n">
         <v>0</v>
@@ -12514,7 +12571,7 @@
     </row>
     <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -12538,7 +12595,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B20" s="55" t="n">
         <v>866</v>
@@ -12601,7 +12658,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="41" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B21" s="147" t="n">
         <v>0</v>
@@ -12664,227 +12721,227 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="41" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B22" s="55" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="C22" s="55" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="D22" s="55" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="E22" s="55" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="F22" s="55" t="n">
-        <v>3100</v>
+        <v>0</v>
       </c>
       <c r="G22" s="55" t="n">
-        <v>3450</v>
+        <v>0</v>
       </c>
       <c r="H22" s="55" t="n">
-        <v>4700</v>
+        <v>0</v>
       </c>
       <c r="I22" s="55" t="n">
-        <v>4700</v>
+        <v>0</v>
       </c>
       <c r="J22" s="55" t="n">
-        <v>4700</v>
+        <v>0</v>
       </c>
       <c r="K22" s="55" t="n">
-        <v>4700</v>
+        <v>0</v>
       </c>
       <c r="L22" s="55" t="n">
-        <v>5550</v>
+        <v>0</v>
       </c>
       <c r="M22" s="55" t="n">
-        <v>5550</v>
+        <v>0</v>
       </c>
       <c r="N22" s="55" t="n">
-        <v>5550</v>
+        <v>0</v>
       </c>
       <c r="O22" s="55" t="n">
-        <v>6750</v>
+        <v>0</v>
       </c>
       <c r="P22" s="55" t="n">
-        <v>6750</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="55" t="n">
-        <v>6750</v>
+        <v>0</v>
       </c>
       <c r="R22" s="55" t="n">
-        <v>6750</v>
+        <v>0</v>
       </c>
       <c r="S22" s="55" t="n">
-        <v>6750</v>
+        <v>0</v>
       </c>
       <c r="T22" s="72" t="n">
         <f aca="false">SUM(B22:S22)</f>
-        <v>83500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="124" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B23" s="46" t="n">
-        <f aca="false">B20+B21+B22</f>
-        <v>2616</v>
+        <f aca="false">B20+B21</f>
+        <v>866</v>
       </c>
       <c r="C23" s="46" t="n">
-        <f aca="false">C20+C21+C22</f>
-        <v>2631</v>
+        <f aca="false">C20+C21</f>
+        <v>881</v>
       </c>
       <c r="D23" s="46" t="n">
-        <f aca="false">D20+D21+D22</f>
-        <v>2662</v>
+        <f aca="false">D20+D21</f>
+        <v>912</v>
       </c>
       <c r="E23" s="46" t="n">
-        <f aca="false">E20+E21+E22</f>
-        <v>3746</v>
+        <f aca="false">E20+E21</f>
+        <v>1246</v>
       </c>
       <c r="F23" s="46" t="n">
-        <f aca="false">F20+F21+F22</f>
-        <v>4650</v>
+        <f aca="false">F20+F21</f>
+        <v>1550</v>
       </c>
       <c r="G23" s="46" t="n">
-        <f aca="false">G20+G21+G22</f>
-        <v>5205</v>
+        <f aca="false">G20+G21</f>
+        <v>1755</v>
       </c>
       <c r="H23" s="46" t="n">
-        <f aca="false">H20+H21+H22</f>
-        <v>7020</v>
+        <f aca="false">H20+H21</f>
+        <v>2320</v>
       </c>
       <c r="I23" s="46" t="n">
-        <f aca="false">I20+I21+I22</f>
-        <v>7093</v>
+        <f aca="false">I20+I21</f>
+        <v>2393</v>
       </c>
       <c r="J23" s="46" t="n">
-        <f aca="false">J20+J21+J22</f>
-        <v>7174</v>
+        <f aca="false">J20+J21</f>
+        <v>2474</v>
       </c>
       <c r="K23" s="46" t="n">
-        <f aca="false">K20+K21+K22</f>
-        <v>7250</v>
+        <f aca="false">K20+K21</f>
+        <v>2550</v>
       </c>
       <c r="L23" s="46" t="n">
-        <f aca="false">L20+L21+L22</f>
-        <v>8539</v>
+        <f aca="false">L20+L21</f>
+        <v>2989</v>
       </c>
       <c r="M23" s="46" t="n">
-        <f aca="false">M20+M21+M22</f>
-        <v>8636</v>
+        <f aca="false">M20+M21</f>
+        <v>3086</v>
       </c>
       <c r="N23" s="46" t="n">
-        <f aca="false">N20+N21+N22</f>
-        <v>8753</v>
+        <f aca="false">N20+N21</f>
+        <v>3203</v>
       </c>
       <c r="O23" s="46" t="n">
-        <f aca="false">O20+O21+O22</f>
-        <v>10527</v>
+        <f aca="false">O20+O21</f>
+        <v>3777</v>
       </c>
       <c r="P23" s="46" t="n">
-        <f aca="false">P20+P21+P22</f>
-        <v>10635</v>
+        <f aca="false">P20+P21</f>
+        <v>3885</v>
       </c>
       <c r="Q23" s="46" t="n">
-        <f aca="false">Q20+Q21+Q22</f>
-        <v>10730</v>
+        <f aca="false">Q20+Q21</f>
+        <v>3980</v>
       </c>
       <c r="R23" s="46" t="n">
-        <f aca="false">R20+R21+R22</f>
-        <v>10827</v>
+        <f aca="false">R20+R21</f>
+        <v>4077</v>
       </c>
       <c r="S23" s="46" t="n">
-        <f aca="false">S20+S21+S22</f>
-        <v>10920</v>
+        <f aca="false">S20+S21</f>
+        <v>4170</v>
       </c>
       <c r="T23" s="125" t="n">
         <f aca="false">SUM(B23:S23)</f>
-        <v>129614</v>
+        <v>46114</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="165" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B24" s="166" t="n">
         <f aca="false">B18+B23</f>
-        <v>2616</v>
+        <v>866</v>
       </c>
       <c r="C24" s="166" t="n">
         <f aca="false">C18+C23</f>
-        <v>2631</v>
+        <v>881</v>
       </c>
       <c r="D24" s="166" t="n">
         <f aca="false">D18+D23</f>
-        <v>2662</v>
+        <v>912</v>
       </c>
       <c r="E24" s="166" t="n">
         <f aca="false">E18+E23</f>
-        <v>3746</v>
+        <v>1246</v>
       </c>
       <c r="F24" s="166" t="n">
         <f aca="false">F18+F23</f>
-        <v>4650</v>
+        <v>1550</v>
       </c>
       <c r="G24" s="166" t="n">
         <f aca="false">G18+G23</f>
-        <v>5205</v>
+        <v>1755</v>
       </c>
       <c r="H24" s="166" t="n">
         <f aca="false">H18+H23</f>
-        <v>7020</v>
+        <v>2320</v>
       </c>
       <c r="I24" s="166" t="n">
         <f aca="false">I18+I23</f>
-        <v>7093</v>
+        <v>2393</v>
       </c>
       <c r="J24" s="166" t="n">
         <f aca="false">J18+J23</f>
-        <v>7174</v>
+        <v>2474</v>
       </c>
       <c r="K24" s="166" t="n">
         <f aca="false">K18+K23</f>
-        <v>7250</v>
+        <v>2550</v>
       </c>
       <c r="L24" s="166" t="n">
         <f aca="false">L18+L23</f>
-        <v>8539</v>
+        <v>2989</v>
       </c>
       <c r="M24" s="166" t="n">
         <f aca="false">M18+M23</f>
-        <v>8636</v>
+        <v>3086</v>
       </c>
       <c r="N24" s="166" t="n">
         <f aca="false">N18+N23</f>
-        <v>8753</v>
+        <v>3203</v>
       </c>
       <c r="O24" s="166" t="n">
         <f aca="false">O18+O23</f>
-        <v>10527</v>
+        <v>3777</v>
       </c>
       <c r="P24" s="166" t="n">
         <f aca="false">P18+P23</f>
-        <v>10635</v>
+        <v>3885</v>
       </c>
       <c r="Q24" s="166" t="n">
         <f aca="false">Q18+Q23</f>
-        <v>10730</v>
+        <v>3980</v>
       </c>
       <c r="R24" s="166" t="n">
         <f aca="false">R18+R23</f>
-        <v>10827</v>
+        <v>4077</v>
       </c>
       <c r="S24" s="166" t="n">
         <f aca="false">S18+S23</f>
-        <v>10920</v>
+        <v>4170</v>
       </c>
       <c r="T24" s="167" t="n">
         <f aca="false">SUM(B24:S24)</f>
-        <v>129614</v>
+        <v>46114</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12911,7 +12968,7 @@
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="151" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B26" s="151"/>
       <c r="C26" s="151"/>
@@ -12935,70 +12992,70 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="41" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B27" s="55" t="n">
         <v>10001</v>
       </c>
       <c r="C27" s="55" t="n">
-        <v>1</v>
+        <v>10001</v>
       </c>
       <c r="D27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="E27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="F27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="G27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="H27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="I27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="J27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="K27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="L27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="M27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="N27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="O27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="P27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="Q27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="R27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="S27" s="55" t="n">
-        <v>75001</v>
+        <v>85001</v>
       </c>
       <c r="T27" s="72" t="n">
         <f aca="false">SUM(B27:S27)</f>
-        <v>1210018</v>
+        <v>1380018</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="90" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B28" s="91" t="n">
         <v>0</v>
@@ -13078,7 +13135,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="41" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B29" s="50" t="n">
         <f aca="false">MASTER!B30</f>
@@ -13159,7 +13216,7 @@
     </row>
     <row r="30" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="137" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B30" s="168" t="n">
         <f aca="false">B27+B28+B29</f>
@@ -13167,75 +13224,75 @@
       </c>
       <c r="C30" s="168" t="n">
         <f aca="false">C27+C28+C29</f>
-        <v>-8183</v>
+        <v>1817</v>
       </c>
       <c r="D30" s="168" t="n">
         <f aca="false">D27+D28+D29</f>
-        <v>63313</v>
+        <v>73313</v>
       </c>
       <c r="E30" s="168" t="n">
         <f aca="false">E27+E28+E29</f>
-        <v>59132</v>
+        <v>69132</v>
       </c>
       <c r="F30" s="168" t="n">
         <f aca="false">F27+F28+F29</f>
-        <v>54415</v>
+        <v>64415</v>
       </c>
       <c r="G30" s="168" t="n">
         <f aca="false">G27+G28+G29</f>
-        <v>49976</v>
+        <v>59976</v>
       </c>
       <c r="H30" s="168" t="n">
         <f aca="false">H27+H28+H29</f>
-        <v>44284</v>
+        <v>54284</v>
       </c>
       <c r="I30" s="168" t="n">
         <f aca="false">I27+I28+I29</f>
-        <v>39659</v>
+        <v>49659</v>
       </c>
       <c r="J30" s="168" t="n">
         <f aca="false">J27+J28+J29</f>
-        <v>36229</v>
+        <v>46229</v>
       </c>
       <c r="K30" s="168" t="n">
         <f aca="false">K27+K28+K29</f>
-        <v>33869</v>
+        <v>43869</v>
       </c>
       <c r="L30" s="168" t="n">
         <f aca="false">L27+L28+L29</f>
-        <v>31199</v>
+        <v>41199</v>
       </c>
       <c r="M30" s="168" t="n">
         <f aca="false">M27+M28+M29</f>
-        <v>29730</v>
+        <v>39730</v>
       </c>
       <c r="N30" s="168" t="n">
         <f aca="false">N27+N28+N29</f>
-        <v>30400.53</v>
+        <v>40400.53</v>
       </c>
       <c r="O30" s="168" t="n">
         <f aca="false">O27+O28+O29</f>
-        <v>30493.539</v>
+        <v>40493.539</v>
       </c>
       <c r="P30" s="168" t="n">
         <f aca="false">P27+P28+P29</f>
-        <v>32503.687</v>
+        <v>42503.687</v>
       </c>
       <c r="Q30" s="168" t="n">
         <f aca="false">Q27+Q28+Q29</f>
-        <v>35642.921</v>
+        <v>45642.921</v>
       </c>
       <c r="R30" s="168" t="n">
         <f aca="false">R27+R28+R29</f>
-        <v>41004.998</v>
+        <v>51004.998</v>
       </c>
       <c r="S30" s="168" t="n">
         <f aca="false">S27+S28+S29</f>
-        <v>47836.473</v>
+        <v>57836.473</v>
       </c>
       <c r="T30" s="169" t="n">
         <f aca="false">SUM(B30:S30)</f>
-        <v>657373.148</v>
+        <v>827373.148</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13262,7 +13319,7 @@
     </row>
     <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -13286,168 +13343,168 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="41" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B33" s="50" t="n">
         <f aca="false">B14-B24-B30</f>
-        <v>-2404</v>
+        <v>-654</v>
       </c>
       <c r="C33" s="50" t="n">
         <f aca="false">C14-C24-C30</f>
-        <v>7741</v>
+        <v>-509</v>
       </c>
       <c r="D33" s="50" t="n">
         <f aca="false">D14-D24-D30</f>
-        <v>7351</v>
+        <v>-899</v>
       </c>
       <c r="E33" s="50" t="n">
         <f aca="false">E14-E24-E30</f>
-        <v>6435</v>
+        <v>-1065</v>
       </c>
       <c r="F33" s="50" t="n">
         <f aca="false">F14-F24-F30</f>
-        <v>5669</v>
+        <v>-1231</v>
       </c>
       <c r="G33" s="50" t="n">
         <f aca="false">G14-G24-G30</f>
-        <v>5141</v>
+        <v>-1409</v>
       </c>
       <c r="H33" s="50" t="n">
         <f aca="false">H14-H24-H30</f>
-        <v>3679</v>
+        <v>-1621</v>
       </c>
       <c r="I33" s="50" t="n">
         <f aca="false">I14-I24-I30</f>
-        <v>3451</v>
+        <v>-1849</v>
       </c>
       <c r="J33" s="50" t="n">
         <f aca="false">J14-J24-J30</f>
-        <v>3224</v>
+        <v>-2076</v>
       </c>
       <c r="K33" s="50" t="n">
         <f aca="false">K14-K24-K30</f>
-        <v>2994</v>
+        <v>-2306</v>
       </c>
       <c r="L33" s="50" t="n">
         <f aca="false">L14-L24-L30</f>
-        <v>1821</v>
+        <v>-2629</v>
       </c>
       <c r="M33" s="50" t="n">
         <f aca="false">M14-M24-M30</f>
-        <v>1511</v>
+        <v>-2939</v>
       </c>
       <c r="N33" s="50" t="n">
         <f aca="false">N14-N24-N30</f>
-        <v>1202</v>
+        <v>-3248</v>
       </c>
       <c r="O33" s="50" t="n">
         <f aca="false">O14-O24-O30</f>
-        <v>-270</v>
+        <v>-3520</v>
       </c>
       <c r="P33" s="50" t="n">
         <f aca="false">P14-P24-P30</f>
-        <v>-563</v>
+        <v>-3813</v>
       </c>
       <c r="Q33" s="50" t="n">
         <f aca="false">Q14-Q24-Q30</f>
-        <v>-823</v>
+        <v>-4073</v>
       </c>
       <c r="R33" s="50" t="n">
         <f aca="false">R14-R24-R30</f>
-        <v>-1049</v>
+        <v>-4299</v>
       </c>
       <c r="S33" s="50" t="n">
         <f aca="false">S14-S24-S30</f>
-        <v>-1291</v>
+        <v>-4541</v>
       </c>
       <c r="T33" s="72" t="n">
         <f aca="false">SUM(B33:S33)</f>
-        <v>43819</v>
+        <v>-42681</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="90" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B34" s="126" t="str">
-        <f aca="false">IF(ABS(B33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(B33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(B33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-654)</v>
       </c>
       <c r="C34" s="126" t="str">
-        <f aca="false">IF(ABS(C33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(C33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(C33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-509)</v>
       </c>
       <c r="D34" s="126" t="str">
-        <f aca="false">IF(ABS(D33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(D33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(D33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-899)</v>
       </c>
       <c r="E34" s="126" t="str">
-        <f aca="false">IF(ABS(E33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(E33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(E33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-1065)</v>
       </c>
       <c r="F34" s="126" t="str">
-        <f aca="false">IF(ABS(F33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(F33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(F33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-1231)</v>
       </c>
       <c r="G34" s="126" t="str">
-        <f aca="false">IF(ABS(G33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(G33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(G33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-1409)</v>
       </c>
       <c r="H34" s="126" t="str">
-        <f aca="false">IF(ABS(H33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(H33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(H33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-1621)</v>
       </c>
       <c r="I34" s="126" t="str">
-        <f aca="false">IF(ABS(I33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(I33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(I33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-1849)</v>
       </c>
       <c r="J34" s="126" t="str">
-        <f aca="false">IF(ABS(J33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(J33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(J33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-2076)</v>
       </c>
       <c r="K34" s="126" t="str">
-        <f aca="false">IF(ABS(K33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(K33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(K33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-2306)</v>
       </c>
       <c r="L34" s="126" t="str">
-        <f aca="false">IF(ABS(L33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(L33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(L33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-2629)</v>
       </c>
       <c r="M34" s="126" t="str">
-        <f aca="false">IF(ABS(M33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(M33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(M33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-2939)</v>
       </c>
       <c r="N34" s="126" t="str">
-        <f aca="false">IF(ABS(N33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(N33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(N33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-3248)</v>
       </c>
       <c r="O34" s="126" t="str">
-        <f aca="false">IF(ABS(O33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(O33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(O33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-3520)</v>
       </c>
       <c r="P34" s="126" t="str">
-        <f aca="false">IF(ABS(P33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(P33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(P33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-3813)</v>
       </c>
       <c r="Q34" s="126" t="str">
-        <f aca="false">IF(ABS(Q33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(Q33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(Q33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-4073)</v>
       </c>
       <c r="R34" s="126" t="str">
-        <f aca="false">IF(ABS(R33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(R33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(R33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-4299)</v>
       </c>
       <c r="S34" s="126" t="str">
-        <f aca="false">IF(ABS(S33)&lt;15000,"✅ OK","⚠️ RIVEDI")</f>
-        <v>✅ OK</v>
+        <f aca="false">IF(ABS(S33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(S33,0) &amp; ")")</f>
+        <v>⚠️ RIVEDI (-4541)</v>
       </c>
       <c r="T34" s="127" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="170" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B35" s="170"/>
       <c r="C35" s="170"/>

</xml_diff>

<commit_message>
🔄 Switch B6=1 (SMB Phase 2 ON) — fee overage SMB attive
TOTALE A.4 ora include B2B (€80.580) + SMB (€49.456) = €130.036 su 18M
TOTALE PRODUZIONE M1: €348 (era €196 con solo subscription)
EBIT M3: -€2.992 (migliorato da -€3.504 con SMB fee attive)
</commit_message>
<xml_diff>
--- a/03-FINANCIAL-MODELS/DLOOP_Budget_Guerriglia_FULL_v2.xlsx
+++ b/03-FINANCIAL-MODELS/DLOOP_Budget_Guerriglia_FULL_v2.xlsx
@@ -5349,79 +5349,79 @@
       </c>
       <c r="B5" s="50" t="n">
         <f aca="false">MASTER!B9</f>
-        <v>196</v>
+        <v>348</v>
       </c>
       <c r="C5" s="50" t="n">
         <f aca="false">MASTER!C9</f>
-        <v>353</v>
+        <v>633</v>
       </c>
       <c r="D5" s="50" t="n">
         <f aca="false">MASTER!D9</f>
-        <v>1056</v>
+        <v>1568</v>
       </c>
       <c r="E5" s="50" t="n">
         <f aca="false">MASTER!E9</f>
-        <v>2001</v>
+        <v>2745</v>
       </c>
       <c r="F5" s="50" t="n">
         <f aca="false">MASTER!F9</f>
-        <v>2984</v>
+        <v>3984</v>
       </c>
       <c r="G5" s="50" t="n">
         <f aca="false">MASTER!G9</f>
-        <v>4285</v>
+        <v>5565</v>
       </c>
       <c r="H5" s="50" t="n">
         <f aca="false">MASTER!H9</f>
-        <v>5828</v>
+        <v>7444</v>
       </c>
       <c r="I5" s="50" t="n">
         <f aca="false">MASTER!I9</f>
-        <v>7259</v>
+        <v>9235</v>
       </c>
       <c r="J5" s="50" t="n">
         <f aca="false">MASTER!J9</f>
-        <v>8861</v>
+        <v>11197</v>
       </c>
       <c r="K5" s="50" t="n">
         <f aca="false">MASTER!K9</f>
-        <v>10312</v>
+        <v>13064</v>
       </c>
       <c r="L5" s="50" t="n">
         <f aca="false">MASTER!L9</f>
-        <v>12173</v>
+        <v>15365</v>
       </c>
       <c r="M5" s="50" t="n">
         <f aca="false">MASTER!M9</f>
-        <v>13863</v>
+        <v>17495</v>
       </c>
       <c r="N5" s="50" t="n">
         <f aca="false">MASTER!N9</f>
-        <v>16823</v>
+        <v>20895</v>
       </c>
       <c r="O5" s="50" t="n">
         <f aca="false">MASTER!O9</f>
-        <v>18894</v>
+        <v>23302</v>
       </c>
       <c r="P5" s="50" t="n">
         <f aca="false">MASTER!P9</f>
-        <v>22094</v>
+        <v>26918</v>
       </c>
       <c r="Q5" s="50" t="n">
         <f aca="false">MASTER!Q9</f>
-        <v>24134</v>
+        <v>29374</v>
       </c>
       <c r="R5" s="50" t="n">
         <f aca="false">MASTER!R9</f>
-        <v>27674</v>
+        <v>33226</v>
       </c>
       <c r="S5" s="50" t="n">
         <f aca="false">MASTER!S9</f>
-        <v>30174</v>
+        <v>36062</v>
       </c>
       <c r="T5" s="72" t="n">
         <f aca="false">SUM(B5:S5)</f>
-        <v>208964</v>
+        <v>258420</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5430,75 +5430,75 @@
       </c>
       <c r="B6" s="91" t="n">
         <f aca="false">MASTER!B9</f>
-        <v>196</v>
+        <v>348</v>
       </c>
       <c r="C6" s="91" t="n">
         <f aca="false">B6+MASTER!C9</f>
-        <v>549</v>
+        <v>981</v>
       </c>
       <c r="D6" s="91" t="n">
         <f aca="false">C6+MASTER!D9</f>
-        <v>1605</v>
+        <v>2549</v>
       </c>
       <c r="E6" s="91" t="n">
         <f aca="false">D6+MASTER!E9</f>
-        <v>3606</v>
+        <v>5294</v>
       </c>
       <c r="F6" s="91" t="n">
         <f aca="false">E6+MASTER!F9</f>
-        <v>6590</v>
+        <v>9278</v>
       </c>
       <c r="G6" s="91" t="n">
         <f aca="false">F6+MASTER!G9</f>
-        <v>10875</v>
+        <v>14843</v>
       </c>
       <c r="H6" s="91" t="n">
         <f aca="false">G6+MASTER!H9</f>
-        <v>16703</v>
+        <v>22287</v>
       </c>
       <c r="I6" s="91" t="n">
         <f aca="false">H6+MASTER!I9</f>
-        <v>23962</v>
+        <v>31522</v>
       </c>
       <c r="J6" s="91" t="n">
         <f aca="false">I6+MASTER!J9</f>
-        <v>32823</v>
+        <v>42719</v>
       </c>
       <c r="K6" s="91" t="n">
         <f aca="false">J6+MASTER!K9</f>
-        <v>43135</v>
+        <v>55783</v>
       </c>
       <c r="L6" s="91" t="n">
         <f aca="false">K6+MASTER!L9</f>
-        <v>55308</v>
+        <v>71148</v>
       </c>
       <c r="M6" s="91" t="n">
         <f aca="false">L6+MASTER!M9</f>
-        <v>69171</v>
+        <v>88643</v>
       </c>
       <c r="N6" s="91" t="n">
         <f aca="false">M6+MASTER!N9</f>
-        <v>85994</v>
+        <v>109538</v>
       </c>
       <c r="O6" s="91" t="n">
         <f aca="false">N6+MASTER!O9</f>
-        <v>104888</v>
+        <v>132840</v>
       </c>
       <c r="P6" s="91" t="n">
         <f aca="false">O6+MASTER!P9</f>
-        <v>126982</v>
+        <v>159758</v>
       </c>
       <c r="Q6" s="91" t="n">
         <f aca="false">P6+MASTER!Q9</f>
-        <v>151116</v>
+        <v>189132</v>
       </c>
       <c r="R6" s="91" t="n">
         <f aca="false">Q6+MASTER!R9</f>
-        <v>178790</v>
+        <v>222358</v>
       </c>
       <c r="S6" s="91" t="n">
         <f aca="false">R6+MASTER!S9</f>
-        <v>208964</v>
+        <v>258420</v>
       </c>
       <c r="T6" s="112"/>
     </row>
@@ -5856,79 +5856,79 @@
       </c>
       <c r="B12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!B9&gt;0,MASTER!B9/'A — Ricavi'!B9,0)</f>
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="C12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!C9&gt;0,MASTER!C9/'A — Ricavi'!C9,0)</f>
-        <v>50.4285714285714</v>
+        <v>90.4285714285714</v>
       </c>
       <c r="D12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!D9&gt;0,MASTER!D9/'A — Ricavi'!D9,0)</f>
-        <v>81.2307692307692</v>
+        <v>120.615384615385</v>
       </c>
       <c r="E12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!E9&gt;0,MASTER!E9/'A — Ricavi'!E9,0)</f>
-        <v>105.315789473684</v>
+        <v>144.473684210526</v>
       </c>
       <c r="F12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!F9&gt;0,MASTER!F9/'A — Ricavi'!F9,0)</f>
-        <v>114.769230769231</v>
+        <v>153.230769230769</v>
       </c>
       <c r="G12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!G9&gt;0,MASTER!G9/'A — Ricavi'!G9,0)</f>
-        <v>126.029411764706</v>
+        <v>163.676470588235</v>
       </c>
       <c r="H12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!H9&gt;0,MASTER!H9/'A — Ricavi'!H9,0)</f>
-        <v>138.761904761905</v>
+        <v>177.238095238095</v>
       </c>
       <c r="I12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!I9&gt;0,MASTER!I9/'A — Ricavi'!I9,0)</f>
-        <v>142.333333333333</v>
+        <v>181.078431372549</v>
       </c>
       <c r="J12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!J9&gt;0,MASTER!J9/'A — Ricavi'!J9,0)</f>
-        <v>147.683333333333</v>
+        <v>186.616666666667</v>
       </c>
       <c r="K12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!K9&gt;0,MASTER!K9/'A — Ricavi'!K9,0)</f>
-        <v>149.449275362319</v>
+        <v>189.333333333333</v>
       </c>
       <c r="L12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!L9&gt;0,MASTER!L9/'A — Ricavi'!L9,0)</f>
-        <v>152.1625</v>
+        <v>192.0625</v>
       </c>
       <c r="M12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!M9&gt;0,MASTER!M9/'A — Ricavi'!M9,0)</f>
-        <v>152.340659340659</v>
+        <v>192.252747252747</v>
       </c>
       <c r="N12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!N9&gt;0,MASTER!N9/'A — Ricavi'!N9,0)</f>
-        <v>164.93137254902</v>
+        <v>204.852941176471</v>
       </c>
       <c r="O12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!O9&gt;0,MASTER!O9/'A — Ricavi'!O9,0)</f>
-        <v>170.216216216216</v>
+        <v>209.927927927928</v>
       </c>
       <c r="P12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!P9&gt;0,MASTER!P9/'A — Ricavi'!P9,0)</f>
-        <v>182.595041322314</v>
+        <v>222.462809917355</v>
       </c>
       <c r="Q12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!Q9&gt;0,MASTER!Q9/'A — Ricavi'!Q9,0)</f>
-        <v>184.229007633588</v>
+        <v>224.229007633588</v>
       </c>
       <c r="R12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!R9&gt;0,MASTER!R9/'A — Ricavi'!R9,0)</f>
-        <v>199.093525179856</v>
+        <v>239.035971223022</v>
       </c>
       <c r="S12" s="50" t="n">
         <f aca="false">IF('A — Ricavi'!S9&gt;0,MASTER!S9/'A — Ricavi'!S9,0)</f>
-        <v>203.878378378378</v>
+        <v>243.662162162162</v>
       </c>
       <c r="T12" s="72" t="n">
         <f aca="false">SUM(B12:S12)</f>
-        <v>2514.44832007788</v>
+        <v>3222.1774739774</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6309,79 +6309,79 @@
       </c>
       <c r="B19" s="116" t="n">
         <f aca="false">MASTER!B20</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C19" s="116" t="n">
         <f aca="false">MASTER!C20</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D19" s="116" t="n">
         <f aca="false">MASTER!D20</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E19" s="116" t="n">
         <f aca="false">MASTER!E20</f>
-        <v>-4231</v>
+        <v>-3487</v>
       </c>
       <c r="F19" s="116" t="n">
         <f aca="false">MASTER!F20</f>
-        <v>-4767</v>
+        <v>-3767</v>
       </c>
       <c r="G19" s="116" t="n">
         <f aca="false">MASTER!G20</f>
-        <v>-4489</v>
+        <v>-3209</v>
       </c>
       <c r="H19" s="116" t="n">
         <f aca="false">MASTER!H20</f>
-        <v>-5772</v>
+        <v>-4156</v>
       </c>
       <c r="I19" s="116" t="n">
         <f aca="false">MASTER!I20</f>
-        <v>-4705</v>
+        <v>-2729</v>
       </c>
       <c r="J19" s="116" t="n">
         <f aca="false">MASTER!J20</f>
-        <v>-3510</v>
+        <v>-1174</v>
       </c>
       <c r="K19" s="116" t="n">
         <f aca="false">MASTER!K20</f>
-        <v>-2440</v>
+        <v>312</v>
       </c>
       <c r="L19" s="116" t="n">
         <f aca="false">MASTER!L20</f>
-        <v>-2770</v>
+        <v>422</v>
       </c>
       <c r="M19" s="116" t="n">
         <f aca="false">MASTER!M20</f>
-        <v>-1569</v>
+        <v>2063</v>
       </c>
       <c r="N19" s="116" t="n">
         <f aca="false">MASTER!N20</f>
-        <v>810</v>
+        <v>4882</v>
       </c>
       <c r="O19" s="116" t="n">
         <f aca="false">MASTER!O20</f>
-        <v>9</v>
+        <v>4417</v>
       </c>
       <c r="P19" s="116" t="n">
         <f aca="false">MASTER!P20</f>
-        <v>2668</v>
+        <v>7492</v>
       </c>
       <c r="Q19" s="116" t="n">
         <f aca="false">MASTER!Q20</f>
-        <v>4234</v>
+        <v>9474</v>
       </c>
       <c r="R19" s="116" t="n">
         <f aca="false">MASTER!R20</f>
-        <v>7287</v>
+        <v>12839</v>
       </c>
       <c r="S19" s="116" t="n">
         <f aca="false">MASTER!S20</f>
-        <v>9325</v>
+        <v>15213</v>
       </c>
       <c r="T19" s="72" t="n">
         <f aca="false">SUM(B19:S19)</f>
-        <v>-21608</v>
+        <v>27848</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6390,79 +6390,79 @@
       </c>
       <c r="B20" s="116" t="n">
         <f aca="false">MASTER!B25</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C20" s="116" t="n">
         <f aca="false">MASTER!C25</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D20" s="116" t="n">
         <f aca="false">MASTER!D25</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E20" s="116" t="n">
         <f aca="false">MASTER!E25</f>
-        <v>-4181</v>
+        <v>-3437</v>
       </c>
       <c r="F20" s="116" t="n">
         <f aca="false">MASTER!F25</f>
-        <v>-4717</v>
+        <v>-3717</v>
       </c>
       <c r="G20" s="116" t="n">
         <f aca="false">MASTER!G25</f>
-        <v>-4439</v>
+        <v>-3159</v>
       </c>
       <c r="H20" s="116" t="n">
         <f aca="false">MASTER!H25</f>
-        <v>-5692</v>
+        <v>-4076</v>
       </c>
       <c r="I20" s="116" t="n">
         <f aca="false">MASTER!I25</f>
-        <v>-4625</v>
+        <v>-2649</v>
       </c>
       <c r="J20" s="116" t="n">
         <f aca="false">MASTER!J25</f>
-        <v>-3430</v>
+        <v>-1094</v>
       </c>
       <c r="K20" s="116" t="n">
         <f aca="false">MASTER!K25</f>
-        <v>-2360</v>
+        <v>392</v>
       </c>
       <c r="L20" s="116" t="n">
         <f aca="false">MASTER!L25</f>
-        <v>-2670</v>
+        <v>522</v>
       </c>
       <c r="M20" s="116" t="n">
         <f aca="false">MASTER!M25</f>
-        <v>-1469</v>
+        <v>2163</v>
       </c>
       <c r="N20" s="116" t="n">
         <f aca="false">MASTER!N25</f>
-        <v>930</v>
+        <v>5002</v>
       </c>
       <c r="O20" s="116" t="n">
         <f aca="false">MASTER!O25</f>
-        <v>129</v>
+        <v>4537</v>
       </c>
       <c r="P20" s="116" t="n">
         <f aca="false">MASTER!P25</f>
-        <v>2788</v>
+        <v>7612</v>
       </c>
       <c r="Q20" s="116" t="n">
         <f aca="false">MASTER!Q25</f>
-        <v>4354</v>
+        <v>9594</v>
       </c>
       <c r="R20" s="116" t="n">
         <f aca="false">MASTER!R25</f>
-        <v>7437</v>
+        <v>12989</v>
       </c>
       <c r="S20" s="116" t="n">
         <f aca="false">MASTER!S25</f>
-        <v>9475</v>
+        <v>15363</v>
       </c>
       <c r="T20" s="72" t="n">
         <f aca="false">SUM(B20:S20)</f>
-        <v>-20158</v>
+        <v>29298</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6471,79 +6471,79 @@
       </c>
       <c r="B21" s="118" t="n">
         <f aca="false">MASTER!B30</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C21" s="118" t="n">
         <f aca="false">MASTER!C30</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D21" s="118" t="n">
         <f aca="false">MASTER!D30</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E21" s="118" t="n">
         <f aca="false">MASTER!E30</f>
-        <v>-4181</v>
+        <v>-3437</v>
       </c>
       <c r="F21" s="118" t="n">
         <f aca="false">MASTER!F30</f>
-        <v>-4717</v>
+        <v>-3717</v>
       </c>
       <c r="G21" s="118" t="n">
         <f aca="false">MASTER!G30</f>
-        <v>-4439</v>
+        <v>-3159</v>
       </c>
       <c r="H21" s="118" t="n">
         <f aca="false">MASTER!H30</f>
-        <v>-5692</v>
+        <v>-4076</v>
       </c>
       <c r="I21" s="118" t="n">
         <f aca="false">MASTER!I30</f>
-        <v>-4625</v>
+        <v>-2649</v>
       </c>
       <c r="J21" s="118" t="n">
         <f aca="false">MASTER!J30</f>
-        <v>-3430</v>
+        <v>-1094</v>
       </c>
       <c r="K21" s="118" t="n">
         <f aca="false">MASTER!K30</f>
-        <v>-2360</v>
+        <v>282.632</v>
       </c>
       <c r="L21" s="118" t="n">
         <f aca="false">MASTER!L30</f>
-        <v>-2670</v>
+        <v>376.362</v>
       </c>
       <c r="M21" s="118" t="n">
         <f aca="false">MASTER!M30</f>
-        <v>-1469</v>
+        <v>1559.523</v>
       </c>
       <c r="N21" s="118" t="n">
         <f aca="false">MASTER!N30</f>
-        <v>670.53</v>
+        <v>3606.442</v>
       </c>
       <c r="O21" s="118" t="n">
         <f aca="false">MASTER!O30</f>
-        <v>93.009</v>
+        <v>3271.177</v>
       </c>
       <c r="P21" s="118" t="n">
         <f aca="false">MASTER!P30</f>
-        <v>2010.148</v>
+        <v>5488.252</v>
       </c>
       <c r="Q21" s="118" t="n">
         <f aca="false">MASTER!Q30</f>
-        <v>3139.234</v>
+        <v>6917.274</v>
       </c>
       <c r="R21" s="118" t="n">
         <f aca="false">MASTER!R30</f>
-        <v>5362.077</v>
+        <v>9365.069</v>
       </c>
       <c r="S21" s="118" t="n">
         <f aca="false">MASTER!S30</f>
-        <v>6831.475</v>
+        <v>11076.723</v>
       </c>
       <c r="T21" s="72" t="n">
         <f aca="false">SUM(B21:S21)</f>
-        <v>-27164.527</v>
+        <v>13067.454</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6576,79 +6576,79 @@
       </c>
       <c r="B23" s="119" t="n">
         <f aca="false">IF(MASTER!B9&gt;0,(MASTER!B9-'B1 — Infrastruttura'!B18-'B6 — Costi Variabili'!B16)/MASTER!B9,0)</f>
-        <v>0.0204081632653061</v>
+        <v>0.448275862068966</v>
       </c>
       <c r="C23" s="119" t="n">
         <f aca="false">IF(MASTER!C9&gt;0,(MASTER!C9-'B1 — Infrastruttura'!C18-'B6 — Costi Variabili'!C16)/MASTER!C9,0)</f>
-        <v>0.286118980169972</v>
+        <v>0.601895734597156</v>
       </c>
       <c r="D23" s="119" t="n">
         <f aca="false">IF(MASTER!D9&gt;0,(MASTER!D9-'B1 — Infrastruttura'!D18-'B6 — Costi Variabili'!D16)/MASTER!D9,0)</f>
-        <v>0.670454545454545</v>
+        <v>0.778061224489796</v>
       </c>
       <c r="E23" s="119" t="n">
         <f aca="false">IF(MASTER!E9&gt;0,(MASTER!E9-'B1 — Infrastruttura'!E18-'B6 — Costi Variabili'!E16)/MASTER!E9,0)</f>
-        <v>0.762618690654673</v>
+        <v>0.82695810564663</v>
       </c>
       <c r="F23" s="119" t="n">
         <f aca="false">IF(MASTER!F9&gt;0,(MASTER!F9-'B1 — Infrastruttura'!F18-'B6 — Costi Variabili'!F16)/MASTER!F9,0)</f>
-        <v>0.770777479892761</v>
+        <v>0.828313253012048</v>
       </c>
       <c r="G23" s="119" t="n">
         <f aca="false">IF(MASTER!G9&gt;0,(MASTER!G9-'B1 — Infrastruttura'!G18-'B6 — Costi Variabili'!G16)/MASTER!G9,0)</f>
-        <v>0.790665110851809</v>
+        <v>0.838814016172507</v>
       </c>
       <c r="H23" s="119" t="n">
         <f aca="false">IF(MASTER!H9&gt;0,(MASTER!H9-'B1 — Infrastruttura'!H18-'B6 — Costi Variabili'!H16)/MASTER!H9,0)</f>
-        <v>0.810741249142073</v>
+        <v>0.851826974744761</v>
       </c>
       <c r="I23" s="119" t="n">
         <f aca="false">IF(MASTER!I9&gt;0,(MASTER!I9-'B1 — Infrastruttura'!I18-'B6 — Costi Variabili'!I16)/MASTER!I9,0)</f>
-        <v>0.81443725030996</v>
+        <v>0.854141851651327</v>
       </c>
       <c r="J23" s="119" t="n">
         <f aca="false">IF(MASTER!J9&gt;0,(MASTER!J9-'B1 — Infrastruttura'!J18-'B6 — Costi Variabili'!J16)/MASTER!J9,0)</f>
-        <v>0.816724974607832</v>
+        <v>0.854961150308118</v>
       </c>
       <c r="K23" s="119" t="n">
         <f aca="false">IF(MASTER!K9&gt;0,(MASTER!K9-'B1 — Infrastruttura'!K18-'B6 — Costi Variabili'!K16)/MASTER!K9,0)</f>
-        <v>0.815748642358417</v>
+        <v>0.854562155541947</v>
       </c>
       <c r="L23" s="119" t="n">
         <f aca="false">IF(MASTER!L9&gt;0,(MASTER!L9-'B1 — Infrastruttura'!L18-'B6 — Costi Variabili'!L16)/MASTER!L9,0)</f>
-        <v>0.81836852049618</v>
+        <v>0.856101529450049</v>
       </c>
       <c r="M23" s="119" t="n">
         <f aca="false">IF(MASTER!M9&gt;0,(MASTER!M9-'B1 — Infrastruttura'!M18-'B6 — Costi Variabili'!M16)/MASTER!M9,0)</f>
-        <v>0.813893096732309</v>
+        <v>0.852529294084024</v>
       </c>
       <c r="N23" s="119" t="n">
         <f aca="false">IF(MASTER!N9&gt;0,(MASTER!N9-'B1 — Infrastruttura'!N18-'B6 — Costi Variabili'!N16)/MASTER!N9,0)</f>
-        <v>0.823396540450574</v>
+        <v>0.857812873893276</v>
       </c>
       <c r="O23" s="119" t="n">
         <f aca="false">IF(MASTER!O9&gt;0,(MASTER!O9-'B1 — Infrastruttura'!O18-'B6 — Costi Variabili'!O16)/MASTER!O9,0)</f>
-        <v>0.823859426272891</v>
+        <v>0.857179641232512</v>
       </c>
       <c r="P23" s="119" t="n">
         <f aca="false">IF(MASTER!P9&gt;0,(MASTER!P9-'B1 — Infrastruttura'!P18-'B6 — Costi Variabili'!P16)/MASTER!P9,0)</f>
-        <v>0.832578980718747</v>
+        <v>0.862582658444164</v>
       </c>
       <c r="Q23" s="119" t="n">
         <f aca="false">IF(MASTER!Q9&gt;0,(MASTER!Q9-'B1 — Infrastruttura'!Q18-'B6 — Costi Variabili'!Q16)/MASTER!Q9,0)</f>
-        <v>0.832269826800365</v>
+        <v>0.862191053312453</v>
       </c>
       <c r="R23" s="119" t="n">
         <f aca="false">IF(MASTER!R9&gt;0,(MASTER!R9-'B1 — Infrastruttura'!R18-'B6 — Costi Variabili'!R16)/MASTER!R9,0)</f>
-        <v>0.841728698417287</v>
+        <v>0.868175525191115</v>
       </c>
       <c r="S23" s="119" t="n">
         <f aca="false">IF(MASTER!S9&gt;0,(MASTER!S9-'B1 — Infrastruttura'!S18-'B6 — Costi Variabili'!S16)/MASTER!S9,0)</f>
-        <v>0.844004772320541</v>
+        <v>0.869474793411347</v>
       </c>
       <c r="T23" s="120" t="n">
         <f aca="false">AVERAGE(B23:S23)</f>
-        <v>0.732710830495347</v>
+        <v>0.812436538736233</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6657,79 +6657,79 @@
       </c>
       <c r="B24" s="121" t="n">
         <f aca="false">IF(MASTER!B9&gt;0,'B3 — Marketing'!B28/MASTER!B9,0)</f>
-        <v>0.86734693877551</v>
+        <v>0.488505747126437</v>
       </c>
       <c r="C24" s="121" t="n">
         <f aca="false">IF(MASTER!C9&gt;0,'B3 — Marketing'!C28/MASTER!C9,0)</f>
-        <v>0.509915014164306</v>
+        <v>0.28436018957346</v>
       </c>
       <c r="D24" s="121" t="n">
         <f aca="false">IF(MASTER!D9&gt;0,'B3 — Marketing'!D28/MASTER!D9,0)</f>
-        <v>0.208333333333333</v>
+        <v>0.14030612244898</v>
       </c>
       <c r="E24" s="121" t="n">
         <f aca="false">IF(MASTER!E9&gt;0,'B3 — Marketing'!E28/MASTER!E9,0)</f>
-        <v>0.114942528735632</v>
+        <v>0.0837887067395264</v>
       </c>
       <c r="F24" s="121" t="n">
         <f aca="false">IF(MASTER!F9&gt;0,'B3 — Marketing'!F28/MASTER!F9,0)</f>
-        <v>0.103887399463807</v>
+        <v>0.0778112449799197</v>
       </c>
       <c r="G24" s="121" t="n">
         <f aca="false">IF(MASTER!G9&gt;0,'B3 — Marketing'!G28/MASTER!G9,0)</f>
-        <v>0.0910151691948658</v>
+        <v>0.0700808625336927</v>
       </c>
       <c r="H24" s="121" t="n">
         <f aca="false">IF(MASTER!H9&gt;0,'B3 — Marketing'!H28/MASTER!H9,0)</f>
-        <v>0.0806451612903226</v>
+        <v>0.0631380977968834</v>
       </c>
       <c r="I24" s="121" t="n">
         <f aca="false">IF(MASTER!I9&gt;0,'B3 — Marketing'!I28/MASTER!I9,0)</f>
-        <v>0.0757680121228819</v>
+        <v>0.0595560368164591</v>
       </c>
       <c r="J24" s="121" t="n">
         <f aca="false">IF(MASTER!J9&gt;0,'B3 — Marketing'!J28/MASTER!J9,0)</f>
-        <v>0.0722266109919874</v>
+        <v>0.0571581673662588</v>
       </c>
       <c r="K24" s="121" t="n">
         <f aca="false">IF(MASTER!K9&gt;0,'B3 — Marketing'!K28/MASTER!K9,0)</f>
-        <v>0.0678820791311094</v>
+        <v>0.0535823637477036</v>
       </c>
       <c r="L24" s="121" t="n">
         <f aca="false">IF(MASTER!L9&gt;0,'B3 — Marketing'!L28/MASTER!L9,0)</f>
-        <v>0.0648977244721926</v>
+        <v>0.0514155548324113</v>
       </c>
       <c r="M24" s="121" t="n">
         <f aca="false">IF(MASTER!M9&gt;0,'B3 — Marketing'!M28/MASTER!M9,0)</f>
-        <v>0.0627569790088725</v>
+        <v>0.0497284938553873</v>
       </c>
       <c r="N24" s="121" t="n">
         <f aca="false">IF(MASTER!N9&gt;0,'B3 — Marketing'!N28/MASTER!N9,0)</f>
-        <v>0.0570647328062771</v>
+        <v>0.0459440057430007</v>
       </c>
       <c r="O24" s="121" t="n">
         <f aca="false">IF(MASTER!O9&gt;0,'B3 — Marketing'!O28/MASTER!O9,0)</f>
-        <v>0.0550439292897216</v>
+        <v>0.0446313621148399</v>
       </c>
       <c r="P24" s="121" t="n">
         <f aca="false">IF(MASTER!P9&gt;0,'B3 — Marketing'!P28/MASTER!P9,0)</f>
-        <v>0.0511451072689418</v>
+        <v>0.0419793446764247</v>
       </c>
       <c r="Q24" s="121" t="n">
         <f aca="false">IF(MASTER!Q9&gt;0,'B3 — Marketing'!Q28/MASTER!Q9,0)</f>
-        <v>0.0501367365542388</v>
+        <v>0.041192891672908</v>
       </c>
       <c r="R24" s="121" t="n">
         <f aca="false">IF(MASTER!R9&gt;0,'B3 — Marketing'!R28/MASTER!R9,0)</f>
-        <v>0.0466141504661415</v>
+        <v>0.0388250165533016</v>
       </c>
       <c r="S24" s="121" t="n">
         <f aca="false">IF(MASTER!S9&gt;0,'B3 — Marketing'!S28/MASTER!S9,0)</f>
-        <v>0.0454033273679327</v>
+        <v>0.0379901281126948</v>
       </c>
       <c r="T24" s="122" t="n">
         <f aca="false">AVERAGE(B24:S24)</f>
-        <v>0.145834718579893</v>
+        <v>0.0961107964827938</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6819,79 +6819,79 @@
       </c>
       <c r="B26" s="119" t="n">
         <f aca="false">IF(MASTER!B9&gt;0,MASTER!B20/MASTER!B9,0)</f>
-        <v>-21.0867346938776</v>
+        <v>-11.4396551724138</v>
       </c>
       <c r="C26" s="119" t="n">
         <f aca="false">IF(MASTER!C9&gt;0,MASTER!C20/MASTER!C9,0)</f>
-        <v>-11.4759206798867</v>
+        <v>-5.95734597156398</v>
       </c>
       <c r="D26" s="119" t="n">
         <f aca="false">IF(MASTER!D9&gt;0,MASTER!D20/MASTER!D9,0)</f>
-        <v>-3.31818181818182</v>
+        <v>-1.90816326530612</v>
       </c>
       <c r="E26" s="119" t="n">
         <f aca="false">IF(MASTER!E9&gt;0,MASTER!E20/MASTER!E9,0)</f>
-        <v>-2.11444277861069</v>
+        <v>-1.27030965391621</v>
       </c>
       <c r="F26" s="119" t="n">
         <f aca="false">IF(MASTER!F9&gt;0,MASTER!F20/MASTER!F9,0)</f>
-        <v>-1.59752010723861</v>
+        <v>-0.945532128514056</v>
       </c>
       <c r="G26" s="119" t="n">
         <f aca="false">IF(MASTER!G9&gt;0,MASTER!G20/MASTER!G9,0)</f>
-        <v>-1.04760793465578</v>
+        <v>-0.576639712488769</v>
       </c>
       <c r="H26" s="119" t="n">
         <f aca="false">IF(MASTER!H9&gt;0,MASTER!H20/MASTER!H9,0)</f>
-        <v>-0.990391214824983</v>
+        <v>-0.558301988178399</v>
       </c>
       <c r="I26" s="119" t="n">
         <f aca="false">IF(MASTER!I9&gt;0,MASTER!I20/MASTER!I9,0)</f>
-        <v>-0.648160903705745</v>
+        <v>-0.29550622631294</v>
       </c>
       <c r="J26" s="119" t="n">
         <f aca="false">IF(MASTER!J9&gt;0,MASTER!J20/MASTER!J9,0)</f>
-        <v>-0.396117819659181</v>
+        <v>-0.104849513262481</v>
       </c>
       <c r="K26" s="119" t="n">
         <f aca="false">IF(MASTER!K9&gt;0,MASTER!K20/MASTER!K9,0)</f>
-        <v>-0.236617532971296</v>
+        <v>0.0238824249846908</v>
       </c>
       <c r="L26" s="119" t="n">
         <f aca="false">IF(MASTER!L9&gt;0,MASTER!L20/MASTER!L9,0)</f>
-        <v>-0.22755278074427</v>
+        <v>0.0274650178978197</v>
       </c>
       <c r="M26" s="119" t="n">
         <f aca="false">IF(MASTER!M9&gt;0,MASTER!M20/MASTER!M9,0)</f>
-        <v>-0.113178965591863</v>
+        <v>0.117919405544441</v>
       </c>
       <c r="N26" s="119" t="n">
         <f aca="false">IF(MASTER!N9&gt;0,MASTER!N20/MASTER!N9,0)</f>
-        <v>0.0481483683052963</v>
+        <v>0.233644412538885</v>
       </c>
       <c r="O26" s="119" t="n">
         <f aca="false">IF(MASTER!O9&gt;0,MASTER!O20/MASTER!O9,0)</f>
-        <v>0.000476341695776437</v>
+        <v>0.189554544674277</v>
       </c>
       <c r="P26" s="119" t="n">
         <f aca="false">IF(MASTER!P9&gt;0,MASTER!P20/MASTER!P9,0)</f>
-        <v>0.120756766542953</v>
+        <v>0.27832677019095</v>
       </c>
       <c r="Q26" s="119" t="n">
         <f aca="false">IF(MASTER!Q9&gt;0,MASTER!Q20/MASTER!Q9,0)</f>
-        <v>0.17543714262037</v>
+        <v>0.322530128685232</v>
       </c>
       <c r="R26" s="119" t="n">
         <f aca="false">IF(MASTER!R9&gt;0,MASTER!R20/MASTER!R9,0)</f>
-        <v>0.263315747633157</v>
+        <v>0.38641425389755</v>
       </c>
       <c r="S26" s="119" t="n">
         <f aca="false">IF(MASTER!S9&gt;0,MASTER!S20/MASTER!S9,0)</f>
-        <v>0.309040896135746</v>
+        <v>0.421856802174034</v>
       </c>
       <c r="T26" s="120" t="n">
         <f aca="false">AVERAGE(B26:S26)</f>
-        <v>-2.35195844261195</v>
+        <v>-1.16970610396494</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8897,79 +8897,79 @@
       </c>
       <c r="B11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!B9&gt;0,MASTER!B9/'A — Ricavi'!B9,0)</f>
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="C11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!C9&gt;0,MASTER!C9/'A — Ricavi'!C9,0)</f>
-        <v>50.4285714285714</v>
+        <v>90.4285714285714</v>
       </c>
       <c r="D11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!D9&gt;0,MASTER!D9/'A — Ricavi'!D9,0)</f>
-        <v>81.2307692307692</v>
+        <v>120.615384615385</v>
       </c>
       <c r="E11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!E9&gt;0,MASTER!E9/'A — Ricavi'!E9,0)</f>
-        <v>105.315789473684</v>
+        <v>144.473684210526</v>
       </c>
       <c r="F11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!F9&gt;0,MASTER!F9/'A — Ricavi'!F9,0)</f>
-        <v>114.769230769231</v>
+        <v>153.230769230769</v>
       </c>
       <c r="G11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!G9&gt;0,MASTER!G9/'A — Ricavi'!G9,0)</f>
-        <v>126.029411764706</v>
+        <v>163.676470588235</v>
       </c>
       <c r="H11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!H9&gt;0,MASTER!H9/'A — Ricavi'!H9,0)</f>
-        <v>138.761904761905</v>
+        <v>177.238095238095</v>
       </c>
       <c r="I11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!I9&gt;0,MASTER!I9/'A — Ricavi'!I9,0)</f>
-        <v>142.333333333333</v>
+        <v>181.078431372549</v>
       </c>
       <c r="J11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!J9&gt;0,MASTER!J9/'A — Ricavi'!J9,0)</f>
-        <v>147.683333333333</v>
+        <v>186.616666666667</v>
       </c>
       <c r="K11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!K9&gt;0,MASTER!K9/'A — Ricavi'!K9,0)</f>
-        <v>149.449275362319</v>
+        <v>189.333333333333</v>
       </c>
       <c r="L11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!L9&gt;0,MASTER!L9/'A — Ricavi'!L9,0)</f>
-        <v>152.1625</v>
+        <v>192.0625</v>
       </c>
       <c r="M11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!M9&gt;0,MASTER!M9/'A — Ricavi'!M9,0)</f>
-        <v>152.340659340659</v>
+        <v>192.252747252747</v>
       </c>
       <c r="N11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!N9&gt;0,MASTER!N9/'A — Ricavi'!N9,0)</f>
-        <v>164.93137254902</v>
+        <v>204.852941176471</v>
       </c>
       <c r="O11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!O9&gt;0,MASTER!O9/'A — Ricavi'!O9,0)</f>
-        <v>170.216216216216</v>
+        <v>209.927927927928</v>
       </c>
       <c r="P11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!P9&gt;0,MASTER!P9/'A — Ricavi'!P9,0)</f>
-        <v>182.595041322314</v>
+        <v>222.462809917355</v>
       </c>
       <c r="Q11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!Q9&gt;0,MASTER!Q9/'A — Ricavi'!Q9,0)</f>
-        <v>184.229007633588</v>
+        <v>224.229007633588</v>
       </c>
       <c r="R11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!R9&gt;0,MASTER!R9/'A — Ricavi'!R9,0)</f>
-        <v>199.093525179856</v>
+        <v>239.035971223022</v>
       </c>
       <c r="S11" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!S9&gt;0,MASTER!S9/'A — Ricavi'!S9,0)</f>
-        <v>203.878378378378</v>
+        <v>243.662162162162</v>
       </c>
       <c r="T11" s="72" t="n">
         <f aca="false">SUM(B11:S11)</f>
-        <v>2514.44832007788</v>
+        <v>3222.1774739774</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9140,79 +9140,79 @@
       </c>
       <c r="B14" s="104" t="n">
         <f aca="false">B11*B13</f>
-        <v>980</v>
+        <v>1740</v>
       </c>
       <c r="C14" s="104" t="n">
         <f aca="false">C11*C13</f>
-        <v>1008.57142857143</v>
+        <v>1808.57142857143</v>
       </c>
       <c r="D14" s="104" t="n">
         <f aca="false">D11*D13</f>
-        <v>2030.76923076923</v>
+        <v>3015.38461538462</v>
       </c>
       <c r="E14" s="104" t="n">
         <f aca="false">E11*E13</f>
-        <v>2632.89473684211</v>
+        <v>3611.84210526316</v>
       </c>
       <c r="F14" s="104" t="n">
         <f aca="false">F11*F13</f>
-        <v>2869.23076923077</v>
+        <v>3830.76923076923</v>
       </c>
       <c r="G14" s="104" t="n">
         <f aca="false">G11*G13</f>
-        <v>4200.98039215686</v>
+        <v>5455.88235294118</v>
       </c>
       <c r="H14" s="104" t="n">
         <f aca="false">H11*H13</f>
-        <v>4625.39682539683</v>
+        <v>5907.93650793651</v>
       </c>
       <c r="I14" s="104" t="n">
         <f aca="false">I11*I13</f>
-        <v>4744.44444444445</v>
+        <v>6035.9477124183</v>
       </c>
       <c r="J14" s="104" t="n">
         <f aca="false">J11*J13</f>
-        <v>4922.77777777778</v>
+        <v>6220.55555555556</v>
       </c>
       <c r="K14" s="104" t="n">
         <f aca="false">K11*K13</f>
-        <v>4981.6425120773</v>
+        <v>6311.11111111111</v>
       </c>
       <c r="L14" s="104" t="n">
         <f aca="false">L11*L13</f>
-        <v>7608.125</v>
+        <v>9603.125</v>
       </c>
       <c r="M14" s="104" t="n">
         <f aca="false">M11*M13</f>
-        <v>7617.03296703297</v>
+        <v>9612.63736263736</v>
       </c>
       <c r="N14" s="104" t="n">
         <f aca="false">N11*N13</f>
-        <v>8246.56862745098</v>
+        <v>10242.6470588235</v>
       </c>
       <c r="O14" s="104" t="n">
         <f aca="false">O11*O13</f>
-        <v>8510.81081081081</v>
+        <v>10496.3963963964</v>
       </c>
       <c r="P14" s="104" t="n">
         <f aca="false">P11*P13</f>
-        <v>9129.7520661157</v>
+        <v>11123.1404958678</v>
       </c>
       <c r="Q14" s="104" t="n">
         <f aca="false">Q11*Q13</f>
-        <v>9211.45038167939</v>
+        <v>11211.4503816794</v>
       </c>
       <c r="R14" s="104" t="n">
         <f aca="false">R11*R13</f>
-        <v>9954.67625899281</v>
+        <v>11951.7985611511</v>
       </c>
       <c r="S14" s="104" t="n">
         <f aca="false">S11*S13</f>
-        <v>10193.9189189189</v>
+        <v>12183.1081081081</v>
       </c>
       <c r="T14" s="133" t="n">
         <f aca="false">AVERAGE(B14:S14)</f>
-        <v>5748.2801749038</v>
+        <v>7242.35022136749</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9267,79 +9267,79 @@
       </c>
       <c r="B17" s="138" t="n">
         <f aca="false">IF(B7&gt;0,B14/B7,0)</f>
-        <v>23.0588235294118</v>
+        <v>40.9411764705882</v>
       </c>
       <c r="C17" s="138" t="n">
         <f aca="false">IF(C7&gt;0,C14/C7,0)</f>
-        <v>16.8095238095238</v>
+        <v>30.1428571428571</v>
       </c>
       <c r="D17" s="138" t="n">
         <f aca="false">IF(D7&gt;0,D14/D7,0)</f>
-        <v>55.3846153846154</v>
+        <v>82.2377622377622</v>
       </c>
       <c r="E17" s="138" t="n">
         <f aca="false">IF(E7&gt;0,E14/E7,0)</f>
-        <v>19.0329740012682</v>
+        <v>26.1097019657578</v>
       </c>
       <c r="F17" s="138" t="n">
         <f aca="false">IF(F7&gt;0,F14/F7,0)</f>
-        <v>9.51877506379876</v>
+        <v>12.70871308786</v>
       </c>
       <c r="G17" s="138" t="n">
         <f aca="false">IF(G7&gt;0,G14/G7,0)</f>
-        <v>15.3460470946369</v>
+        <v>19.9301638463605</v>
       </c>
       <c r="H17" s="138" t="n">
         <f aca="false">IF(H7&gt;0,H14/H7,0)</f>
-        <v>13.8588668925748</v>
+        <v>17.7016824207836</v>
       </c>
       <c r="I17" s="138" t="n">
         <f aca="false">IF(I7&gt;0,I14/I7,0)</f>
-        <v>15.5272727272727</v>
+        <v>19.7540106951872</v>
       </c>
       <c r="J17" s="138" t="n">
         <f aca="false">IF(J7&gt;0,J14/J7,0)</f>
-        <v>15.6003521126761</v>
+        <v>19.7130281690141</v>
       </c>
       <c r="K17" s="138" t="n">
         <f aca="false">IF(K7&gt;0,K14/K7,0)</f>
-        <v>15.4602698650675</v>
+        <v>19.5862068965517</v>
       </c>
       <c r="L17" s="138" t="n">
         <f aca="false">IF(L7&gt;0,L14/L7,0)</f>
-        <v>27.0839401294498</v>
+        <v>34.1858818770227</v>
       </c>
       <c r="M17" s="138" t="n">
         <f aca="false">IF(M7&gt;0,M14/M7,0)</f>
-        <v>26.431344680556</v>
+        <v>33.3561548861233</v>
       </c>
       <c r="N17" s="138" t="n">
         <f aca="false">IF(N7&gt;0,N14/N7,0)</f>
-        <v>27.8258450619512</v>
+        <v>34.5610790328401</v>
       </c>
       <c r="O17" s="138" t="n">
         <f aca="false">IF(O7&gt;0,O14/O7,0)</f>
-        <v>18.9597270537865</v>
+        <v>23.3830612791009</v>
       </c>
       <c r="P17" s="138" t="n">
         <f aca="false">IF(P7&gt;0,P14/P7,0)</f>
-        <v>22.1059372060913</v>
+        <v>26.9325435735297</v>
       </c>
       <c r="Q17" s="138" t="n">
         <f aca="false">IF(Q7&gt;0,Q14/Q7,0)</f>
-        <v>21.8799296476945</v>
+        <v>26.6305234719225</v>
       </c>
       <c r="R17" s="138" t="n">
         <f aca="false">IF(R7&gt;0,R14/R7,0)</f>
-        <v>18.5634988512686</v>
+        <v>22.2877362445708</v>
       </c>
       <c r="S17" s="138" t="n">
         <f aca="false">IF(S7&gt;0,S14/S7,0)</f>
-        <v>20.9943410229451</v>
+        <v>25.0910693301998</v>
       </c>
       <c r="T17" s="139" t="n">
         <f aca="false">AVERAGE(B17:S17)</f>
-        <v>21.3023380074772</v>
+        <v>28.6251862571129</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9418,79 +9418,79 @@
       </c>
       <c r="B21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!B9&gt;0,B11-('B1 — Infrastruttura'!B18+'B6 — Costi Variabili'!B16)/'A — Ricavi'!B9,0)</f>
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="C21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!C9&gt;0,C11-('B1 — Infrastruttura'!C18+'B6 — Costi Variabili'!C16)/'A — Ricavi'!C9,0)</f>
-        <v>14.4285714285714</v>
+        <v>54.4285714285714</v>
       </c>
       <c r="D21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!D9&gt;0,D11-('B1 — Infrastruttura'!D18+'B6 — Costi Variabili'!D16)/'A — Ricavi'!D9,0)</f>
-        <v>54.4615384615385</v>
+        <v>93.8461538461538</v>
       </c>
       <c r="E21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!E9&gt;0,E11-('B1 — Infrastruttura'!E18+'B6 — Costi Variabili'!E16)/'A — Ricavi'!E9,0)</f>
-        <v>80.3157894736842</v>
+        <v>119.473684210526</v>
       </c>
       <c r="F21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!F9&gt;0,F11-('B1 — Infrastruttura'!F18+'B6 — Costi Variabili'!F16)/'A — Ricavi'!F9,0)</f>
-        <v>88.4615384615385</v>
+        <v>126.923076923077</v>
       </c>
       <c r="G21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!G9&gt;0,G11-('B1 — Infrastruttura'!G18+'B6 — Costi Variabili'!G16)/'A — Ricavi'!G9,0)</f>
-        <v>99.6470588235294</v>
+        <v>137.294117647059</v>
       </c>
       <c r="H21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!H9&gt;0,H11-('B1 — Infrastruttura'!H18+'B6 — Costi Variabili'!H16)/'A — Ricavi'!H9,0)</f>
-        <v>112.5</v>
+        <v>150.97619047619</v>
       </c>
       <c r="I21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!I9&gt;0,I11-('B1 — Infrastruttura'!I18+'B6 — Costi Variabili'!I16)/'A — Ricavi'!I9,0)</f>
-        <v>115.921568627451</v>
+        <v>154.666666666667</v>
       </c>
       <c r="J21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!J9&gt;0,J11-('B1 — Infrastruttura'!J18+'B6 — Costi Variabili'!J16)/'A — Ricavi'!J9,0)</f>
-        <v>120.616666666667</v>
+        <v>159.55</v>
       </c>
       <c r="K21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!K9&gt;0,K11-('B1 — Infrastruttura'!K18+'B6 — Costi Variabili'!K16)/'A — Ricavi'!K9,0)</f>
-        <v>121.913043478261</v>
+        <v>161.797101449275</v>
       </c>
       <c r="L21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!L9&gt;0,L11-('B1 — Infrastruttura'!L18+'B6 — Costi Variabili'!L16)/'A — Ricavi'!L9,0)</f>
-        <v>124.525</v>
+        <v>164.425</v>
       </c>
       <c r="M21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!M9&gt;0,M11-('B1 — Infrastruttura'!M18+'B6 — Costi Variabili'!M16)/'A — Ricavi'!M9,0)</f>
-        <v>123.989010989011</v>
+        <v>163.901098901099</v>
       </c>
       <c r="N21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!N9&gt;0,N11-('B1 — Infrastruttura'!N18+'B6 — Costi Variabili'!N16)/'A — Ricavi'!N9,0)</f>
-        <v>135.803921568627</v>
+        <v>175.725490196078</v>
       </c>
       <c r="O21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!O9&gt;0,O11-('B1 — Infrastruttura'!O18+'B6 — Costi Variabili'!O16)/'A — Ricavi'!O9,0)</f>
-        <v>140.234234234234</v>
+        <v>179.945945945946</v>
       </c>
       <c r="P21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!P9&gt;0,P11-('B1 — Infrastruttura'!P18+'B6 — Costi Variabili'!P16)/'A — Ricavi'!P9,0)</f>
-        <v>152.02479338843</v>
+        <v>191.892561983471</v>
       </c>
       <c r="Q21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!Q9&gt;0,Q11-('B1 — Infrastruttura'!Q18+'B6 — Costi Variabili'!Q16)/'A — Ricavi'!Q9,0)</f>
-        <v>153.328244274809</v>
+        <v>193.328244274809</v>
       </c>
       <c r="R21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!R9&gt;0,R11-('B1 — Infrastruttura'!R18+'B6 — Costi Variabili'!R16)/'A — Ricavi'!R9,0)</f>
-        <v>167.58273381295</v>
+        <v>207.525179856115</v>
       </c>
       <c r="S21" s="91" t="n">
         <f aca="false">IF('A — Ricavi'!S9&gt;0,S11-('B1 — Infrastruttura'!S18+'B6 — Costi Variabili'!S16)/'A — Ricavi'!S9,0)</f>
-        <v>172.074324324324</v>
+        <v>211.858108108108</v>
       </c>
       <c r="T21" s="72" t="n">
         <f aca="false">SUM(B21:S21)</f>
-        <v>1978.82803801363</v>
+        <v>2686.55719191315</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9499,79 +9499,79 @@
       </c>
       <c r="B22" s="140" t="n">
         <f aca="false">IF(B21&gt;0,B7/B21,0)</f>
-        <v>42.5</v>
+        <v>1.08974358974359</v>
       </c>
       <c r="C22" s="140" t="n">
         <f aca="false">IF(C21&gt;0,C7/C21,0)</f>
-        <v>4.15841584158416</v>
+        <v>1.10236220472441</v>
       </c>
       <c r="D22" s="140" t="n">
         <f aca="false">IF(D21&gt;0,D7/D21,0)</f>
-        <v>0.673258003766478</v>
+        <v>0.390710382513661</v>
       </c>
       <c r="E22" s="140" t="n">
         <f aca="false">IF(E21&gt;0,E7/E21,0)</f>
-        <v>1.72236784622106</v>
+        <v>1.15785609397944</v>
       </c>
       <c r="F22" s="140" t="n">
         <f aca="false">IF(F21&gt;0,F7/F21,0)</f>
-        <v>3.40745341614907</v>
+        <v>2.37489177489178</v>
       </c>
       <c r="G22" s="140" t="n">
         <f aca="false">IF(G21&gt;0,G7/G21,0)</f>
-        <v>2.74719598583235</v>
+        <v>1.99389460154242</v>
       </c>
       <c r="H22" s="140" t="n">
         <f aca="false">IF(H21&gt;0,H7/H21,0)</f>
-        <v>2.96666666666667</v>
+        <v>2.21061346790727</v>
       </c>
       <c r="I22" s="140" t="n">
         <f aca="false">IF(I21&gt;0,I7/I21,0)</f>
-        <v>2.63588182228236</v>
+        <v>1.97557471264368</v>
       </c>
       <c r="J22" s="140" t="n">
         <f aca="false">IF(J21&gt;0,J7/J21,0)</f>
-        <v>2.61618534383492</v>
+        <v>1.97778474180856</v>
       </c>
       <c r="K22" s="140" t="n">
         <f aca="false">IF(K21&gt;0,K7/K21,0)</f>
-        <v>2.64304961166587</v>
+        <v>1.99152036307178</v>
       </c>
       <c r="L22" s="140" t="n">
         <f aca="false">IF(L21&gt;0,L7/L21,0)</f>
-        <v>2.25584493803727</v>
+        <v>1.70843296888606</v>
       </c>
       <c r="M22" s="140" t="n">
         <f aca="false">IF(M21&gt;0,M7/M21,0)</f>
-        <v>2.32425289856824</v>
+        <v>1.75826654070033</v>
       </c>
       <c r="N22" s="140" t="n">
         <f aca="false">IF(N21&gt;0,N7/N21,0)</f>
-        <v>2.18229070957919</v>
+        <v>1.68651477957436</v>
       </c>
       <c r="O22" s="140" t="n">
         <f aca="false">IF(O21&gt;0,O7/O21,0)</f>
-        <v>3.20099361857039</v>
+        <v>2.49457628250058</v>
       </c>
       <c r="P22" s="140" t="n">
         <f aca="false">IF(P21&gt;0,P7/P21,0)</f>
-        <v>2.71666213645012</v>
+        <v>2.15224600542659</v>
       </c>
       <c r="Q22" s="140" t="n">
         <f aca="false">IF(Q21&gt;0,Q7/Q21,0)</f>
-        <v>2.74574330379369</v>
+        <v>2.1776435283898</v>
       </c>
       <c r="R22" s="140" t="n">
         <f aca="false">IF(R21&gt;0,R7/R21,0)</f>
-        <v>3.19991199450502</v>
+        <v>2.58402378146017</v>
       </c>
       <c r="S22" s="140" t="n">
         <f aca="false">IF(S21&gt;0,S7/S21,0)</f>
-        <v>2.82177807445801</v>
+        <v>2.29189035950318</v>
       </c>
       <c r="T22" s="141" t="n">
         <f aca="false">AVERAGE(B22:S22)</f>
-        <v>4.86210845622027</v>
+        <v>1.83991923218154</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9731,79 +9731,79 @@
       </c>
       <c r="B27" s="119" t="n">
         <f aca="false">IF(MASTER!B9&gt;0,MASTER!B20/MASTER!B9,0)</f>
-        <v>-21.0867346938776</v>
+        <v>-11.4396551724138</v>
       </c>
       <c r="C27" s="119" t="n">
         <f aca="false">IF(MASTER!C9&gt;0,MASTER!C20/MASTER!C9,0)</f>
-        <v>-11.4759206798867</v>
+        <v>-5.95734597156398</v>
       </c>
       <c r="D27" s="119" t="n">
         <f aca="false">IF(MASTER!D9&gt;0,MASTER!D20/MASTER!D9,0)</f>
-        <v>-3.31818181818182</v>
+        <v>-1.90816326530612</v>
       </c>
       <c r="E27" s="119" t="n">
         <f aca="false">IF(MASTER!E9&gt;0,MASTER!E20/MASTER!E9,0)</f>
-        <v>-2.11444277861069</v>
+        <v>-1.27030965391621</v>
       </c>
       <c r="F27" s="119" t="n">
         <f aca="false">IF(MASTER!F9&gt;0,MASTER!F20/MASTER!F9,0)</f>
-        <v>-1.59752010723861</v>
+        <v>-0.945532128514056</v>
       </c>
       <c r="G27" s="119" t="n">
         <f aca="false">IF(MASTER!G9&gt;0,MASTER!G20/MASTER!G9,0)</f>
-        <v>-1.04760793465578</v>
+        <v>-0.576639712488769</v>
       </c>
       <c r="H27" s="119" t="n">
         <f aca="false">IF(MASTER!H9&gt;0,MASTER!H20/MASTER!H9,0)</f>
-        <v>-0.990391214824983</v>
+        <v>-0.558301988178399</v>
       </c>
       <c r="I27" s="119" t="n">
         <f aca="false">IF(MASTER!I9&gt;0,MASTER!I20/MASTER!I9,0)</f>
-        <v>-0.648160903705745</v>
+        <v>-0.29550622631294</v>
       </c>
       <c r="J27" s="119" t="n">
         <f aca="false">IF(MASTER!J9&gt;0,MASTER!J20/MASTER!J9,0)</f>
-        <v>-0.396117819659181</v>
+        <v>-0.104849513262481</v>
       </c>
       <c r="K27" s="119" t="n">
         <f aca="false">IF(MASTER!K9&gt;0,MASTER!K20/MASTER!K9,0)</f>
-        <v>-0.236617532971296</v>
+        <v>0.0238824249846908</v>
       </c>
       <c r="L27" s="119" t="n">
         <f aca="false">IF(MASTER!L9&gt;0,MASTER!L20/MASTER!L9,0)</f>
-        <v>-0.22755278074427</v>
+        <v>0.0274650178978197</v>
       </c>
       <c r="M27" s="119" t="n">
         <f aca="false">IF(MASTER!M9&gt;0,MASTER!M20/MASTER!M9,0)</f>
-        <v>-0.113178965591863</v>
+        <v>0.117919405544441</v>
       </c>
       <c r="N27" s="119" t="n">
         <f aca="false">IF(MASTER!N9&gt;0,MASTER!N20/MASTER!N9,0)</f>
-        <v>0.0481483683052963</v>
+        <v>0.233644412538885</v>
       </c>
       <c r="O27" s="119" t="n">
         <f aca="false">IF(MASTER!O9&gt;0,MASTER!O20/MASTER!O9,0)</f>
-        <v>0.000476341695776437</v>
+        <v>0.189554544674277</v>
       </c>
       <c r="P27" s="119" t="n">
         <f aca="false">IF(MASTER!P9&gt;0,MASTER!P20/MASTER!P9,0)</f>
-        <v>0.120756766542953</v>
+        <v>0.27832677019095</v>
       </c>
       <c r="Q27" s="119" t="n">
         <f aca="false">IF(MASTER!Q9&gt;0,MASTER!Q20/MASTER!Q9,0)</f>
-        <v>0.17543714262037</v>
+        <v>0.322530128685232</v>
       </c>
       <c r="R27" s="119" t="n">
         <f aca="false">IF(MASTER!R9&gt;0,MASTER!R20/MASTER!R9,0)</f>
-        <v>0.263315747633157</v>
+        <v>0.38641425389755</v>
       </c>
       <c r="S27" s="119" t="n">
         <f aca="false">IF(MASTER!S9&gt;0,MASTER!S20/MASTER!S9,0)</f>
-        <v>0.309040896135746</v>
+        <v>0.421856802174034</v>
       </c>
       <c r="T27" s="120" t="n">
         <f aca="false">AVERAGE(B27:S27)</f>
-        <v>-2.35195844261195</v>
+        <v>-1.16970610396494</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9812,79 +9812,79 @@
       </c>
       <c r="B28" s="142" t="n">
         <f aca="false">B26+B27</f>
-        <v>-21.0867346938776</v>
+        <v>-11.4396551724138</v>
       </c>
       <c r="C28" s="142" t="n">
         <f aca="false">C26+C27</f>
-        <v>-10.731022720703</v>
+        <v>-5.21244801238031</v>
       </c>
       <c r="D28" s="142" t="n">
         <f aca="false">D26+D27</f>
-        <v>-2.21053309296935</v>
+        <v>-0.800514540093658</v>
       </c>
       <c r="E28" s="142" t="n">
         <f aca="false">E26+E27</f>
-        <v>-1.56535602061983</v>
+        <v>-0.721222895925344</v>
       </c>
       <c r="F28" s="142" t="n">
         <f aca="false">F26+F27</f>
-        <v>-1.22853949435555</v>
+        <v>-0.576551515631004</v>
       </c>
       <c r="G28" s="142" t="n">
         <f aca="false">G26+G27</f>
-        <v>-0.746013794199076</v>
+        <v>-0.275045572032069</v>
       </c>
       <c r="H28" s="142" t="n">
         <f aca="false">H26+H27</f>
-        <v>-0.74109853956563</v>
+        <v>-0.309009312919046</v>
       </c>
       <c r="I28" s="142" t="n">
         <f aca="false">I26+I27</f>
-        <v>-0.420618949115419</v>
+        <v>-0.0679642717226141</v>
       </c>
       <c r="J28" s="142" t="n">
         <f aca="false">J26+J27</f>
-        <v>-0.21268936069441</v>
+        <v>0.0785789457022897</v>
       </c>
       <c r="K28" s="142" t="n">
         <f aca="false">K26+K27</f>
-        <v>-0.0774094145217864</v>
+        <v>0.1830905434342</v>
       </c>
       <c r="L28" s="142" t="n">
         <f aca="false">L26+L27</f>
-        <v>-0.0601306844269897</v>
+        <v>0.1948871142151</v>
       </c>
       <c r="M28" s="142" t="n">
         <f aca="false">M26+M27</f>
-        <v>0.0328152429023453</v>
+        <v>0.26391361403865</v>
       </c>
       <c r="N28" s="142" t="n">
         <f aca="false">N26+N27</f>
-        <v>0.177737551872639</v>
+        <v>0.363233596106228</v>
       </c>
       <c r="O28" s="142" t="n">
         <f aca="false">O26+O27</f>
-        <v>0.0998242859087813</v>
+        <v>0.288902488887282</v>
       </c>
       <c r="P28" s="142" t="n">
         <f aca="false">P26+P27</f>
-        <v>0.218639119484129</v>
+        <v>0.376209123132127</v>
       </c>
       <c r="Q28" s="142" t="n">
         <f aca="false">Q26+Q27</f>
-        <v>0.263587736144286</v>
+        <v>0.410680722209148</v>
       </c>
       <c r="R28" s="142" t="n">
         <f aca="false">R26+R27</f>
-        <v>0.333137465623433</v>
+        <v>0.456235971887826</v>
       </c>
       <c r="S28" s="142" t="n">
         <f aca="false">S26+S27</f>
-        <v>0.380033750373822</v>
+        <v>0.49284965641211</v>
       </c>
       <c r="T28" s="143" t="n">
         <f aca="false">AVERAGE(B28:S28)</f>
-        <v>-2.08746508959662</v>
+        <v>-0.905212750949604</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10246,79 +10246,79 @@
       </c>
       <c r="B5" s="50" t="n">
         <f aca="false">MASTER!B30</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C5" s="50" t="n">
         <f aca="false">MASTER!C30</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D5" s="50" t="n">
         <f aca="false">MASTER!D30</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E5" s="50" t="n">
         <f aca="false">MASTER!E30</f>
-        <v>-4181</v>
+        <v>-3437</v>
       </c>
       <c r="F5" s="50" t="n">
         <f aca="false">MASTER!F30</f>
-        <v>-4717</v>
+        <v>-3717</v>
       </c>
       <c r="G5" s="50" t="n">
         <f aca="false">MASTER!G30</f>
-        <v>-4439</v>
+        <v>-3159</v>
       </c>
       <c r="H5" s="50" t="n">
         <f aca="false">MASTER!H30</f>
-        <v>-5692</v>
+        <v>-4076</v>
       </c>
       <c r="I5" s="50" t="n">
         <f aca="false">MASTER!I30</f>
-        <v>-4625</v>
+        <v>-2649</v>
       </c>
       <c r="J5" s="50" t="n">
         <f aca="false">MASTER!J30</f>
-        <v>-3430</v>
+        <v>-1094</v>
       </c>
       <c r="K5" s="50" t="n">
         <f aca="false">MASTER!K30</f>
-        <v>-2360</v>
+        <v>282.632</v>
       </c>
       <c r="L5" s="50" t="n">
         <f aca="false">MASTER!L30</f>
-        <v>-2670</v>
+        <v>376.362</v>
       </c>
       <c r="M5" s="50" t="n">
         <f aca="false">MASTER!M30</f>
-        <v>-1469</v>
+        <v>1559.523</v>
       </c>
       <c r="N5" s="50" t="n">
         <f aca="false">MASTER!N30</f>
-        <v>670.53</v>
+        <v>3606.442</v>
       </c>
       <c r="O5" s="50" t="n">
         <f aca="false">MASTER!O30</f>
-        <v>93.009</v>
+        <v>3271.177</v>
       </c>
       <c r="P5" s="50" t="n">
         <f aca="false">MASTER!P30</f>
-        <v>2010.148</v>
+        <v>5488.252</v>
       </c>
       <c r="Q5" s="50" t="n">
         <f aca="false">MASTER!Q30</f>
-        <v>3139.234</v>
+        <v>6917.274</v>
       </c>
       <c r="R5" s="50" t="n">
         <f aca="false">MASTER!R30</f>
-        <v>5362.077</v>
+        <v>9365.069</v>
       </c>
       <c r="S5" s="50" t="n">
         <f aca="false">MASTER!S30</f>
-        <v>6831.475</v>
+        <v>11076.723</v>
       </c>
       <c r="T5" s="72" t="n">
         <f aca="false">SUM(B5:S5)</f>
-        <v>-27164.527</v>
+        <v>13067.454</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10558,79 +10558,79 @@
       </c>
       <c r="B10" s="149" t="n">
         <f aca="false">B5+B7+B8+B9</f>
-        <v>-3933</v>
+        <v>-3781</v>
       </c>
       <c r="C10" s="149" t="n">
         <f aca="false">C5+C7+C8+C9</f>
-        <v>-3883</v>
+        <v>-3603</v>
       </c>
       <c r="D10" s="149" t="n">
         <f aca="false">D5+D7+D8+D9</f>
-        <v>-3430</v>
+        <v>-2918</v>
       </c>
       <c r="E10" s="149" t="n">
         <f aca="false">E5+E7+E8+E9</f>
-        <v>-3864</v>
+        <v>-3120</v>
       </c>
       <c r="F10" s="149" t="n">
         <f aca="false">F5+F7+F8+F9</f>
-        <v>-4430</v>
+        <v>-3430</v>
       </c>
       <c r="G10" s="149" t="n">
         <f aca="false">G5+G7+G8+G9</f>
-        <v>-4292</v>
+        <v>-3012</v>
       </c>
       <c r="H10" s="149" t="n">
         <f aca="false">H5+H7+H8+H9</f>
-        <v>-5188</v>
+        <v>-3572</v>
       </c>
       <c r="I10" s="149" t="n">
         <f aca="false">I5+I7+I8+I9</f>
-        <v>-4661</v>
+        <v>-2685</v>
       </c>
       <c r="J10" s="149" t="n">
         <f aca="false">J5+J7+J8+J9</f>
-        <v>-3428</v>
+        <v>-1092</v>
       </c>
       <c r="K10" s="149" t="n">
         <f aca="false">K5+K7+K8+K9</f>
-        <v>-2399</v>
+        <v>243.632</v>
       </c>
       <c r="L10" s="149" t="n">
         <f aca="false">L5+L7+L8+L9</f>
-        <v>-2400</v>
+        <v>646.362</v>
       </c>
       <c r="M10" s="149" t="n">
         <f aca="false">M5+M7+M8+M9</f>
-        <v>-1569</v>
+        <v>1459.523</v>
       </c>
       <c r="N10" s="149" t="n">
         <f aca="false">N5+N7+N8+N9</f>
-        <v>558.53</v>
+        <v>3494.442</v>
       </c>
       <c r="O10" s="149" t="n">
         <f aca="false">O5+O7+O8+O9</f>
-        <v>355.009</v>
+        <v>3533.177</v>
       </c>
       <c r="P10" s="149" t="n">
         <f aca="false">P5+P7+P8+P9</f>
-        <v>1872.148</v>
+        <v>5350.252</v>
       </c>
       <c r="Q10" s="149" t="n">
         <f aca="false">Q5+Q7+Q8+Q9</f>
-        <v>3078.234</v>
+        <v>6856.274</v>
       </c>
       <c r="R10" s="149" t="n">
         <f aca="false">R5+R7+R8+R9</f>
-        <v>5123.077</v>
+        <v>9126.069</v>
       </c>
       <c r="S10" s="149" t="n">
         <f aca="false">S5+S7+S8+S9</f>
-        <v>6719.475</v>
+        <v>10964.723</v>
       </c>
       <c r="T10" s="150" t="n">
         <f aca="false">SUM(B10:S10)</f>
-        <v>-25770.527</v>
+        <v>14461.454</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11128,79 +11128,79 @@
       </c>
       <c r="B22" s="153" t="n">
         <f aca="false">B10+B14+B19</f>
-        <v>6067</v>
+        <v>6219</v>
       </c>
       <c r="C22" s="153" t="n">
         <f aca="false">C10+C14+C19</f>
-        <v>-3883</v>
+        <v>-3603</v>
       </c>
       <c r="D22" s="153" t="n">
         <f aca="false">D10+D14+D19</f>
-        <v>66170</v>
+        <v>66682</v>
       </c>
       <c r="E22" s="153" t="n">
         <f aca="false">E10+E14+E19</f>
-        <v>-3864</v>
+        <v>-3120</v>
       </c>
       <c r="F22" s="153" t="n">
         <f aca="false">F10+F14+F19</f>
-        <v>-4430</v>
+        <v>-3430</v>
       </c>
       <c r="G22" s="153" t="n">
         <f aca="false">G10+G14+G19</f>
-        <v>-4292</v>
+        <v>-3012</v>
       </c>
       <c r="H22" s="153" t="n">
         <f aca="false">H10+H14+H19</f>
-        <v>-5188</v>
+        <v>-3572</v>
       </c>
       <c r="I22" s="153" t="n">
         <f aca="false">I10+I14+I19</f>
-        <v>-4661</v>
+        <v>-2685</v>
       </c>
       <c r="J22" s="153" t="n">
         <f aca="false">J10+J14+J19</f>
-        <v>-3428</v>
+        <v>-1092</v>
       </c>
       <c r="K22" s="153" t="n">
         <f aca="false">K10+K14+K19</f>
-        <v>-2399</v>
+        <v>243.632</v>
       </c>
       <c r="L22" s="153" t="n">
         <f aca="false">L10+L14+L19</f>
-        <v>-6000</v>
+        <v>-2953.638</v>
       </c>
       <c r="M22" s="153" t="n">
         <f aca="false">M10+M14+M19</f>
-        <v>-1569</v>
+        <v>1459.523</v>
       </c>
       <c r="N22" s="153" t="n">
         <f aca="false">N10+N14+N19</f>
-        <v>558.53</v>
+        <v>3494.442</v>
       </c>
       <c r="O22" s="153" t="n">
         <f aca="false">O10+O14+O19</f>
-        <v>355.009</v>
+        <v>3533.177</v>
       </c>
       <c r="P22" s="153" t="n">
         <f aca="false">P10+P14+P19</f>
-        <v>1872.148</v>
+        <v>5350.252</v>
       </c>
       <c r="Q22" s="153" t="n">
         <f aca="false">Q10+Q14+Q19</f>
-        <v>3078.234</v>
+        <v>6856.274</v>
       </c>
       <c r="R22" s="153" t="n">
         <f aca="false">R10+R14+R19</f>
-        <v>5123.077</v>
+        <v>9126.069</v>
       </c>
       <c r="S22" s="153" t="n">
         <f aca="false">S10+S14+S19</f>
-        <v>6719.475</v>
+        <v>10964.723</v>
       </c>
       <c r="T22" s="154" t="n">
         <f aca="false">SUM(B22:S22)</f>
-        <v>50229.473</v>
+        <v>90461.454</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11212,75 +11212,75 @@
       </c>
       <c r="C23" s="91" t="n">
         <f aca="false">B24</f>
-        <v>6067</v>
+        <v>6219</v>
       </c>
       <c r="D23" s="91" t="n">
         <f aca="false">C24</f>
-        <v>2184</v>
+        <v>2616</v>
       </c>
       <c r="E23" s="91" t="n">
         <f aca="false">D24</f>
-        <v>68354</v>
+        <v>69298</v>
       </c>
       <c r="F23" s="91" t="n">
         <f aca="false">E24</f>
-        <v>64490</v>
+        <v>66178</v>
       </c>
       <c r="G23" s="91" t="n">
         <f aca="false">F24</f>
-        <v>60060</v>
+        <v>62748</v>
       </c>
       <c r="H23" s="91" t="n">
         <f aca="false">G24</f>
-        <v>55768</v>
+        <v>59736</v>
       </c>
       <c r="I23" s="91" t="n">
         <f aca="false">H24</f>
-        <v>50580</v>
+        <v>56164</v>
       </c>
       <c r="J23" s="91" t="n">
         <f aca="false">I24</f>
-        <v>45919</v>
+        <v>53479</v>
       </c>
       <c r="K23" s="91" t="n">
         <f aca="false">J24</f>
-        <v>42491</v>
+        <v>52387</v>
       </c>
       <c r="L23" s="91" t="n">
         <f aca="false">K24</f>
-        <v>40092</v>
+        <v>52630.632</v>
       </c>
       <c r="M23" s="91" t="n">
         <f aca="false">L24</f>
-        <v>34092</v>
+        <v>49676.994</v>
       </c>
       <c r="N23" s="91" t="n">
         <f aca="false">M24</f>
-        <v>32523</v>
+        <v>51136.517</v>
       </c>
       <c r="O23" s="91" t="n">
         <f aca="false">N24</f>
-        <v>33081.53</v>
+        <v>54630.959</v>
       </c>
       <c r="P23" s="91" t="n">
         <f aca="false">O24</f>
-        <v>33436.539</v>
+        <v>58164.136</v>
       </c>
       <c r="Q23" s="91" t="n">
         <f aca="false">P24</f>
-        <v>35308.687</v>
+        <v>63514.388</v>
       </c>
       <c r="R23" s="91" t="n">
         <f aca="false">Q24</f>
-        <v>38386.921</v>
+        <v>70370.662</v>
       </c>
       <c r="S23" s="91" t="n">
         <f aca="false">R24</f>
-        <v>43509.998</v>
+        <v>79496.731</v>
       </c>
       <c r="T23" s="72" t="n">
         <f aca="false">SUM(B23:S23)</f>
-        <v>686343.675</v>
+        <v>908446.019</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11289,79 +11289,79 @@
       </c>
       <c r="B24" s="156" t="n">
         <f aca="false">B23+B22</f>
-        <v>6067</v>
+        <v>6219</v>
       </c>
       <c r="C24" s="156" t="n">
         <f aca="false">C23+C22</f>
-        <v>2184</v>
+        <v>2616</v>
       </c>
       <c r="D24" s="156" t="n">
         <f aca="false">D23+D22</f>
-        <v>68354</v>
+        <v>69298</v>
       </c>
       <c r="E24" s="156" t="n">
         <f aca="false">E23+E22</f>
-        <v>64490</v>
+        <v>66178</v>
       </c>
       <c r="F24" s="156" t="n">
         <f aca="false">F23+F22</f>
-        <v>60060</v>
+        <v>62748</v>
       </c>
       <c r="G24" s="156" t="n">
         <f aca="false">G23+G22</f>
-        <v>55768</v>
+        <v>59736</v>
       </c>
       <c r="H24" s="156" t="n">
         <f aca="false">H23+H22</f>
-        <v>50580</v>
+        <v>56164</v>
       </c>
       <c r="I24" s="156" t="n">
         <f aca="false">I23+I22</f>
-        <v>45919</v>
+        <v>53479</v>
       </c>
       <c r="J24" s="156" t="n">
         <f aca="false">J23+J22</f>
-        <v>42491</v>
+        <v>52387</v>
       </c>
       <c r="K24" s="156" t="n">
         <f aca="false">K23+K22</f>
-        <v>40092</v>
+        <v>52630.632</v>
       </c>
       <c r="L24" s="156" t="n">
         <f aca="false">L23+L22</f>
-        <v>34092</v>
+        <v>49676.994</v>
       </c>
       <c r="M24" s="156" t="n">
         <f aca="false">M23+M22</f>
-        <v>32523</v>
+        <v>51136.517</v>
       </c>
       <c r="N24" s="156" t="n">
         <f aca="false">N23+N22</f>
-        <v>33081.53</v>
+        <v>54630.959</v>
       </c>
       <c r="O24" s="156" t="n">
         <f aca="false">O23+O22</f>
-        <v>33436.539</v>
+        <v>58164.136</v>
       </c>
       <c r="P24" s="156" t="n">
         <f aca="false">P23+P22</f>
-        <v>35308.687</v>
+        <v>63514.388</v>
       </c>
       <c r="Q24" s="156" t="n">
         <f aca="false">Q23+Q22</f>
-        <v>38386.921</v>
+        <v>70370.662</v>
       </c>
       <c r="R24" s="156" t="n">
         <f aca="false">R23+R22</f>
-        <v>43509.998</v>
+        <v>79496.731</v>
       </c>
       <c r="S24" s="156" t="n">
         <f aca="false">S23+S22</f>
-        <v>50229.473</v>
+        <v>90461.454</v>
       </c>
       <c r="T24" s="157" t="n">
         <f aca="false">SUM(B24:S24)</f>
-        <v>736573.148</v>
+        <v>998907.473</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11416,79 +11416,79 @@
       </c>
       <c r="B27" s="50" t="n">
         <f aca="false">B22</f>
-        <v>6067</v>
+        <v>6219</v>
       </c>
       <c r="C27" s="50" t="n">
         <f aca="false">C22</f>
-        <v>-3883</v>
+        <v>-3603</v>
       </c>
       <c r="D27" s="50" t="n">
         <f aca="false">D22</f>
-        <v>66170</v>
+        <v>66682</v>
       </c>
       <c r="E27" s="50" t="n">
         <f aca="false">E22</f>
-        <v>-3864</v>
+        <v>-3120</v>
       </c>
       <c r="F27" s="50" t="n">
         <f aca="false">F22</f>
-        <v>-4430</v>
+        <v>-3430</v>
       </c>
       <c r="G27" s="50" t="n">
         <f aca="false">G22</f>
-        <v>-4292</v>
+        <v>-3012</v>
       </c>
       <c r="H27" s="50" t="n">
         <f aca="false">H22</f>
-        <v>-5188</v>
+        <v>-3572</v>
       </c>
       <c r="I27" s="50" t="n">
         <f aca="false">I22</f>
-        <v>-4661</v>
+        <v>-2685</v>
       </c>
       <c r="J27" s="50" t="n">
         <f aca="false">J22</f>
-        <v>-3428</v>
+        <v>-1092</v>
       </c>
       <c r="K27" s="50" t="n">
         <f aca="false">K22</f>
-        <v>-2399</v>
+        <v>243.632</v>
       </c>
       <c r="L27" s="50" t="n">
         <f aca="false">L22</f>
-        <v>-6000</v>
+        <v>-2953.638</v>
       </c>
       <c r="M27" s="50" t="n">
         <f aca="false">M22</f>
-        <v>-1569</v>
+        <v>1459.523</v>
       </c>
       <c r="N27" s="50" t="n">
         <f aca="false">N22</f>
-        <v>558.53</v>
+        <v>3494.442</v>
       </c>
       <c r="O27" s="50" t="n">
         <f aca="false">O22</f>
-        <v>355.009</v>
+        <v>3533.177</v>
       </c>
       <c r="P27" s="50" t="n">
         <f aca="false">P22</f>
-        <v>1872.148</v>
+        <v>5350.252</v>
       </c>
       <c r="Q27" s="50" t="n">
         <f aca="false">Q22</f>
-        <v>3078.234</v>
+        <v>6856.274</v>
       </c>
       <c r="R27" s="50" t="n">
         <f aca="false">R22</f>
-        <v>5123.077</v>
+        <v>9126.069</v>
       </c>
       <c r="S27" s="50" t="n">
         <f aca="false">S22</f>
-        <v>6719.475</v>
+        <v>10964.723</v>
       </c>
       <c r="T27" s="72" t="n">
         <f aca="false">SUM(B27:S27)</f>
-        <v>50229.473</v>
+        <v>90461.454</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11501,7 +11501,7 @@
       </c>
       <c r="C28" s="159" t="n">
         <f aca="false">IF(C27&lt;0,-C24/C27,IF(C24&gt;0,99,0))</f>
-        <v>0.562451712593356</v>
+        <v>0.726061615320566</v>
       </c>
       <c r="D28" s="159" t="n">
         <f aca="false">IF(D27&lt;0,-D24/D27,IF(D24&gt;0,99,0))</f>
@@ -11509,39 +11509,39 @@
       </c>
       <c r="E28" s="159" t="n">
         <f aca="false">IF(E27&lt;0,-E24/E27,IF(E24&gt;0,99,0))</f>
-        <v>16.6899585921325</v>
+        <v>21.2108974358974</v>
       </c>
       <c r="F28" s="159" t="n">
         <f aca="false">IF(F27&lt;0,-F24/F27,IF(F24&gt;0,99,0))</f>
-        <v>13.5575620767494</v>
+        <v>18.2938775510204</v>
       </c>
       <c r="G28" s="159" t="n">
         <f aca="false">IF(G27&lt;0,-G24/G27,IF(G24&gt;0,99,0))</f>
-        <v>12.9934762348555</v>
+        <v>19.8326693227092</v>
       </c>
       <c r="H28" s="159" t="n">
         <f aca="false">IF(H27&lt;0,-H24/H27,IF(H24&gt;0,99,0))</f>
-        <v>9.74942174248265</v>
+        <v>15.7234042553192</v>
       </c>
       <c r="I28" s="159" t="n">
         <f aca="false">IF(I27&lt;0,-I24/I27,IF(I24&gt;0,99,0))</f>
-        <v>9.85174855181292</v>
+        <v>19.9176908752328</v>
       </c>
       <c r="J28" s="159" t="n">
         <f aca="false">IF(J27&lt;0,-J24/J27,IF(J24&gt;0,99,0))</f>
-        <v>12.3952742123687</v>
+        <v>47.9734432234432</v>
       </c>
       <c r="K28" s="159" t="n">
         <f aca="false">IF(K27&lt;0,-K24/K27,IF(K24&gt;0,99,0))</f>
-        <v>16.7119633180492</v>
+        <v>99</v>
       </c>
       <c r="L28" s="159" t="n">
         <f aca="false">IF(L27&lt;0,-L24/L27,IF(L24&gt;0,99,0))</f>
-        <v>5.682</v>
+        <v>16.8189175518462</v>
       </c>
       <c r="M28" s="159" t="n">
         <f aca="false">IF(M27&lt;0,-M24/M27,IF(M24&gt;0,99,0))</f>
-        <v>20.7284894837476</v>
+        <v>99</v>
       </c>
       <c r="N28" s="159" t="n">
         <f aca="false">IF(N27&lt;0,-N24/N27,IF(N24&gt;0,99,0))</f>
@@ -11569,7 +11569,7 @@
       </c>
       <c r="T28" s="160" t="n">
         <f aca="false">SUM(B28:S28)</f>
-        <v>910.922345924792</v>
+        <v>1150.49696183079</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12055,79 +12055,79 @@
       </c>
       <c r="B10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!B24</f>
-        <v>6067</v>
+        <v>6219</v>
       </c>
       <c r="C10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!C24</f>
-        <v>2184</v>
+        <v>2616</v>
       </c>
       <c r="D10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!D24</f>
-        <v>68354</v>
+        <v>69298</v>
       </c>
       <c r="E10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!E24</f>
-        <v>64490</v>
+        <v>66178</v>
       </c>
       <c r="F10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!F24</f>
-        <v>60060</v>
+        <v>62748</v>
       </c>
       <c r="G10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!G24</f>
-        <v>55768</v>
+        <v>59736</v>
       </c>
       <c r="H10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!H24</f>
-        <v>50580</v>
+        <v>56164</v>
       </c>
       <c r="I10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!I24</f>
-        <v>45919</v>
+        <v>53479</v>
       </c>
       <c r="J10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!J24</f>
-        <v>42491</v>
+        <v>52387</v>
       </c>
       <c r="K10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!K24</f>
-        <v>40092</v>
+        <v>52630.632</v>
       </c>
       <c r="L10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!L24</f>
-        <v>34092</v>
+        <v>49676.994</v>
       </c>
       <c r="M10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!M24</f>
-        <v>32523</v>
+        <v>51136.517</v>
       </c>
       <c r="N10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!N24</f>
-        <v>33081.53</v>
+        <v>54630.959</v>
       </c>
       <c r="O10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!O24</f>
-        <v>33436.539</v>
+        <v>58164.136</v>
       </c>
       <c r="P10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!P24</f>
-        <v>35308.687</v>
+        <v>63514.388</v>
       </c>
       <c r="Q10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!Q24</f>
-        <v>38386.921</v>
+        <v>70370.662</v>
       </c>
       <c r="R10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!R24</f>
-        <v>43509.998</v>
+        <v>79496.731</v>
       </c>
       <c r="S10" s="50" t="n">
         <f aca="false">'Budget di Cassa'!S24</f>
-        <v>50229.473</v>
+        <v>90461.454</v>
       </c>
       <c r="T10" s="72" t="n">
         <f aca="false">SUM(B10:S10)</f>
-        <v>736573.148</v>
+        <v>998907.473</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12207,71 +12207,71 @@
       </c>
       <c r="D12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(D10*0.025/12,0))</f>
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(E10*0.025/12,0))</f>
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(F10*0.025/12,0))</f>
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(G10*0.025/12,0))</f>
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(H10*0.025/12,0))</f>
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="I12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(I10*0.025/12,0))</f>
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="J12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(J10*0.025/12,0))</f>
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="K12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(K10*0.025/12,0))</f>
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="L12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(L10*0.025/12,0))</f>
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="M12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(M10*0.025/12,0))</f>
-        <v>68</v>
+        <v>107</v>
       </c>
       <c r="N12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(N10*0.025/12,0))</f>
-        <v>69</v>
+        <v>114</v>
       </c>
       <c r="O12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(O10*0.025/12,0))</f>
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="P12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(P10*0.025/12,0))</f>
-        <v>74</v>
+        <v>132</v>
       </c>
       <c r="Q12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(Q10*0.025/12,0))</f>
-        <v>80</v>
+        <v>147</v>
       </c>
       <c r="R12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(R10*0.025/12,0))</f>
-        <v>91</v>
+        <v>166</v>
       </c>
       <c r="S12" s="50" t="n">
         <f aca="false">MAX(0,ROUND(S10*0.025/12,0))</f>
-        <v>105</v>
+        <v>188</v>
       </c>
       <c r="T12" s="72" t="n">
         <f aca="false">SUM(B12:S12)</f>
-        <v>1537</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12280,79 +12280,79 @@
       </c>
       <c r="B13" s="46" t="n">
         <f aca="false">B10+B11+B12</f>
-        <v>6080</v>
+        <v>6232</v>
       </c>
       <c r="C13" s="46" t="n">
         <f aca="false">C10+C11+C12</f>
-        <v>2189</v>
+        <v>2621</v>
       </c>
       <c r="D13" s="46" t="n">
         <f aca="false">D10+D11+D12</f>
-        <v>68526</v>
+        <v>69472</v>
       </c>
       <c r="E13" s="46" t="n">
         <f aca="false">E10+E11+E12</f>
-        <v>64713</v>
+        <v>66405</v>
       </c>
       <c r="F13" s="46" t="n">
         <f aca="false">F10+F11+F12</f>
-        <v>60334</v>
+        <v>63028</v>
       </c>
       <c r="G13" s="46" t="n">
         <f aca="false">G10+G11+G12</f>
-        <v>56122</v>
+        <v>60098</v>
       </c>
       <c r="H13" s="46" t="n">
         <f aca="false">H10+H11+H12</f>
-        <v>50983</v>
+        <v>56579</v>
       </c>
       <c r="I13" s="46" t="n">
         <f aca="false">I10+I11+I12</f>
-        <v>46403</v>
+        <v>53978</v>
       </c>
       <c r="J13" s="46" t="n">
         <f aca="false">J10+J11+J12</f>
-        <v>43027</v>
+        <v>52943</v>
       </c>
       <c r="K13" s="46" t="n">
         <f aca="false">K10+K11+K12</f>
-        <v>40713</v>
+        <v>53277.632</v>
       </c>
       <c r="L13" s="46" t="n">
         <f aca="false">L10+L11+L12</f>
-        <v>34759</v>
+        <v>50375.994</v>
       </c>
       <c r="M13" s="46" t="n">
         <f aca="false">M10+M11+M12</f>
-        <v>33277</v>
+        <v>51929.517</v>
       </c>
       <c r="N13" s="46" t="n">
         <f aca="false">N10+N11+N12</f>
-        <v>33955.53</v>
+        <v>55549.959</v>
       </c>
       <c r="O13" s="46" t="n">
         <f aca="false">O10+O11+O12</f>
-        <v>34550.539</v>
+        <v>59329.136</v>
       </c>
       <c r="P13" s="46" t="n">
         <f aca="false">P10+P11+P12</f>
-        <v>36575.687</v>
+        <v>64839.388</v>
       </c>
       <c r="Q13" s="46" t="n">
         <f aca="false">Q10+Q11+Q12</f>
-        <v>39749.921</v>
+        <v>71800.662</v>
       </c>
       <c r="R13" s="46" t="n">
         <f aca="false">R10+R11+R12</f>
-        <v>45182.998</v>
+        <v>81244.731</v>
       </c>
       <c r="S13" s="46" t="n">
         <f aca="false">S10+S11+S12</f>
-        <v>52065.473</v>
+        <v>92380.454</v>
       </c>
       <c r="T13" s="125" t="n">
         <f aca="false">SUM(B13:S13)</f>
-        <v>749206.148</v>
+        <v>1012083.473</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12361,79 +12361,79 @@
       </c>
       <c r="B14" s="58" t="n">
         <f aca="false">B8+B13</f>
-        <v>6080</v>
+        <v>6232</v>
       </c>
       <c r="C14" s="58" t="n">
         <f aca="false">C8+C13</f>
-        <v>2189</v>
+        <v>2621</v>
       </c>
       <c r="D14" s="58" t="n">
         <f aca="false">D8+D13</f>
-        <v>73326</v>
+        <v>74272</v>
       </c>
       <c r="E14" s="58" t="n">
         <f aca="false">E8+E13</f>
-        <v>69313</v>
+        <v>71005</v>
       </c>
       <c r="F14" s="58" t="n">
         <f aca="false">F8+F13</f>
-        <v>64734</v>
+        <v>67428</v>
       </c>
       <c r="G14" s="58" t="n">
         <f aca="false">G8+G13</f>
-        <v>60322</v>
+        <v>64298</v>
       </c>
       <c r="H14" s="58" t="n">
         <f aca="false">H8+H13</f>
-        <v>54983</v>
+        <v>60579</v>
       </c>
       <c r="I14" s="58" t="n">
         <f aca="false">I8+I13</f>
-        <v>50203</v>
+        <v>57778</v>
       </c>
       <c r="J14" s="58" t="n">
         <f aca="false">J8+J13</f>
-        <v>46627</v>
+        <v>56543</v>
       </c>
       <c r="K14" s="58" t="n">
         <f aca="false">K8+K13</f>
-        <v>44113</v>
+        <v>56677.632</v>
       </c>
       <c r="L14" s="58" t="n">
         <f aca="false">L8+L13</f>
-        <v>41559</v>
+        <v>57175.994</v>
       </c>
       <c r="M14" s="58" t="n">
         <f aca="false">M8+M13</f>
-        <v>39877</v>
+        <v>58529.517</v>
       </c>
       <c r="N14" s="58" t="n">
         <f aca="false">N8+N13</f>
-        <v>40355.53</v>
+        <v>61949.959</v>
       </c>
       <c r="O14" s="58" t="n">
         <f aca="false">O8+O13</f>
-        <v>40750.539</v>
+        <v>65529.136</v>
       </c>
       <c r="P14" s="58" t="n">
         <f aca="false">P8+P13</f>
-        <v>42575.687</v>
+        <v>70839.388</v>
       </c>
       <c r="Q14" s="58" t="n">
         <f aca="false">Q8+Q13</f>
-        <v>45549.921</v>
+        <v>77600.662</v>
       </c>
       <c r="R14" s="58" t="n">
         <f aca="false">R8+R13</f>
-        <v>50782.998</v>
+        <v>86844.731</v>
       </c>
       <c r="S14" s="58" t="n">
         <f aca="false">S8+S13</f>
-        <v>57465.473</v>
+        <v>97780.454</v>
       </c>
       <c r="T14" s="58" t="n">
         <f aca="false">SUM(B14:S14)</f>
-        <v>830806.148</v>
+        <v>1093683.473</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13062,75 +13062,75 @@
       </c>
       <c r="C28" s="91" t="n">
         <f aca="false">MASTER!B30</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="D28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30</f>
-        <v>-8184</v>
+        <v>-7752</v>
       </c>
       <c r="E28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30</f>
-        <v>-11688</v>
+        <v>-10744</v>
       </c>
       <c r="F28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30</f>
-        <v>-15869</v>
+        <v>-14181</v>
       </c>
       <c r="G28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30</f>
-        <v>-20586</v>
+        <v>-17898</v>
       </c>
       <c r="H28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30</f>
-        <v>-25025</v>
+        <v>-21057</v>
       </c>
       <c r="I28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30</f>
-        <v>-30717</v>
+        <v>-25133</v>
       </c>
       <c r="J28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30</f>
-        <v>-35342</v>
+        <v>-27782</v>
       </c>
       <c r="K28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30</f>
-        <v>-38772</v>
+        <v>-28876</v>
       </c>
       <c r="L28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30</f>
-        <v>-41132</v>
+        <v>-28593.368</v>
       </c>
       <c r="M28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30</f>
-        <v>-43802</v>
+        <v>-28217.006</v>
       </c>
       <c r="N28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30+MASTER!M30</f>
-        <v>-45271</v>
+        <v>-26657.483</v>
       </c>
       <c r="O28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30+MASTER!M30+MASTER!N30</f>
-        <v>-44600.47</v>
+        <v>-23051.041</v>
       </c>
       <c r="P28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30+MASTER!M30+MASTER!N30+MASTER!O30</f>
-        <v>-44507.461</v>
+        <v>-19779.864</v>
       </c>
       <c r="Q28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30+MASTER!M30+MASTER!N30+MASTER!O30+MASTER!P30</f>
-        <v>-42497.313</v>
+        <v>-14291.612</v>
       </c>
       <c r="R28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30+MASTER!M30+MASTER!N30+MASTER!O30+MASTER!P30+MASTER!Q30</f>
-        <v>-39358.079</v>
+        <v>-7374.338</v>
       </c>
       <c r="S28" s="91" t="n">
         <f aca="false">MASTER!B30+MASTER!C30+MASTER!D30+MASTER!E30+MASTER!F30+MASTER!G30+MASTER!H30+MASTER!I30+MASTER!J30+MASTER!K30+MASTER!L30+MASTER!M30+MASTER!N30+MASTER!O30+MASTER!P30+MASTER!Q30+MASTER!R30</f>
-        <v>-33996.002</v>
+        <v>1990.731</v>
       </c>
       <c r="T28" s="72" t="n">
         <f aca="false">SUM(B28:S28)</f>
-        <v>-525480.325</v>
+        <v>-303377.981</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13139,79 +13139,79 @@
       </c>
       <c r="B29" s="50" t="n">
         <f aca="false">MASTER!B30</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C29" s="50" t="n">
         <f aca="false">MASTER!C30</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D29" s="50" t="n">
         <f aca="false">MASTER!D30</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E29" s="50" t="n">
         <f aca="false">MASTER!E30</f>
-        <v>-4181</v>
+        <v>-3437</v>
       </c>
       <c r="F29" s="50" t="n">
         <f aca="false">MASTER!F30</f>
-        <v>-4717</v>
+        <v>-3717</v>
       </c>
       <c r="G29" s="50" t="n">
         <f aca="false">MASTER!G30</f>
-        <v>-4439</v>
+        <v>-3159</v>
       </c>
       <c r="H29" s="50" t="n">
         <f aca="false">MASTER!H30</f>
-        <v>-5692</v>
+        <v>-4076</v>
       </c>
       <c r="I29" s="50" t="n">
         <f aca="false">MASTER!I30</f>
-        <v>-4625</v>
+        <v>-2649</v>
       </c>
       <c r="J29" s="50" t="n">
         <f aca="false">MASTER!J30</f>
-        <v>-3430</v>
+        <v>-1094</v>
       </c>
       <c r="K29" s="50" t="n">
         <f aca="false">MASTER!K30</f>
-        <v>-2360</v>
+        <v>282.632</v>
       </c>
       <c r="L29" s="50" t="n">
         <f aca="false">MASTER!L30</f>
-        <v>-2670</v>
+        <v>376.362</v>
       </c>
       <c r="M29" s="50" t="n">
         <f aca="false">MASTER!M30</f>
-        <v>-1469</v>
+        <v>1559.523</v>
       </c>
       <c r="N29" s="50" t="n">
         <f aca="false">MASTER!N30</f>
-        <v>670.53</v>
+        <v>3606.442</v>
       </c>
       <c r="O29" s="50" t="n">
         <f aca="false">MASTER!O30</f>
-        <v>93.009</v>
+        <v>3271.177</v>
       </c>
       <c r="P29" s="50" t="n">
         <f aca="false">MASTER!P30</f>
-        <v>2010.148</v>
+        <v>5488.252</v>
       </c>
       <c r="Q29" s="50" t="n">
         <f aca="false">MASTER!Q30</f>
-        <v>3139.234</v>
+        <v>6917.274</v>
       </c>
       <c r="R29" s="50" t="n">
         <f aca="false">MASTER!R30</f>
-        <v>5362.077</v>
+        <v>9365.069</v>
       </c>
       <c r="S29" s="50" t="n">
         <f aca="false">MASTER!S30</f>
-        <v>6831.475</v>
+        <v>11076.723</v>
       </c>
       <c r="T29" s="72" t="n">
         <f aca="false">SUM(B29:S29)</f>
-        <v>-27164.527</v>
+        <v>13067.454</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13220,79 +13220,79 @@
       </c>
       <c r="B30" s="168" t="n">
         <f aca="false">B27+B28+B29</f>
-        <v>5868</v>
+        <v>6020</v>
       </c>
       <c r="C30" s="168" t="n">
         <f aca="false">C27+C28+C29</f>
-        <v>1817</v>
+        <v>2249</v>
       </c>
       <c r="D30" s="168" t="n">
         <f aca="false">D27+D28+D29</f>
-        <v>73313</v>
+        <v>74257</v>
       </c>
       <c r="E30" s="168" t="n">
         <f aca="false">E27+E28+E29</f>
-        <v>69132</v>
+        <v>70820</v>
       </c>
       <c r="F30" s="168" t="n">
         <f aca="false">F27+F28+F29</f>
-        <v>64415</v>
+        <v>67103</v>
       </c>
       <c r="G30" s="168" t="n">
         <f aca="false">G27+G28+G29</f>
-        <v>59976</v>
+        <v>63944</v>
       </c>
       <c r="H30" s="168" t="n">
         <f aca="false">H27+H28+H29</f>
-        <v>54284</v>
+        <v>59868</v>
       </c>
       <c r="I30" s="168" t="n">
         <f aca="false">I27+I28+I29</f>
-        <v>49659</v>
+        <v>57219</v>
       </c>
       <c r="J30" s="168" t="n">
         <f aca="false">J27+J28+J29</f>
-        <v>46229</v>
+        <v>56125</v>
       </c>
       <c r="K30" s="168" t="n">
         <f aca="false">K27+K28+K29</f>
-        <v>43869</v>
+        <v>56407.632</v>
       </c>
       <c r="L30" s="168" t="n">
         <f aca="false">L27+L28+L29</f>
-        <v>41199</v>
+        <v>56783.994</v>
       </c>
       <c r="M30" s="168" t="n">
         <f aca="false">M27+M28+M29</f>
-        <v>39730</v>
+        <v>58343.517</v>
       </c>
       <c r="N30" s="168" t="n">
         <f aca="false">N27+N28+N29</f>
-        <v>40400.53</v>
+        <v>61949.959</v>
       </c>
       <c r="O30" s="168" t="n">
         <f aca="false">O27+O28+O29</f>
-        <v>40493.539</v>
+        <v>65221.136</v>
       </c>
       <c r="P30" s="168" t="n">
         <f aca="false">P27+P28+P29</f>
-        <v>42503.687</v>
+        <v>70709.388</v>
       </c>
       <c r="Q30" s="168" t="n">
         <f aca="false">Q27+Q28+Q29</f>
-        <v>45642.921</v>
+        <v>77626.662</v>
       </c>
       <c r="R30" s="168" t="n">
         <f aca="false">R27+R28+R29</f>
-        <v>51004.998</v>
+        <v>86991.731</v>
       </c>
       <c r="S30" s="168" t="n">
         <f aca="false">S27+S28+S29</f>
-        <v>57836.473</v>
+        <v>98068.454</v>
       </c>
       <c r="T30" s="169" t="n">
         <f aca="false">SUM(B30:S30)</f>
-        <v>827373.148</v>
+        <v>1089707.473</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13355,71 +13355,71 @@
       </c>
       <c r="D33" s="50" t="n">
         <f aca="false">D14-D24-D30</f>
-        <v>-899</v>
+        <v>-897</v>
       </c>
       <c r="E33" s="50" t="n">
         <f aca="false">E14-E24-E30</f>
-        <v>-1065</v>
+        <v>-1061</v>
       </c>
       <c r="F33" s="50" t="n">
         <f aca="false">F14-F24-F30</f>
-        <v>-1231</v>
+        <v>-1225</v>
       </c>
       <c r="G33" s="50" t="n">
         <f aca="false">G14-G24-G30</f>
-        <v>-1409</v>
+        <v>-1401</v>
       </c>
       <c r="H33" s="50" t="n">
         <f aca="false">H14-H24-H30</f>
-        <v>-1621</v>
+        <v>-1609</v>
       </c>
       <c r="I33" s="50" t="n">
         <f aca="false">I14-I24-I30</f>
-        <v>-1849</v>
+        <v>-1834</v>
       </c>
       <c r="J33" s="50" t="n">
         <f aca="false">J14-J24-J30</f>
-        <v>-2076</v>
+        <v>-2056</v>
       </c>
       <c r="K33" s="50" t="n">
         <f aca="false">K14-K24-K30</f>
-        <v>-2306</v>
+        <v>-2280</v>
       </c>
       <c r="L33" s="50" t="n">
         <f aca="false">L14-L24-L30</f>
-        <v>-2629</v>
+        <v>-2597</v>
       </c>
       <c r="M33" s="50" t="n">
         <f aca="false">M14-M24-M30</f>
-        <v>-2939</v>
+        <v>-2900.00000000001</v>
       </c>
       <c r="N33" s="50" t="n">
         <f aca="false">N14-N24-N30</f>
-        <v>-3248</v>
+        <v>-3203.00000000001</v>
       </c>
       <c r="O33" s="50" t="n">
         <f aca="false">O14-O24-O30</f>
-        <v>-3520</v>
+        <v>-3469</v>
       </c>
       <c r="P33" s="50" t="n">
         <f aca="false">P14-P24-P30</f>
-        <v>-3813</v>
+        <v>-3755</v>
       </c>
       <c r="Q33" s="50" t="n">
         <f aca="false">Q14-Q24-Q30</f>
-        <v>-4073</v>
+        <v>-4006.00000000001</v>
       </c>
       <c r="R33" s="50" t="n">
         <f aca="false">R14-R24-R30</f>
-        <v>-4299</v>
+        <v>-4224</v>
       </c>
       <c r="S33" s="50" t="n">
         <f aca="false">S14-S24-S30</f>
-        <v>-4541</v>
+        <v>-4458</v>
       </c>
       <c r="T33" s="72" t="n">
         <f aca="false">SUM(B33:S33)</f>
-        <v>-42681</v>
+        <v>-42138</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13436,67 +13436,67 @@
       </c>
       <c r="D34" s="126" t="str">
         <f aca="false">IF(ABS(D33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(D33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-899)</v>
+        <v>⚠️ RIVEDI (-897)</v>
       </c>
       <c r="E34" s="126" t="str">
         <f aca="false">IF(ABS(E33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(E33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-1065)</v>
+        <v>⚠️ RIVEDI (-1061)</v>
       </c>
       <c r="F34" s="126" t="str">
         <f aca="false">IF(ABS(F33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(F33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-1231)</v>
+        <v>⚠️ RIVEDI (-1225)</v>
       </c>
       <c r="G34" s="126" t="str">
         <f aca="false">IF(ABS(G33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(G33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-1409)</v>
+        <v>⚠️ RIVEDI (-1401)</v>
       </c>
       <c r="H34" s="126" t="str">
         <f aca="false">IF(ABS(H33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(H33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-1621)</v>
+        <v>⚠️ RIVEDI (-1609)</v>
       </c>
       <c r="I34" s="126" t="str">
         <f aca="false">IF(ABS(I33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(I33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-1849)</v>
+        <v>⚠️ RIVEDI (-1834)</v>
       </c>
       <c r="J34" s="126" t="str">
         <f aca="false">IF(ABS(J33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(J33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-2076)</v>
+        <v>⚠️ RIVEDI (-2056)</v>
       </c>
       <c r="K34" s="126" t="str">
         <f aca="false">IF(ABS(K33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(K33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-2306)</v>
+        <v>⚠️ RIVEDI (-2280)</v>
       </c>
       <c r="L34" s="126" t="str">
         <f aca="false">IF(ABS(L33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(L33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-2629)</v>
+        <v>⚠️ RIVEDI (-2597)</v>
       </c>
       <c r="M34" s="126" t="str">
         <f aca="false">IF(ABS(M33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(M33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-2939)</v>
+        <v>⚠️ RIVEDI (-2900)</v>
       </c>
       <c r="N34" s="126" t="str">
         <f aca="false">IF(ABS(N33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(N33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-3248)</v>
+        <v>⚠️ RIVEDI (-3203)</v>
       </c>
       <c r="O34" s="126" t="str">
         <f aca="false">IF(ABS(O33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(O33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-3520)</v>
+        <v>⚠️ RIVEDI (-3469)</v>
       </c>
       <c r="P34" s="126" t="str">
         <f aca="false">IF(ABS(P33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(P33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-3813)</v>
+        <v>⚠️ RIVEDI (-3755)</v>
       </c>
       <c r="Q34" s="126" t="str">
         <f aca="false">IF(ABS(Q33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(Q33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-4073)</v>
+        <v>⚠️ RIVEDI (-4006)</v>
       </c>
       <c r="R34" s="126" t="str">
         <f aca="false">IF(ABS(R33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(R33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-4299)</v>
+        <v>⚠️ RIVEDI (-4224)</v>
       </c>
       <c r="S34" s="126" t="str">
         <f aca="false">IF(ABS(S33)&lt;500,"✅ OK","⚠️ RIVEDI (" &amp; ROUND(S33,0) &amp; ")")</f>
-        <v>⚠️ RIVEDI (-4541)</v>
+        <v>⚠️ RIVEDI (-4458)</v>
       </c>
       <c r="T34" s="127" t="s">
         <v>527</v>
@@ -14009,79 +14009,79 @@
       </c>
       <c r="B9" s="21" t="n">
         <f aca="false">B6+B7+B8+IF(ISNUMBER('A.4 — Fee per Ordine'!B39),'A.4 — Fee per Ordine'!B39,0)</f>
-        <v>196</v>
+        <v>348</v>
       </c>
       <c r="C9" s="21" t="n">
         <f aca="false">C6+C7+C8+IF(ISNUMBER('A.4 — Fee per Ordine'!C39),'A.4 — Fee per Ordine'!C39,0)</f>
-        <v>353</v>
+        <v>633</v>
       </c>
       <c r="D9" s="21" t="n">
         <f aca="false">D6+D7+D8+IF(ISNUMBER('A.4 — Fee per Ordine'!D39),'A.4 — Fee per Ordine'!D39,0)</f>
-        <v>1056</v>
+        <v>1568</v>
       </c>
       <c r="E9" s="21" t="n">
         <f aca="false">E6+E7+E8+IF(ISNUMBER('A.4 — Fee per Ordine'!E39),'A.4 — Fee per Ordine'!E39,0)</f>
-        <v>2001</v>
+        <v>2745</v>
       </c>
       <c r="F9" s="21" t="n">
         <f aca="false">F6+F7+F8+IF(ISNUMBER('A.4 — Fee per Ordine'!F39),'A.4 — Fee per Ordine'!F39,0)</f>
-        <v>2984</v>
+        <v>3984</v>
       </c>
       <c r="G9" s="21" t="n">
         <f aca="false">G6+G7+G8+IF(ISNUMBER('A.4 — Fee per Ordine'!G39),'A.4 — Fee per Ordine'!G39,0)</f>
-        <v>4285</v>
+        <v>5565</v>
       </c>
       <c r="H9" s="21" t="n">
         <f aca="false">H6+H7+H8+IF(ISNUMBER('A.4 — Fee per Ordine'!H39),'A.4 — Fee per Ordine'!H39,0)</f>
-        <v>5828</v>
+        <v>7444</v>
       </c>
       <c r="I9" s="21" t="n">
         <f aca="false">I6+I7+I8+IF(ISNUMBER('A.4 — Fee per Ordine'!I39),'A.4 — Fee per Ordine'!I39,0)</f>
-        <v>7259</v>
+        <v>9235</v>
       </c>
       <c r="J9" s="21" t="n">
         <f aca="false">J6+J7+J8+IF(ISNUMBER('A.4 — Fee per Ordine'!J39),'A.4 — Fee per Ordine'!J39,0)</f>
-        <v>8861</v>
+        <v>11197</v>
       </c>
       <c r="K9" s="21" t="n">
         <f aca="false">K6+K7+K8+IF(ISNUMBER('A.4 — Fee per Ordine'!K39),'A.4 — Fee per Ordine'!K39,0)</f>
-        <v>10312</v>
+        <v>13064</v>
       </c>
       <c r="L9" s="21" t="n">
         <f aca="false">L6+L7+L8+IF(ISNUMBER('A.4 — Fee per Ordine'!L39),'A.4 — Fee per Ordine'!L39,0)</f>
-        <v>12173</v>
+        <v>15365</v>
       </c>
       <c r="M9" s="21" t="n">
         <f aca="false">M6+M7+M8+IF(ISNUMBER('A.4 — Fee per Ordine'!M39),'A.4 — Fee per Ordine'!M39,0)</f>
-        <v>13863</v>
+        <v>17495</v>
       </c>
       <c r="N9" s="21" t="n">
         <f aca="false">N6+N7+N8+IF(ISNUMBER('A.4 — Fee per Ordine'!N39),'A.4 — Fee per Ordine'!N39,0)</f>
-        <v>16823</v>
+        <v>20895</v>
       </c>
       <c r="O9" s="21" t="n">
         <f aca="false">O6+O7+O8+IF(ISNUMBER('A.4 — Fee per Ordine'!O39),'A.4 — Fee per Ordine'!O39,0)</f>
-        <v>18894</v>
+        <v>23302</v>
       </c>
       <c r="P9" s="21" t="n">
         <f aca="false">P6+P7+P8+IF(ISNUMBER('A.4 — Fee per Ordine'!P39),'A.4 — Fee per Ordine'!P39,0)</f>
-        <v>22094</v>
+        <v>26918</v>
       </c>
       <c r="Q9" s="21" t="n">
         <f aca="false">Q6+Q7+Q8+IF(ISNUMBER('A.4 — Fee per Ordine'!Q39),'A.4 — Fee per Ordine'!Q39,0)</f>
-        <v>24134</v>
+        <v>29374</v>
       </c>
       <c r="R9" s="21" t="n">
         <f aca="false">R6+R7+R8+IF(ISNUMBER('A.4 — Fee per Ordine'!R39),'A.4 — Fee per Ordine'!R39,0)</f>
-        <v>27674</v>
+        <v>33226</v>
       </c>
       <c r="S9" s="21" t="n">
         <f aca="false">S6+S7+S8+IF(ISNUMBER('A.4 — Fee per Ordine'!S39),'A.4 — Fee per Ordine'!S39,0)</f>
-        <v>30174</v>
+        <v>36062</v>
       </c>
       <c r="T9" s="21" t="n">
         <f aca="false">SUM(B9:S9)</f>
-        <v>208964</v>
+        <v>258420</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14725,79 +14725,79 @@
       </c>
       <c r="B20" s="35" t="n">
         <f aca="false">B9-B18</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C20" s="35" t="n">
         <f aca="false">C9-C18</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D20" s="35" t="n">
         <f aca="false">D9-D18</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E20" s="35" t="n">
         <f aca="false">E9-E18</f>
-        <v>-4231</v>
+        <v>-3487</v>
       </c>
       <c r="F20" s="35" t="n">
         <f aca="false">F9-F18</f>
-        <v>-4767</v>
+        <v>-3767</v>
       </c>
       <c r="G20" s="35" t="n">
         <f aca="false">G9-G18</f>
-        <v>-4489</v>
+        <v>-3209</v>
       </c>
       <c r="H20" s="35" t="n">
         <f aca="false">H9-H18</f>
-        <v>-5772</v>
+        <v>-4156</v>
       </c>
       <c r="I20" s="35" t="n">
         <f aca="false">I9-I18</f>
-        <v>-4705</v>
+        <v>-2729</v>
       </c>
       <c r="J20" s="35" t="n">
         <f aca="false">J9-J18</f>
-        <v>-3510</v>
+        <v>-1174</v>
       </c>
       <c r="K20" s="35" t="n">
         <f aca="false">K9-K18</f>
-        <v>-2440</v>
+        <v>312</v>
       </c>
       <c r="L20" s="35" t="n">
         <f aca="false">L9-L18</f>
-        <v>-2770</v>
+        <v>422</v>
       </c>
       <c r="M20" s="35" t="n">
         <f aca="false">M9-M18</f>
-        <v>-1569</v>
+        <v>2063</v>
       </c>
       <c r="N20" s="35" t="n">
         <f aca="false">N9-N18</f>
-        <v>810</v>
+        <v>4882</v>
       </c>
       <c r="O20" s="35" t="n">
         <f aca="false">O9-O18</f>
-        <v>9</v>
+        <v>4417</v>
       </c>
       <c r="P20" s="35" t="n">
         <f aca="false">P9-P18</f>
-        <v>2668</v>
+        <v>7492</v>
       </c>
       <c r="Q20" s="35" t="n">
         <f aca="false">Q9-Q18</f>
-        <v>4234</v>
+        <v>9474</v>
       </c>
       <c r="R20" s="35" t="n">
         <f aca="false">R9-R18</f>
-        <v>7287</v>
+        <v>12839</v>
       </c>
       <c r="S20" s="35" t="n">
         <f aca="false">S9-S18</f>
-        <v>9325</v>
+        <v>15213</v>
       </c>
       <c r="T20" s="35" t="n">
         <f aca="false">SUM(B20:S20)</f>
-        <v>-21608</v>
+        <v>27848</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15014,79 +15014,79 @@
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">B20+B23-B24</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C25" s="33" t="n">
         <f aca="false">C20+C23-C24</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D25" s="33" t="n">
         <f aca="false">D20+D23-D24</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E25" s="33" t="n">
         <f aca="false">E20+E23-E24</f>
-        <v>-4181</v>
+        <v>-3437</v>
       </c>
       <c r="F25" s="33" t="n">
         <f aca="false">F20+F23-F24</f>
-        <v>-4717</v>
+        <v>-3717</v>
       </c>
       <c r="G25" s="33" t="n">
         <f aca="false">G20+G23-G24</f>
-        <v>-4439</v>
+        <v>-3159</v>
       </c>
       <c r="H25" s="33" t="n">
         <f aca="false">H20+H23-H24</f>
-        <v>-5692</v>
+        <v>-4076</v>
       </c>
       <c r="I25" s="33" t="n">
         <f aca="false">I20+I23-I24</f>
-        <v>-4625</v>
+        <v>-2649</v>
       </c>
       <c r="J25" s="33" t="n">
         <f aca="false">J20+J23-J24</f>
-        <v>-3430</v>
+        <v>-1094</v>
       </c>
       <c r="K25" s="33" t="n">
         <f aca="false">K20+K23-K24</f>
-        <v>-2360</v>
+        <v>392</v>
       </c>
       <c r="L25" s="33" t="n">
         <f aca="false">L20+L23-L24</f>
-        <v>-2670</v>
+        <v>522</v>
       </c>
       <c r="M25" s="33" t="n">
         <f aca="false">M20+M23-M24</f>
-        <v>-1469</v>
+        <v>2163</v>
       </c>
       <c r="N25" s="33" t="n">
         <f aca="false">N20+N23-N24</f>
-        <v>930</v>
+        <v>5002</v>
       </c>
       <c r="O25" s="33" t="n">
         <f aca="false">O20+O23-O24</f>
-        <v>129</v>
+        <v>4537</v>
       </c>
       <c r="P25" s="33" t="n">
         <f aca="false">P20+P23-P24</f>
-        <v>2788</v>
+        <v>7612</v>
       </c>
       <c r="Q25" s="33" t="n">
         <f aca="false">Q20+Q23-Q24</f>
-        <v>4354</v>
+        <v>9594</v>
       </c>
       <c r="R25" s="33" t="n">
         <f aca="false">R20+R23-R24</f>
-        <v>7437</v>
+        <v>12989</v>
       </c>
       <c r="S25" s="33" t="n">
         <f aca="false">S20+S23-S24</f>
-        <v>9475</v>
+        <v>15363</v>
       </c>
       <c r="T25" s="33" t="n">
         <f aca="false">SUM(B25:S25)</f>
-        <v>-20158</v>
+        <v>29298</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15177,43 +15177,43 @@
       </c>
       <c r="K28" s="18" t="n">
         <f aca="false">MAX(0,K25*0.279)</f>
-        <v>0</v>
+        <v>109.368</v>
       </c>
       <c r="L28" s="18" t="n">
         <f aca="false">MAX(0,L25*0.279)</f>
-        <v>0</v>
+        <v>145.638</v>
       </c>
       <c r="M28" s="18" t="n">
         <f aca="false">MAX(0,M25*0.279)</f>
-        <v>0</v>
+        <v>603.477</v>
       </c>
       <c r="N28" s="18" t="n">
         <f aca="false">MAX(0,N25*0.279)</f>
-        <v>259.47</v>
+        <v>1395.558</v>
       </c>
       <c r="O28" s="18" t="n">
         <f aca="false">MAX(0,O25*0.279)</f>
-        <v>35.991</v>
+        <v>1265.823</v>
       </c>
       <c r="P28" s="18" t="n">
         <f aca="false">MAX(0,P25*0.279)</f>
-        <v>777.852</v>
+        <v>2123.748</v>
       </c>
       <c r="Q28" s="18" t="n">
         <f aca="false">MAX(0,Q25*0.279)</f>
-        <v>1214.766</v>
+        <v>2676.726</v>
       </c>
       <c r="R28" s="18" t="n">
         <f aca="false">MAX(0,R25*0.279)</f>
-        <v>2074.923</v>
+        <v>3623.931</v>
       </c>
       <c r="S28" s="18" t="n">
         <f aca="false">MAX(0,S25*0.279)</f>
-        <v>2643.525</v>
+        <v>4286.277</v>
       </c>
       <c r="T28" s="19" t="n">
         <f aca="false">SUM(B28:S28)</f>
-        <v>7006.527</v>
+        <v>16230.546</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15244,79 +15244,79 @@
       </c>
       <c r="B30" s="37" t="n">
         <f aca="false">B25-B28</f>
-        <v>-4133</v>
+        <v>-3981</v>
       </c>
       <c r="C30" s="37" t="n">
         <f aca="false">C25-C28</f>
-        <v>-4051</v>
+        <v>-3771</v>
       </c>
       <c r="D30" s="37" t="n">
         <f aca="false">D25-D28</f>
-        <v>-3504</v>
+        <v>-2992</v>
       </c>
       <c r="E30" s="37" t="n">
         <f aca="false">E25-E28</f>
-        <v>-4181</v>
+        <v>-3437</v>
       </c>
       <c r="F30" s="37" t="n">
         <f aca="false">F25-F28</f>
-        <v>-4717</v>
+        <v>-3717</v>
       </c>
       <c r="G30" s="37" t="n">
         <f aca="false">G25-G28</f>
-        <v>-4439</v>
+        <v>-3159</v>
       </c>
       <c r="H30" s="37" t="n">
         <f aca="false">H25-H28</f>
-        <v>-5692</v>
+        <v>-4076</v>
       </c>
       <c r="I30" s="37" t="n">
         <f aca="false">I25-I28</f>
-        <v>-4625</v>
+        <v>-2649</v>
       </c>
       <c r="J30" s="37" t="n">
         <f aca="false">J25-J28</f>
-        <v>-3430</v>
+        <v>-1094</v>
       </c>
       <c r="K30" s="37" t="n">
         <f aca="false">K25-K28</f>
-        <v>-2360</v>
+        <v>282.632</v>
       </c>
       <c r="L30" s="37" t="n">
         <f aca="false">L25-L28</f>
-        <v>-2670</v>
+        <v>376.362</v>
       </c>
       <c r="M30" s="37" t="n">
         <f aca="false">M25-M28</f>
-        <v>-1469</v>
+        <v>1559.523</v>
       </c>
       <c r="N30" s="37" t="n">
         <f aca="false">N25-N28</f>
-        <v>670.53</v>
+        <v>3606.442</v>
       </c>
       <c r="O30" s="37" t="n">
         <f aca="false">O25-O28</f>
-        <v>93.009</v>
+        <v>3271.177</v>
       </c>
       <c r="P30" s="37" t="n">
         <f aca="false">P25-P28</f>
-        <v>2010.148</v>
+        <v>5488.252</v>
       </c>
       <c r="Q30" s="37" t="n">
         <f aca="false">Q25-Q28</f>
-        <v>3139.234</v>
+        <v>6917.274</v>
       </c>
       <c r="R30" s="37" t="n">
         <f aca="false">R25-R28</f>
-        <v>5362.077</v>
+        <v>9365.069</v>
       </c>
       <c r="S30" s="37" t="n">
         <f aca="false">S25-S28</f>
-        <v>6831.475</v>
+        <v>11076.723</v>
       </c>
       <c r="T30" s="37" t="n">
         <f aca="false">SUM(B30:S30)</f>
-        <v>-27164.527</v>
+        <v>13067.454</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17183,7 +17183,7 @@
         <v>189</v>
       </c>
       <c r="B6" s="62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="63" t="s">
         <v>190</v>
@@ -18390,79 +18390,79 @@
       </c>
       <c r="B34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*B33</f>
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="C34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*C33</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*D33</f>
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="E34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*E33</f>
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="F34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*F33</f>
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="G34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*G33</f>
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="H34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*H33</f>
-        <v>0</v>
+        <v>576</v>
       </c>
       <c r="I34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*I33</f>
-        <v>0</v>
+        <v>696</v>
       </c>
       <c r="J34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*J33</f>
-        <v>0</v>
+        <v>816</v>
       </c>
       <c r="K34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*K33</f>
-        <v>0</v>
+        <v>912</v>
       </c>
       <c r="L34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*L33</f>
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="M34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*M33</f>
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="N34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*N33</f>
-        <v>0</v>
+        <v>1272</v>
       </c>
       <c r="O34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*O33</f>
-        <v>0</v>
+        <v>1368</v>
       </c>
       <c r="P34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*P33</f>
-        <v>0</v>
+        <v>1464</v>
       </c>
       <c r="Q34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*Q33</f>
-        <v>0</v>
+        <v>1560</v>
       </c>
       <c r="R34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*R33</f>
-        <v>0</v>
+        <v>1632</v>
       </c>
       <c r="S34" s="50" t="n">
         <f aca="false">$B$6*MAX(0,80-$B$11)*$B$8*S33</f>
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="T34" s="72" t="n">
         <f aca="false">SUM(B34:S34)</f>
-        <v>0</v>
+        <v>15696</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="1" collapsed="false">
@@ -18534,79 +18534,79 @@
       </c>
       <c r="B36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*B35</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="C36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*C35</f>
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="D36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*D35</f>
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="E36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*E35</f>
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="F36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*F35</f>
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*G35</f>
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="H36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*H35</f>
-        <v>0</v>
+        <v>1040</v>
       </c>
       <c r="I36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*I35</f>
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="J36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*J35</f>
-        <v>0</v>
+        <v>1520</v>
       </c>
       <c r="K36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*K35</f>
-        <v>0</v>
+        <v>1840</v>
       </c>
       <c r="L36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*L35</f>
-        <v>0</v>
+        <v>2160</v>
       </c>
       <c r="M36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*M35</f>
-        <v>0</v>
+        <v>2480</v>
       </c>
       <c r="N36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*N35</f>
-        <v>0</v>
+        <v>2800</v>
       </c>
       <c r="O36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*O35</f>
-        <v>0</v>
+        <v>3040</v>
       </c>
       <c r="P36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*P35</f>
-        <v>0</v>
+        <v>3360</v>
       </c>
       <c r="Q36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*Q35</f>
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="R36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*R35</f>
-        <v>0</v>
+        <v>3920</v>
       </c>
       <c r="S36" s="50" t="n">
         <f aca="false">$B$6*MAX(0,200-$B$12)*$B$9*S35</f>
-        <v>0</v>
+        <v>4160</v>
       </c>
       <c r="T36" s="72" t="n">
         <f aca="false">SUM(B36:S36)</f>
-        <v>0</v>
+        <v>33760</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18615,79 +18615,79 @@
       </c>
       <c r="B37" s="80" t="n">
         <f aca="false">B34+B36</f>
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="C37" s="80" t="n">
         <f aca="false">C34+C36</f>
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="D37" s="80" t="n">
         <f aca="false">D34+D36</f>
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="E37" s="80" t="n">
         <f aca="false">E34+E36</f>
-        <v>0</v>
+        <v>744</v>
       </c>
       <c r="F37" s="80" t="n">
         <f aca="false">F34+F36</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G37" s="80" t="n">
         <f aca="false">G34+G36</f>
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="H37" s="80" t="n">
         <f aca="false">H34+H36</f>
-        <v>0</v>
+        <v>1616</v>
       </c>
       <c r="I37" s="80" t="n">
         <f aca="false">I34+I36</f>
-        <v>0</v>
+        <v>1976</v>
       </c>
       <c r="J37" s="80" t="n">
         <f aca="false">J34+J36</f>
-        <v>0</v>
+        <v>2336</v>
       </c>
       <c r="K37" s="80" t="n">
         <f aca="false">K34+K36</f>
-        <v>0</v>
+        <v>2752</v>
       </c>
       <c r="L37" s="80" t="n">
         <f aca="false">L34+L36</f>
-        <v>0</v>
+        <v>3192</v>
       </c>
       <c r="M37" s="80" t="n">
         <f aca="false">M34+M36</f>
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="N37" s="80" t="n">
         <f aca="false">N34+N36</f>
-        <v>0</v>
+        <v>4072</v>
       </c>
       <c r="O37" s="80" t="n">
         <f aca="false">O34+O36</f>
-        <v>0</v>
+        <v>4408</v>
       </c>
       <c r="P37" s="80" t="n">
         <f aca="false">P34+P36</f>
-        <v>0</v>
+        <v>4824</v>
       </c>
       <c r="Q37" s="80" t="n">
         <f aca="false">Q34+Q36</f>
-        <v>0</v>
+        <v>5240</v>
       </c>
       <c r="R37" s="80" t="n">
         <f aca="false">R34+R36</f>
-        <v>0</v>
+        <v>5552</v>
       </c>
       <c r="S37" s="80" t="n">
         <f aca="false">S34+S36</f>
-        <v>0</v>
+        <v>5888</v>
       </c>
       <c r="T37" s="80" t="n">
         <f aca="false">SUM(B37:S37)</f>
-        <v>0</v>
+        <v>49456</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18718,79 +18718,79 @@
       </c>
       <c r="B39" s="58" t="n">
         <f aca="false">B30+B37</f>
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="C39" s="58" t="n">
         <f aca="false">C30+C37</f>
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="D39" s="58" t="n">
         <f aca="false">D30+D37</f>
-        <v>180</v>
+        <v>692</v>
       </c>
       <c r="E39" s="58" t="n">
         <f aca="false">E30+E37</f>
-        <v>480</v>
+        <v>1224</v>
       </c>
       <c r="F39" s="58" t="n">
         <f aca="false">F30+F37</f>
-        <v>780</v>
+        <v>1780</v>
       </c>
       <c r="G39" s="58" t="n">
         <f aca="false">G30+G37</f>
-        <v>1260</v>
+        <v>2540</v>
       </c>
       <c r="H39" s="58" t="n">
         <f aca="false">H30+H37</f>
-        <v>2010</v>
+        <v>3626</v>
       </c>
       <c r="I39" s="58" t="n">
         <f aca="false">I30+I37</f>
-        <v>2490</v>
+        <v>4466</v>
       </c>
       <c r="J39" s="58" t="n">
         <f aca="false">J30+J37</f>
-        <v>3240</v>
+        <v>5576</v>
       </c>
       <c r="K39" s="58" t="n">
         <f aca="false">K30+K37</f>
-        <v>3720</v>
+        <v>6472</v>
       </c>
       <c r="L39" s="58" t="n">
         <f aca="false">L30+L37</f>
-        <v>4470</v>
+        <v>7662</v>
       </c>
       <c r="M39" s="58" t="n">
         <f aca="false">M30+M37</f>
-        <v>4950</v>
+        <v>8582</v>
       </c>
       <c r="N39" s="58" t="n">
         <f aca="false">N30+N37</f>
-        <v>6600</v>
+        <v>10672</v>
       </c>
       <c r="O39" s="58" t="n">
         <f aca="false">O30+O37</f>
-        <v>7080</v>
+        <v>11488</v>
       </c>
       <c r="P39" s="58" t="n">
         <f aca="false">P30+P37</f>
-        <v>8910</v>
+        <v>13734</v>
       </c>
       <c r="Q39" s="58" t="n">
         <f aca="false">Q30+Q37</f>
-        <v>9840</v>
+        <v>15080</v>
       </c>
       <c r="R39" s="58" t="n">
         <f aca="false">R30+R37</f>
-        <v>11670</v>
+        <v>17222</v>
       </c>
       <c r="S39" s="58" t="n">
         <f aca="false">S30+S37</f>
-        <v>12900</v>
+        <v>18788</v>
       </c>
       <c r="T39" s="58" t="n">
         <f aca="false">SUM(B39:S39)</f>
-        <v>80580</v>
+        <v>130036</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>